<commit_message>
Update content batch rule and summary spreadsheet
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/outputs/drafts/content-batch-2026-02-27/content-batch-summary-20260227.xlsx
+++ b/outputs/drafts/content-batch-2026-02-27/content-batch-summary-20260227.xlsx
@@ -1770,10 +1770,10 @@
       <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The $172,000 gap is the emotional center of the post. Presenting the two numbers side by side creates an immediate, undeniable contrast that makes the gap feel personal and urgent.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Upper block: "$31,000" in Playfair Display SemiBold, approximately 64pt, Off-White (#F6F7F5), centered horizontally, positioned above the vertical center. Label text: "contributed" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the upper number. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 32px below the label. Lower block: "$203,000" in Playfair Display SemiBold, approximately 64pt, Antique Gold (#B08D57), centered horizontally, positioned 32px below the rule. Label text: "available" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the lower number. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: sobering, precise, clarifying. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "$31,000" in Playfair Display SemiBold, ~64pt, Off-White (#F6F7F5), above center. "contributed" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below upper number. "$203,000" in Playfair Display SemiBold, ~64pt, Antique Gold (#B08D57), below rule. "available" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below lower number.
+Image type: Conceptual photograph (photorealistic, people)
+Rationale: The $172,000 retirement gap is fundamentally about a surgeon who doesn't realize the capacity available to them. A photorealistic image of a senior surgeon reviewing financial documents creates an immediate sense of "that could be me" and grounds the abstract gap in a concrete, relatable moment.
+AI image prompt: Create a 1080x1080px square photorealistic image. A male surgeon in his late 50s, wearing a tailored charcoal sport coat over a white open-collar dress shirt, seated at a clean modern walnut desk. He is reviewing a multi-page printed financial document, one hand resting on the pages, the other holding a pair of reading glasses. The setting is a private office with a large window behind and to the right, soft late-afternoon natural light illuminating the desk surface and the side of his face. Background softly out of focus: a few books on a minimal shelf, neutral gray wall. His expression is thoughtful and focused, slightly furrowed brow, as if discovering something unexpected in the numbers. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field, sharp focus on his hands and the document. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no handshakes, no stethoscope on money). Mood: sobering, precise, introspective. Photorealistic editorial photography style suitable for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -1824,10 +1824,10 @@
       <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The six-month planning window is the post's central insight. Presenting the two dates as bookends of a strategic period reframes the extension as intentional and creates a visual that feels like a calendar opportunity rather than a deadline.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "April 15" in Playfair Display Regular, approximately 48pt, Off-White (#F6F7F5), centered horizontally, positioned above the vertical center. A horizontal arrow (2px, Antique Gold #B08D57) spanning 20% of canvas width, centered horizontally, positioned 24px below primary text. Secondary text: "October 15" in Playfair Display SemiBold, approximately 48pt, Antique Gold (#B08D57), centered horizontally, positioned 24px below the arrow. Tertiary text: "6 months of planning capacity" in Inter Regular, approximately 18pt, Warm Gray (#9AA3A8), centered horizontally, positioned 40px below the secondary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: calm, strategic, empowering. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "April 15" in Playfair Display Regular, ~48pt, Off-White (#F6F7F5), above center. Arrow in Antique Gold (#B08D57), centered. "October 15" in Playfair Display SemiBold, ~48pt, Antique Gold (#B08D57), below arrow. "6 months of planning capacity" in Inter Regular, ~18pt, Warm Gray (#9AA3A8), below secondary.
+Image type: Simple infographic
+Rationale: The six-month planning window from April to October is a timeline-driven insight that benefits from a clean visual timeline rather than static text. A branded horizontal timeline shows the extension period as a deliberate strategic runway, making the abstract "six months" feel concrete and structured.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (100px all sides). A horizontal timeline runs across the center of the canvas from left to right. Left endpoint: a small filled circle (12px, Deep Muted Blue #243A4B) with the label "April 15" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), positioned above the circle. Right endpoint: a small filled circle (12px, Antique Gold #B08D57) with the label "October 15" in Inter SemiBold, 16pt, Antique Gold (#B08D57), positioned above the circle. The timeline bar connecting them: 3px, Blue Slate (#5F7483). Three evenly spaced milestone markers along the timeline (small open circles, 8px, Blue Slate #5F7483). Below each milestone, labels in Inter Regular, 13pt, Charcoal (#1E2428): "Fund cash balance plan", "Restructure entity elections", "Finalize retirement contributions". Headline above the timeline: "6 Months of Planning Capacity" in Playfair Display SemiBold, 28pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper third. Below the timeline, a supporting line: "The extension is a strategy, not a delay." in Inter Regular, 15pt, Blue Slate (#5F7483), centered, positioned 48px below the timeline. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows, no chart junk. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: strategic, organized, empowering. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "6 Months of Planning Capacity" in Playfair Display SemiBold, ~28pt, Deep Muted Blue (#243A4B), upper third. Timeline labels and milestones in Inter, various sizes, Charcoal and Blue Slate.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -1877,10 +1877,10 @@
       <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The binary nature of the QBI deduction ($29,800 vs. $0) is the post's central tension. Presenting the two amounts side by side makes the stakes immediate and personal for any surgeon who has just filed.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "$29,800" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned above the vertical center. Secondary text: "or" in Inter Regular, approximately 20pt, Warm Gray (#9AA3A8), centered horizontally, positioned 24px below the primary text. Tertiary text: "$0" in Playfair Display SemiBold, approximately 72pt, Off-White (#F6F7F5), centered horizontally, positioned 24px below the secondary text. Subtext: "QBI Deduction" in Inter SemiBold, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 40px below the tertiary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 24px below the subtext. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: precise, clarifying, slightly provocative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "$29,800" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), above center. "or" in Inter Regular, ~20pt, Warm Gray (#9AA3A8), between numbers. "$0" in Playfair Display SemiBold, ~72pt, Off-White (#F6F7F5), below "or." "QBI Deduction" in Inter SemiBold, ~16pt, Warm Gray (#9AA3A8), below tertiary.
+Image type: Conceptual photograph (photorealistic, environment)
+Rationale: The QBI deduction is a hidden lever buried in the tax return. A photorealistic image of a calm, modern professional environment with a tax document visible on the surface creates a contemplative mood that pairs with the "look closer" message of the post without revealing the answer on the image itself.
+AI image prompt: Create a 1080x1080px square photorealistic image. A clean, modern executive desk surface shot from above at a slight angle. On the desk: a neatly printed multi-page tax return (1040 form partially visible), a fine-point pen resting on the pages, and a small potted succulent in the upper-left corner. The desk is walnut or dark wood grain. Soft natural light from a window on the right side casts gentle shadows across the surface. The background beyond the desk is softly out of focus: a neutral gray wall with a hint of a framed credential. No people visible, just the desk and documents suggesting someone has been studying the return. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field with sharp focus on the pen and the center of the document. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: precise, contemplative, quietly provocative. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -1932,10 +1932,10 @@
       <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Infographic
-Rationale: The post synthesizes four weeks of content into one closing argument. A structured visual showing the four diagnostic threads converging on the tax return creates a visual summary that rewards readers who followed the full arc while standing alone for those encountering it fresh.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered composition with generous margins (minimum 100px all sides). Top section: "4 Weeks. 1 Document." in Playfair Display SemiBold, approximately 36pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper quarter. Four rows below, evenly spaced vertically (each approximately 28px apart), left-aligned at 140px from left edge: Row 1: "Week 1: Entity Structure" in Inter Regular, approximately 18pt, Off-White (#F6F7F5). Row 2: "Week 2: S-Corp Salary" in Inter Regular, approximately 18pt, Off-White (#F6F7F5). Row 3: "Week 3: Reimbursement Pressure" in Inter Regular, approximately 18pt, Off-White (#F6F7F5). Row 4: "Week 4: Effective Hourly Rate" in Inter Regular, approximately 18pt, Off-White (#F6F7F5). A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 40% of canvas width, centered horizontally, positioned 40px below the last row. Below the rule: "Your tax return confirms all of it." in Inter SemiBold, approximately 20pt, Antique Gold (#B08D57), centered horizontally, positioned 24px below the rule. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: composed, authoritative, reflective. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "4 Weeks. 1 Document." in Playfair Display SemiBold, ~36pt, Antique Gold (#B08D57), upper quarter center. Four rows of week labels in Inter Regular, ~18pt, Off-White (#F6F7F5), left-aligned. "Your tax return confirms all of it." in Inter SemiBold, ~20pt, Antique Gold (#B08D57), below rule.
+Image type: Data visualization
+Rationale: The post synthesizes four weeks of content into one closing argument. A convergence diagram showing four diagnostic threads flowing into a single document creates a visual summary that makes the cumulative narrative feel inevitable, rewarding readers who followed the arc while standing alone for new viewers.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "4 Weeks. 1 Document." in Playfair Display SemiBold, 28pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, four horizontal rounded-rectangle boxes (approximately 300px wide x 48px tall each) stacked vertically with 20px spacing, centered horizontally. Each box has a 2px border in Blue Slate (#5F7483) with Off-White fill. Labels inside each box in Inter Medium, 15pt, Deep Muted Blue (#243A4B), centered: Box 1: "Entity Structure", Box 2: "S-Corp Salary", Box 3: "Reimbursement Pressure", Box 4: "Effective Hourly Rate". From the right edge of each box, a thin connecting line (2px, Antique Gold #B08D57) curves downward and converges to a single point below all four boxes. At the convergence point, a larger rounded rectangle (320px wide x 56px tall) with a solid Deep Muted Blue (#243A4B) fill. Label inside: "Your Tax Return" in Inter SemiBold, 16pt, Off-White (#F6F7F5), centered. Below the bottom box, 24px of spacing, then: "Every answer is on one document." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: composed, authoritative, clarifying. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "4 Weeks. 1 Document." in Playfair Display SemiBold, ~28pt, Deep Muted Blue. Four labeled boxes and convergence to "Your Tax Return" box.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -2056,10 +2056,10 @@
       <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The "4x per year" framing is a simple, memorable reframe that transforms a routine obligation into a strategic cadence. Presenting it as a bold stat card contrasts the number surgeons expect (a bill) with the concept they should adopt (a strategy session).
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "4x" in Playfair Display SemiBold, approximately 108pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "per year to recalibrate" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "your tax, retirement, and cash flow strategy" in Inter Regular, approximately 15pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: strategic, composed, forward-looking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "4x" in Playfair Display SemiBold, ~108pt, Antique Gold (#B08D57), center. "per year to recalibrate" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "your tax, retirement, and cash flow strategy" in Inter Regular, ~15pt, Warm Gray (#9AA3A8), below secondary.
+Image type: Conceptual photograph (photorealistic, people)
+Rationale: The post reframes estimated tax payments as quarterly strategy sessions. A photorealistic image of a surgeon and financial advisor reviewing numbers together conveys the proactive, collaborative relationship the post advocates, moving the image from an abstract number to a tangible moment of financial intentionality.
+AI image prompt: Create a 1080x1080px square photorealistic image. Two professionals seated across from each other at a clean, modern conference table in a well-lit office. One is a male surgeon in his mid-50s wearing a navy blazer over an open-collar white shirt; the other is a female financial advisor in her 40s wearing a charcoal blazer. Between them on the table: a printed financial summary, a laptop angled toward the advisor, and two ceramic coffee cups. The advisor is pointing at a line on the printed document while the surgeon leans in slightly, expression engaged and focused. The setting is a modern office with floor-to-ceiling windows, natural afternoon light creating soft highlights. Background softly out of focus: a cityscape or green campus visible through the windows. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field, sharp focus on the two professionals and the document between them. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no posed handshakes, no pointing at charts on a whiteboard). Mood: strategic, composed, collaborative. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -2110,10 +2110,10 @@
       <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The number "3" paired with "decisions" creates a scannable, curiosity-driven visual that promises a framework. The clean typographic card matches the post's organizational tone and invites the reader to discover what they're missing.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "3" in Playfair Display SemiBold, approximately 120pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "decisions inside one deadline" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "April 15, 2026" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: clarifying, organized, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "3" in Playfair Display SemiBold, ~120pt, Antique Gold (#B08D57), center. "decisions inside one deadline" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "April 15, 2026" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below secondary.
+Image type: Simple infographic
+Rationale: The post reveals three decisions hidden inside a single deadline. A clean three-panel infographic makes the framework immediately scannable and creates a saveable reference visual that surgeons can revisit as April 15 approaches.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "April 15: Three Decisions, One Date" in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, three vertical panels arranged side by side with 24px spacing between them, each approximately 260px wide x 420px tall. Each panel has a 2px top border only (no sides or bottom). Panel 1 top border: Deep Muted Blue (#243A4B). Inside Panel 1: number "1" in Playfair Display SemiBold, 48pt, Deep Muted Blue (#243A4B), centered, at top. Below: "File or Extend" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Process decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Panel 2 top border: Antique Gold (#B08D57). Inside Panel 2: number "2" in Playfair Display SemiBold, 48pt, Antique Gold (#B08D57), centered, at top. Below: "Prior-Year IRA" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Strategy decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Panel 3 top border: Blue Slate (#5F7483). Inside Panel 3: number "3" in Playfair Display SemiBold, 48pt, Blue Slate (#5F7483), centered, at top. Below: "Q1 Estimated Tax" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Strategy decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Below all three panels, 32px spacing, then: "Which of these three have you addressed?" in Inter Regular, 15pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: clarifying, organized, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "April 15: Three Decisions, One Date" headline. Three numbered panels with decision labels and types.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -2165,10 +2165,10 @@
       <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The side-by-side tax rate comparison (42% vs. 0%) is the post's most powerful data point. Isolating both numbers on a single card creates an immediate visual contrast that captures the opportunity cost argument without requiring the reader to process the full math.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Left-aligned text block: "Roth:" in Inter Medium, approximately 18pt, Warm Gray (#9AA3A8), followed on the same line by "42% tax" in Playfair Display SemiBold, approximately 42pt, Off-White (#F6F7F5). Right-aligned or below text block: "Cash balance:" in Inter Medium, approximately 18pt, Warm Gray (#9AA3A8), followed on the same line by "0% tax" in Playfair Display SemiBold, approximately 42pt, Antique Gold (#B08D57). Both text blocks centered vertically, with 40px vertical spacing between them. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 40% of the canvas width, centered horizontally, positioned 48px below the lower text block. Tertiary text: "Same $7,500. Very different math." in Inter Regular, approximately 16pt, Off-White (#F6F7F5), centered horizontally, positioned 24px below the rule. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: precise, comparative, thought-provoking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Roth: 42% tax" with label in Inter Medium ~18pt Warm Gray (#9AA3A8) and rate in Playfair Display SemiBold ~42pt Off-White (#F6F7F5). "Cash balance: 0% tax" with label in Inter Medium ~18pt Warm Gray (#9AA3A8) and rate in Playfair Display SemiBold ~42pt Antique Gold (#B08D57). "Same $7,500. Very different math." in Inter Regular ~16pt Off-White (#F6F7F5) below rule.
+Image type: Data visualization
+Rationale: The post's entire argument is a side-by-side math comparison. A branded bar chart showing the tax treatment of the same $7,500 in two vehicles makes the opportunity cost immediately visible and creates a visual that surgeons can share with colleagues to illustrate the point.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "Same $7,500. Very Different Math." in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, two vertical bar chart columns centered on the canvas with 80px horizontal spacing between them. Left bar: tall (approximately 340px height), filled with Blue Slate (#5F7483). Labeled above the bar: "42%" in Inter SemiBold, 28pt, Deep Muted Blue (#243A4B). Labeled below the bar in two lines: "Backdoor Roth" in Inter SemiBold, 15pt, Deep Muted Blue (#243A4B), then "Tax on contribution" in Inter Regular, 12pt, Blue Slate (#5F7483). Right bar: very short (approximately 20px height, representing near-zero), filled with Antique Gold (#B08D57). Labeled above the bar: "0%" in Inter SemiBold, 28pt, Antique Gold (#B08D57). Labeled below the bar in two lines: "Cash Balance Plan" in Inter SemiBold, 15pt, Deep Muted Blue (#243A4B), then "Immediate deduction" in Inter Regular, 12pt, Blue Slate (#5F7483). A thin Warm Gray (#9AA3A8) baseline (1px) connects the base of both bars. Below the chart, 40px spacing, then: "At surgeon income levels, the opportunity cost compounds." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows, no chart junk. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: precise, comparative, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "Same $7,500. Very Different Math." headline, "42%" and "0%" bar labels, vehicle names and descriptions below bars.
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -2220,10 +2220,10 @@
       <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: A clean list card with the four vital signs creates a scannable, saveable reference that surgeons can screenshot or revisit each quarter. The list format matches the post's framework-driven tone and invites the reader to adopt the cadence.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: left-aligned text composition with generous margins (120px top and bottom, 100px left, 80px right). Header text: "Quarterly vital signs" in Playfair Display SemiBold, approximately 36pt, Off-White (#F6F7F5), left-aligned, positioned in the upper quarter of the canvas. A thin horizontal rule (1px, Antique Gold #B08D57) spans 50% of the canvas width, left-aligned with the header text, positioned 24px below the header. Four list items below the rule, each in Inter Medium, approximately 20pt, Off-White (#F6F7F5), left-aligned, with 36px vertical spacing between items. Item 1: "Income vs. projection". Item 2: "Retirement contribution pace". Item 3: "Estimated tax adequacy". Item 4: "Cash reserve level". A small square bullet (6px, Antique Gold #B08D57) precedes each item with 16px horizontal spacing. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: organized, empowering, methodical. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Quarterly vital signs" in Playfair Display SemiBold, ~36pt, Off-White (#F6F7F5), upper quarter left. Four list items in Inter Medium, ~20pt, Off-White (#F6F7F5), with Antique Gold (#B08D57) bullet squares.
+Image type: Conceptual photograph (photorealistic, environment)
+Rationale: The post introduces a quarterly discipline framework using a clinical vital-signs analogy. A photorealistic image of a modern medical office environment evokes the clinical rigor the post advocates, connecting the surgeon's professional world to their financial discipline without being literal or heavy-handed.
+AI image prompt: Create a 1080x1080px square photorealistic image. A modern, well-lit medical office corridor viewed from a slight angle, early morning natural light filtering through large windows on the right side. The corridor is clean, minimal, and empty, with polished light-gray floors and white walls. A glass-walled conference room is partially visible on the left, with a clean table and two chairs inside, suggesting a structured meeting space. A single potted green plant sits at the far end of the corridor, providing a subtle touch of warmth. The overall feeling is one of order, discipline, and calm professionalism. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field with the far end of the corridor softly out of focus. No people, no text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: organized, professional, forward-looking. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: LinkedIn, 1080x1080</t>
         </is>
       </c>
@@ -2952,10 +2952,10 @@
       <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: A single reframing statement presented typographically reinforces the normalizing message without visual clutter.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Charcoal (#1E2428) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "An extension isn't a delay. It's a planning window." in Playfair Display Medium, approximately 36pt, Off-White (#F6F7F5), centered horizontally, positioned in the upper-center area, maximum width 78% of canvas. Line height 1.4. Below the quote, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 25% of the canvas width, centered horizontally, with 32px spacing above and below. Subtext: "You have until October 15." in Inter Regular, approximately 18pt, Blue Slate (#5F7483), centered horizontally, positioned below the accent line. Brand mark: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), bottom-center with 40px bottom margin. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling. Mood: reassuring, calm, professional. For orthopedic surgeons ages 45-65.
-Text overlay: "An extension isn't a delay. It's a planning window." in Playfair Display Medium, ~36pt, Off-White (#F6F7F5), centered. "You have until October 15." in Inter Regular, ~18pt, Blue Slate (#5F7483), centered below accent line. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), bottom-center.
+Image type: Conceptual photograph (photorealistic, people)
+Rationale: The post normalizes the extension with a warm, over-coffee tone. A photorealistic image of a senior professional in a calm, contemplative moment reinforces the reassurance of the message and creates an immediate sense of trust and relatability.
+AI image prompt: Create a 1200x630px landscape photorealistic image. A male physician in his early 60s, wearing a light blue button-down shirt with no tie, seated in a leather armchair in a well-appointed home office or study. He is holding a ceramic coffee mug in one hand while glancing at a printed financial document resting on the arm of the chair. Bookshelves with medical and business texts are softly out of focus behind him. Morning light streams in from a window on the left, casting warm highlights across the room. His expression is calm, unhurried, and quietly confident. Color grading: slightly desaturated, warm tones in the highlights, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483). Shallow depth of field, sharp focus on the subject's face and hands. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no smiling into camera, no handshakes). Mood: reassuring, calm, trustworthy. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3005,10 +3005,10 @@
       <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: Presenting the effective tax rate concept as a simple typographic question invites curiosity and self-reflection without overwhelming the reader with data.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "Do you know your effective tax rate?" in Playfair Display Medium, approximately 38pt, Off-White (#F6F7F5), centered horizontally, positioned in the upper-center area, maximum width 75% of canvas. Line height 1.4. Below the question, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 28% of the canvas width, centered horizontally, with 32px spacing above and below. Subtext: "Line 24 ÷ Line 15" in Inter Medium, approximately 20pt, Antique Gold (#B08D57), centered horizontally, below accent line. Brand mark: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), bottom-center with 40px bottom margin. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling. Mood: curious, warm, inviting. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Do you know your effective tax rate?" in Playfair Display Medium, ~38pt, Off-White (#F6F7F5), centered. "Line 24 ÷ Line 15" in Inter Medium, ~20pt, Antique Gold (#B08D57), centered below accent line. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), bottom-center.
+Image type: Data visualization
+Rationale: The post walks readers through a concrete two-line calculation. A simple branded visual showing the formula (Total Tax / Total Income = Effective Rate) as a clean equation graphic makes the takeaway scannable and actionable, and gives readers a visual they can screenshot and reference when reviewing their own return.
+AI image prompt: Create a 1200x630px landscape infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "Your Effective Tax Rate" in Playfair Display SemiBold, 26pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper quarter. Below the headline, a clean equation layout centered on the canvas: three rounded rectangles arranged horizontally. Left rectangle (220px x 60px, 2px border Blue Slate #5F7483, Off-White fill): "Line 24: Total Tax" in Inter Medium, 14pt, Deep Muted Blue (#243A4B), centered inside. A division symbol (÷) in Inter SemiBold, 24pt, Antique Gold (#B08D57), centered between the left and middle rectangles with 20px horizontal spacing. Middle rectangle (220px x 60px, 2px border Blue Slate #5F7483, Off-White fill): "Line 15: Total Income" in Inter Medium, 14pt, Deep Muted Blue (#243A4B), centered inside. An equals sign (=) in Inter SemiBold, 24pt, Antique Gold (#B08D57), centered between the middle and right rectangles with 20px horizontal spacing. Right rectangle (200px x 60px, solid Deep Muted Blue #243A4B fill): "Effective Rate" in Inter SemiBold, 14pt, Off-White (#F6F7F5), centered inside. Below the equation, 40px spacing, then supporting text: "This single percentage tells you more than your bracket." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: curious, clear, inviting. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "Your Effective Tax Rate" headline, equation layout with labeled boxes, and supporting text.
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3057,10 +3057,10 @@
       <c r="G20" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: A single dollar figure presented typographically creates immediate curiosity. The specificity of $29,800 suggests precision and insider knowledge without requiring complex visuals.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Charcoal (#1E2428) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "$29,800" in Playfair Display Bold, approximately 64pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above center. Below, secondary text: "The deduction most surgeons don't know exists." in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, maximum width 70% of canvas, with 24px spacing above. A thin horizontal accent line (2px, Blue Slate #5F7483) spanning 20% of the canvas width, centered horizontally, with 32px spacing above and below secondary text. Brand mark: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), bottom-center with 40px bottom margin. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling. Mood: intriguing, knowledgeable, precise. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "$29,800" in Playfair Display Bold, ~64pt, Antique Gold (#B08D57), centered. "The deduction most surgeons don't know exists." in Inter Regular, ~20pt, Off-White (#F6F7F5), centered below. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), bottom-center.
+Image type: Conceptual photograph (photorealistic, environment)
+Rationale: The post reveals a hidden deduction most surgeons overlook. A photorealistic image of a professional environment with a tax document creates visual intrigue ("what's hiding in those pages?") that mirrors the post's discovery narrative, without giving away the punchline in the image itself.
+AI image prompt: Create a 1200x630px landscape photorealistic image. A modern, well-organized professional desk viewed from a slightly elevated angle. On the desk surface: a printed tax return with several pages spread out, a highlighter with its cap off resting near one page as if a line has just been marked, a slim laptop half-closed in the background, and a glass of water on a stone coaster. The desk is light oak or birch. Natural morning light from a large window behind the desk illuminates the scene evenly, creating soft shadows. The room beyond is a minimalist professional office: a single framed credential on the wall, a potted fiddle-leaf fig in the corner, neutral gray walls. No people visible. Color grading: slightly desaturated, warm tones in the highlights, shadows shifted toward Deep Muted Blue (#243A4B), midtones clean and neutral. Shallow depth of field with sharp focus on the highlighted document and the highlighter pen. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: intriguing, precise, professional. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3109,10 +3109,10 @@
       <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Conceptual photograph
-Rationale: A reflective, transition-themed image pairs well with the month-closing tone. A clean, contemplative composition signals the shift from looking backward (March, diagnosis) to looking forward (April, interpretation).
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: a soft gradient from Deep Muted Blue (#243A4B) on the left to Charcoal (#1E2428) on the right, covering the full canvas. Layout: left-aligned text composition with generous margins (minimum 80px all sides). Primary text: "You've seen the numbers. Now let's read them." in Playfair Display Medium, approximately 34pt, Off-White (#F6F7F5), left-aligned, positioned in the left half of the canvas, maximum width 55% of canvas. Line height 1.4. Below, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 20% of the canvas width, left-aligned with the text, with 28px spacing above and below. Subtext: "April: Post-Filing Insights" in Inter Medium, approximately 16pt, Antique Gold (#B08D57), left-aligned below accent line. Brand mark: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), bottom-left with 40px margins. No photography, no illustrations, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling. Mood: reflective, forward-looking, calm. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "You've seen the numbers. Now let's read them." in Playfair Display Medium, ~34pt, Off-White (#F6F7F5), left-aligned. "April: Post-Filing Insights" in Inter Medium, ~16pt, Antique Gold (#B08D57), left-aligned below accent line. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), bottom-left.
+Image type: Simple infographic
+Rationale: The post bridges from March's diagnosis arc to April's interpretation arc. A clean two-phase visual showing the transition creates a visual bookend that rewards followers who tracked the month-long narrative while making the forward direction clear for new readers.
+AI image prompt: Create a 1200x630px landscape infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Two large rounded rectangles side by side, horizontally centered, each approximately 400px wide x 200px tall with 40px horizontal spacing between them. Left rectangle: 2px border in Blue Slate (#5F7483), Off-White fill. Inside, header: "March" in Playfair Display SemiBold, 20pt, Deep Muted Blue (#243A4B), centered at top of box. Below header, a thin rule (1px, Warm Gray #9AA3A8) spanning 60% of box width. Below rule, four lines in Inter Regular, 13pt, Blue Slate (#5F7483), centered, 10px spacing: "Entity Structure", "S-Corp Salary", "Reimbursement Pressure", "Effective Hourly Rate". Below the four lines: "Diagnosis" in Inter SemiBold, 14pt, Deep Muted Blue (#243A4B), centered. Right rectangle: 2px border in Antique Gold (#B08D57), Off-White fill. Inside, header: "April" in Playfair Display SemiBold, 20pt, Antique Gold (#B08D57), centered at top of box. Below header, a thin rule (1px, Warm Gray #9AA3A8) spanning 60% of box width. Below rule, four lines in Inter Regular, 13pt, Blue Slate (#5F7483), centered, 10px spacing: "Filing Decisions", "Estimated Tax Strategy", "Roth Evaluation", "Quarterly Calibration". Below the four lines: "Interpretation" in Inter SemiBold, 14pt, Antique Gold (#B08D57), centered. Between the two rectangles, a horizontal arrow (3px, Antique Gold #B08D57) pointing from left box to right box. Headline above both boxes: "From Diagnosis to Interpretation" in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: reflective, forward-looking, organized. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "From Diagnosis to Interpretation" headline, two labeled phase boxes with content themes, connecting arrow.
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3225,10 +3225,10 @@
       <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Quote/insight card
-Rationale: A clean, encouraging typographic card reframes the extension narrative and creates a shareable moment of reassurance for the many surgeons who file extensions every year.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "An extension isn't a delay. It's six months of planning runway." in Playfair Display Medium, approximately 32pt, Off-White (#F6F7F5), centered horizontally, positioned in the upper-center area of the canvas, maximum width 80% of canvas. Line height 1.5. Below the quote, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 25% of the canvas width, centered horizontally, with 32px spacing above and below. Attribution text: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), centered horizontally, positioned below the accent line. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling, no busy compositions. Mood: warm, encouraging, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "An extension isn't a delay. It's six months of planning runway." in Playfair Display Medium, ~32pt, Off-White (#F6F7F5), upper-center. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), centered below accent line.
+Image type: Conceptual photograph (photorealistic, people)
+Rationale: The post normalizes filing an extension with a warm, reassuring tone. A photorealistic image of a relaxed professional in a calm setting reinforces the message that extending is a deliberate, confident move and creates an emotional connection that a text card cannot achieve.
+AI image prompt: Create a 1200x630px landscape photorealistic image. A female surgeon in her early 50s, wearing a soft cream cashmere sweater, seated at a sunlit kitchen island in a modern, well-appointed home. She is holding a tablet displaying a calendar view (the screen content is not readable, just the general impression of a calendar layout), with a cup of coffee and a small stack of papers beside her. Morning light streams through a large kitchen window behind her, creating a warm, inviting atmosphere. Her expression is calm and unhurried, a slight hint of a relaxed smile, as if she has time and feels good about it. The kitchen is clean and modern: light stone countertops, minimal styling, a vase of fresh greenery. Color grading: slightly desaturated, warm tones in the highlights, shadows shifted toward Deep Muted Blue (#243A4B), midtones neutral to warm. Shallow depth of field, sharp focus on the subject and the tablet. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no posed smile at camera). Mood: warm, encouraging, unhurried. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3277,10 +3277,10 @@
       <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Quote/insight card
-Rationale: A reflective question card works well for Facebook's conversational tone and invites engagement without requiring data or statistics. The question itself is the hook.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "When was the last time you checked whether your backdoor Roth still makes sense?" in Playfair Display Medium, approximately 30pt, Off-White (#F6F7F5), centered horizontally, positioned in the upper-center area of the canvas, maximum width 78% of canvas. Line height 1.5. Below the quote, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 25% of the canvas width, centered horizontally, with 36px spacing above and below. Secondary text: "The answer might surprise you." in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 16px below the accent line. Attribution text: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), centered horizontally, positioned 32px below the secondary text. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling, no busy compositions. Mood: curious, warm, thoughtful. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "When was the last time you checked whether your backdoor Roth still makes sense?" in Playfair Display Medium, ~30pt, Off-White (#F6F7F5), upper-center. "The answer might surprise you." in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below accent line. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), bottom center.
+Image type: Simple infographic
+Rationale: The post challenges an automatic financial habit (backdoor Roth) and prompts readers to re-evaluate. A clean decision-tree infographic visually captures the "should you or shouldn't you?" question and gives the reader a framework to think through the post's argument.
+AI image prompt: Create a 1200x630px landscape infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (60px all sides). Headline: "Should You Still Fund a Backdoor Roth?" in Playfair Display SemiBold, 22pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, a simple branching flowchart. Starting node: a rounded rectangle (200px x 44px, solid Deep Muted Blue #243A4B fill) with text "Current tax rate: 37%" in Inter SemiBold, 13pt, Off-White (#F6F7F5), centered. From the bottom of this node, two branches diverge left and right, each a 2px line in Blue Slate (#5F7483). Left branch leads to a rounded rectangle (200px x 44px, 2px border Antique Gold #B08D57, Off-White fill) labeled "Expect lower rate in retirement" in Inter Regular, 12pt, Deep Muted Blue (#243A4B), centered. Below it, a result box (200px x 36px, 2px border Antique Gold #B08D57, Off-White fill): "Re-evaluate the Roth" in Inter SemiBold, 13pt, Antique Gold (#B08D57), centered. Right branch leads to a rounded rectangle (200px x 44px, 2px border Blue Slate #5F7483, Off-White fill) labeled "Expect same or higher rate" in Inter Regular, 12pt, Deep Muted Blue (#243A4B), centered. Below it, a result box (200px x 36px, 2px border Blue Slate #5F7483, Off-White fill): "Roth may still work" in Inter SemiBold, 13pt, Blue Slate (#5F7483), centered. Branch labels: "Yes" in Inter Medium, 11pt, Antique Gold (#B08D57) on the left branch, "No" in Inter Medium, 11pt, Blue Slate (#5F7483) on the right branch. Below the flowchart, 28px spacing, then: "The 37% rate is now permanent under OBBBA. The old assumptions may not apply." in Inter Regular, 12pt, Blue Slate (#5F7483), centered, maximum width 85% of canvas. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 50px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette. No cartoons, no clip art. Mood: curious, thoughtful, clarifying. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "Should You Still Fund a Backdoor Roth?" headline, flowchart with labeled decision nodes and outcomes.
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3329,10 +3329,10 @@
       <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Quote/insight card
-Rationale: A simple, action-oriented card with a single prompt works well on Facebook for driving engagement and sharing. The brevity of the message matches the brevity of the recommended action.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Charcoal (#1E2428) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "Before you write that Q1 check, take 10 minutes." in Playfair Display Medium, approximately 34pt, Off-White (#F6F7F5), centered horizontally, positioned in the upper-center area of the canvas, maximum width 78% of canvas. Line height 1.5. Below the primary text, secondary text: "One question: Am I pacing correctly for the year?" in Inter Regular, approximately 20pt, Antique Gold (#B08D57), centered horizontally, positioned 36px below the primary text. Below the secondary text, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 20% of the canvas width, centered horizontally, with 32px spacing above and below. Attribution text: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), centered horizontally, positioned below the accent line. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling, no busy compositions. Mood: focused, practical, warm. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Before you write that Q1 check, take 10 minutes." in Playfair Display Medium, ~34pt, Off-White (#F6F7F5), upper-center. "One question: Am I pacing correctly for the year?" in Inter Regular, ~20pt, Antique Gold (#B08D57), centered below. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), below accent line.
+Image type: Data visualization
+Rationale: The post asks surgeons to check whether their Q1 estimated payment is pacing correctly. A simple branded bar chart showing quarterly pacing (Q1 at 25% vs. full-year target) makes the calibration concept immediately visual and creates an actionable reference that complements the "10 minutes" prompt.
+AI image prompt: Create a 1200x630px landscape infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (60px all sides). Headline: "Q1 Estimated Tax: Are You Pacing Correctly?" in Playfair Display SemiBold, 22pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper quarter. Below the headline, a horizontal progress bar spanning 75% of the canvas width, centered. The bar has a light Warm Gray (#9AA3A8) background track (16px tall, rounded corners). Filled portion: 25% of the bar filled with Deep Muted Blue (#243A4B), representing Q1. A small vertical tick mark (2px wide, 28px tall, Antique Gold #B08D57) at the 25% mark, extending above and below the bar. Label above the tick: "Q1: 25%" in Inter SemiBold, 14pt, Antique Gold (#B08D57). Four quarter labels below the bar, evenly spaced: "Q1", "Q2", "Q3", "Q4" in Inter Regular, 12pt, Blue Slate (#5F7483). At the right end of the bar: "Annual Target" in Inter Medium, 13pt, Deep Muted Blue (#243A4B). Below the progress bar, 36px spacing, then two side-by-side comparison blocks. Left block: a small down-arrow icon (in Blue Slate #5F7483) with "Overpaying" in Inter SemiBold, 13pt, Deep Muted Blue (#243A4B), and below it: "Cash sitting idle" in Inter Regular, 11pt, Blue Slate (#5F7483). Right block: a small up-arrow icon (in Antique Gold #B08D57) with "Underpaying" in Inter SemiBold, 13pt, Deep Muted Blue (#243A4B), and below it: "Penalties ahead" in Inter Regular, 11pt, Blue Slate (#5F7483). Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 50px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette. No cartoons, no clip art. Mood: focused, practical, clear. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "Q1 Estimated Tax: Are You Pacing Correctly?" headline, progress bar with quarter labels, overpaying/underpaying comparison.
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -3382,10 +3382,10 @@
       <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Quote/insight card
-Rationale: A contemplative typographic card captures the reflective tone of the post and gives surgeons something worth pausing on in their feed as the deadline approaches. The simplicity of the message mirrors the simplicity of the reframe.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with generous margins (minimum 80px all sides). Primary text: "April 15 feels like a deadline. The best use of it is as a decision point." in Playfair Display Medium, approximately 30pt, Off-White (#F6F7F5), centered horizontally, positioned in the center of the canvas, maximum width 76% of canvas. Line height 1.5. Below the quote, a thin horizontal accent line (2px, Antique Gold #B08D57) spanning 20% of the canvas width, centered horizontally, with 36px spacing above and below. Attribution text: "Capable Wealth" in Inter Regular, approximately 14pt, Warm Gray (#9AA3A8), centered horizontally, positioned 24px below the accent line. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock imagery, no clickbait styling, no busy compositions. Mood: reflective, calm, grounded. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "April 15 feels like a deadline. The best use of it is as a decision point." in Playfair Display Medium, ~30pt, Off-White (#F6F7F5), centered. "Capable Wealth" in Inter Regular, ~14pt, Warm Gray (#9AA3A8), below accent line.
+Image type: Conceptual photograph (photorealistic, environment)
+Rationale: The post closes the week with a philosophical reflection on April 15 as a decision point rather than a deadline. A photorealistic image of a quiet, contemplative environment conveys the pause-and-reflect mood of the post and creates a visual moment of calm in a feed full of tax-season noise.
+AI image prompt: Create a 1200x630px landscape photorealistic image. A modern home office viewed through an open doorway, shot from the hallway looking in. Inside the room: a clean walnut desk positioned near a large window, with an open leather portfolio and a pen resting on it. A comfortable high-back chair is pulled slightly away from the desk, as if someone just stepped away for a moment of reflection. Late afternoon golden light streams through the window, casting long warm shadows across the desk and the hardwood floor. A small bookshelf with a few carefully placed books and a framed family photo (not clearly visible, just the impression of one) is on the far wall. The room is quiet, orderly, and personal. No people visible. Color grading: warm and slightly desaturated, shadows shifted toward Deep Muted Blue (#243A4B), golden tones preserved in the highlights, midtones neutral. Shallow depth of field with the doorframe slightly soft in the foreground and the window softly glowing in the background. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: reflective, calm, grounded. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Revise all content drafts, add integrity rules and experience docs
- Add content-integrity and content-date-alignment cursor rules
- Add experience inventory and interview guide
- Update content recipe and quarterly plan
- Revise all week 1-6 drafts (blogs, social posts, podcasts/videos)
- Update batch summaries for both content batches

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/outputs/drafts/content-batch-2026-02-27/content-batch-summary-20260227.xlsx
+++ b/outputs/drafts/content-batch-2026-02-27/content-batch-summary-20260227.xlsx
@@ -546,7 +546,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>WEEK 3 (MARCH 16–22)</t>
+          <t>WEEK 3 (MARCH 9–15)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -560,7 +560,7 @@
     <row r="3" ht="200" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -585,11 +585,11 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Last Tuesday, I was on a call with a surgeon I've worked with for three years. Midway through our conversation about his Q1 numbers, he mentioned, almost in passing, that his practice manager had flagged a drop in reimbursements on several of his most-performed procedures.
-"It's that CMS efficiency adjustment," he said. "About 2.5% across the board on the non-time-based codes. My practice manager showed me the numbers in our staff meeting."
-Then he said the part that made me sit up in my chair.
+          <t>Here's a scenario playing out in orthopedic practices right now. A surgeon reviews his Q1 numbers and notices something his practice manager already flagged: a drop in reimbursements on several of his most-performed procedures.
+"It's that CMS efficiency adjustment. About 2.5% across the board on the non-time-based codes."
+And the natural next thought?
 "I guess I'll just have to add a few more cases to the schedule to make up the difference."
-I hear some version of this from surgeons every time reimbursement comes up. Revenue goes down, so volume goes up. It's the instinctive response. It feels logical. And it's one of the most expensive ways to solve the problem.
+This is the instinctive response when reimbursement drops. Revenue goes down, so volume goes up. It feels logical. And it's one of the most expensive ways to solve the problem.
 ## The Imaging Result
 Let me frame this the way you would in a clinical setting. Think of the CMS reimbursement cut as an imaging result. The image itself (a 2.5% reduction in per-procedure revenue on non-time-based orthopedic codes) is the finding. But the finding isn't the diagnosis.
 Most surgeons will look at this result and treat the most obvious symptom: less revenue. The reflexive prescription? More procedures. More volume. More time in the OR.
@@ -609,7 +609,7 @@
 The average orthopedic practice runs overhead between 50% and 60% of collections. For a practice collecting $1.6 million annually (our 400-procedure surgeon at $3,200 average), that's $800K to $960K flowing out of the practice in overhead before the surgeon keeps a dollar.
 A 2% reduction in overhead, across a $1.6M practice, saves $32,000.
 That's the entire reimbursement loss, recovered. No additional procedures. No additional OR time. No additional staff costs. No additional physical wear.
-And 2% is realistic. In my experience working with surgeon-owned practices, there are almost always opportunities in three categories that go unexamined:
+And 2% is realistic. In practice structures like these, there are almost always opportunities in three categories that go unexamined:
 **Supply and vendor contracts.** When was the last time your practice benchmarked its supply costs against peer practices? Implant pricing, surgical supplies, and office materials are negotiable, and most practices haven't renegotiated in years. A 5% reduction in supply costs alone can recover $10K to $20K annually for a typical orthopedic practice.
 **Staffing efficiency.** And to be clear, I'm not talking about cutting staff. Most practices that have grown over time carry staffing structures built for an earlier era of the practice. Aligning staffing ratios with current patient volume, reviewing scheduling workflows, and clarifying role allocation can reduce staffing overhead by 1% to 3% without reducing quality of care.
 **Facility utilization.** If you own your space or have a long-term lease, are you using it efficiently? Unused operatory time, underutilized square footage, and energy costs all add up. For practices that own their building, a cost segregation study (which we discussed in Week 1) can also accelerate depreciation deductions, creating additional tax savings on top of the overhead reduction.
@@ -662,7 +662,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>WEEK 4 (MARCH 23–29)</t>
+          <t>WEEK 4 (MARCH 16–22)</t>
         </is>
       </c>
       <c r="B5" s="3" t="n"/>
@@ -676,12 +676,12 @@
     <row r="6" ht="200" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Your Q1 Revenue Is In. Here's the One Number That Matters More Than Collections.</t>
+          <t>Before Q1 Closes: The One Number That Matters More Than Collections</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -701,12 +701,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Last Tuesday I sat across from a surgeon (let's call him Dr. M) who had just finished reviewing his Q1 practice numbers. Collections were strong. In fact, they were up 4% over the same quarter last year. He was genuinely pleased, and he should have been. Running a busy orthopedic practice and growing collections in an environment of tightening reimbursements is no small thing.
-Then I asked him a question he hadn't considered.
+          <t>Let's build a hypothetical profile for a surgeon we'll call Dr. A. He's pulling together his year-to-date practice numbers. Collections are tracking strong. In fact, they're up 4% over the same period last year. He's genuinely pleased, and he should be. Running a busy orthopedic practice and growing collections in an environment of tightening reimbursements is no small thing.
+But here's a question he hasn't considered.
 "What's your effective hourly rate?"
-He paused. He knew his collections. He knew his overhead percentage (roughly). He had a general sense of his tax burden. But he had never pulled those numbers together into a single figure that captured what he actually keeps for every hour of clinical work.
-We spent the next twenty minutes doing the math. And when we arrived at the number, the room got quiet.
-His collections said $2.4 million. His effective hourly rate said $185.
+He knows his collections. He knows his overhead percentage (roughly). He has a general sense of his tax burden. But he's never pulled those numbers together into a single figure that captures what he actually keeps for every hour of clinical work.
+Here's how the math works for a surgeon in this position. When you run the calculation, the result is sobering.
+His collections say $2.4 million. His effective hourly rate says $185.
 ## Why Collections Lie to You
 Collections are the number everyone celebrates. It's the headline in every practice meeting, the figure on the dashboard, the benchmark you compare against your partners. And it makes sense. Collections represent the top-line revenue your skills and effort produce.
 But collections measure how much the practice earned. They do not measure how much the surgeon kept.
@@ -715,7 +715,7 @@
 ## The Five Components of Your Effective Hourly Rate
 Your effective hourly rate is what remains after five forces act on your collections. Every one of these is measurable, and most of them are (at least partially) within your control.
 **1. Gross Collections**
-This is the starting point. For our example, we'll use $2.4 million annually, which sits in the range I see most often among mid-career orthopedic practice owners.
+This is the starting point. For our example, we'll use $2.4 million annually, which sits in the typical range for mid-career orthopedic practice owners.
 **2. Practice Overhead**
 Rent, staff, supplies, implant costs, malpractice insurance, billing, IT, all of it. For a typical orthopedic practice, overhead runs between 50% and 60% of collections. At 55%, that's $1.32 million, leaving $1.08 million flowing to the surgeon.
 **3. Taxes**
@@ -738,26 +738,26 @@
 **Collections** (the one everybody focuses on) are the hardest to move. Reimbursement rates are set by payers. Case volume is constrained by OR availability and your own physical capacity. Yes, you can optimize your payer mix and coding practices. But the ceiling on collections is lower and harder to push than most surgeons assume.
 The counterintuitive insight: the surgeon who improves structure by 5% often gains more than the surgeon who grows collections by 5%.
 ## The Same Practice, Restructured
-Let's take Dr. M's $2.4 million practice and apply the structural improvements from the first three weeks of this series.
+Let's take Dr. A's $2.4 million practice and apply the structural improvements from the first three weeks of this series.
 Overhead drops from 55% to 52% through a vendor contract renegotiation and a billing audit that recovered underpayments. That's $1.248 million in overhead instead of $1.32 million. The surgeon's pre-tax share rises to $1.152 million.
 S-Corp salary is recalibrated from an arbitrary number to an optimized one, reducing self-employment tax by $18,000. A cash balance plan is established, sheltering an additional $180,000 from current-year taxation and increasing total retirement contributions from $72,000 to $104,000 (the additional $32,000 is offset by the tax savings the plan generates). After accounting for the restructured tax picture, the effective tax burden drops from $432,000 to $396,000.
 Debt service remains the same at $96,000. The practice didn't take on new debt; it didn't pay off old debt early. That number is unchanged.
 The result: the surgeon keeps $560,000 instead of $480,000.
 Divide by the same 2,600 clinical hours, and the effective hourly rate rises from $185 to $215.
 That's a $30 per hour difference. Over 2,600 hours, it's $78,000 per year. Over ten years, assuming even modest investment returns on the difference, it's well north of a million dollars.
-And here's what matters most: Dr. M didn't work a single additional hour to capture that $78,000. He didn't add cases. He didn't take on more call. He didn't negotiate higher reimbursements (though he should explore that, too). The improvement came entirely from how the money flowed after he earned it.
+And here's what matters most: Dr. A didn't work a single additional hour to capture that $78,000. He didn't add cases. He didn't take on more call. He didn't negotiate higher reimbursements (though he should explore that, too). The improvement came entirely from how the money flowed after he earned it.
 ## Your Q1 Checkpoint
-Q1 data is in, or close to it. You have three months of real numbers to work with. Here's what I'd encourage you to do this week.
-**Step 1: Pull your Q1 collections.** Your billing department or practice management software has this number. Write it down.
+Q1 closes at the end of March. In two weeks, you'll have three months of real numbers to work with. Here's the framework I'd encourage you to have ready so you can run the calculation the moment that data is available.
+**Step 1: Pull your Q1 collections.** Your billing department or practice management software will have this number as soon as the quarter closes. Write it down.
 **Step 2: Calculate your annualized overhead rate.** Take Q1 operating expenses, multiply by four, and divide by your annualized collections. If you're above 55%, there's almost certainly room to tighten.
 **Step 3: Estimate your effective tax rate.** Look at your 2025 return (or your Q1 estimated payments for 2026) and calculate what percentage of your surgeon income went to federal and state taxes. If you're north of 38% and you don't have a cash balance plan, that number has room to come down.
 **Step 4: Add up your committed outflows.** Retirement contributions plus debt service. These are the non-negotiable draws on your take-home.
 **Step 5: Do the division.** Take what's left after overhead, taxes, retirement, and debt service. Divide by the number of clinical hours you worked in Q1 (multiply by four to annualize). That's your effective hourly rate.
 Now compare it to last year. Is it higher or lower? If it's lower, and your collections held steady or grew, then the issue isn't revenue. The issue is somewhere in the structure. And the three topics we covered in the previous weeks of this series (entity structure, S-Corp salary, reimbursement adjustments) are the most likely places where value is leaking out.
 ## The Number That Changes the Conversation
-I started tracking effective hourly rates with my surgeon clients about four years ago. What struck me was how often the conversation changed once they saw it.
-Before the calculation, the questions were always about the top line. "How do I collect more?" "Should I add another surgery day?" "Can I renegotiate my payer contracts?"
-Those are good questions. But after seeing their effective hourly rate, the questions shifted. "Where is the money going between collections and my bank account?" "Which of those buckets can I actually shrink?" "Am I structured the way I should be?"
+As a CFP who focuses on complex planning for high-income professionals, one thing stands out about the effective hourly rate: it changes the conversation.
+Before running this calculation, the questions tend to be about the top line. "How do I collect more?" "Should I add another surgery day?" "Can I renegotiate my payer contracts?"
+Those are good questions. But after seeing the effective hourly rate, the questions shift. "Where is the money going between collections and my bank account?" "Which of those buckets can I actually shrink?" "Am I structured the way I should be?"
 The second set of questions is where the real leverage lives.
 You spent years training to perform complex procedures with precision. You understand, better than almost anyone, that outcomes depend on getting the small things right. A 2-millimeter difference in implant placement changes the functional result. A single overlooked variable in the pre-op plan creates complications downstream.
 Your financial structure works the same way. A 3% reduction in overhead, a properly calibrated S-Corp salary, a cash balance plan that matches your age and income profile: these are the small, precise adjustments that compound into significant differences over a career.
@@ -791,7 +791,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>WEEK 5 (MARCH 30 – APRIL 5)</t>
+          <t>WEEK 5 (MARCH 23–29)</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
@@ -805,7 +805,7 @@
     <row r="9" ht="200" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -830,8 +830,8 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>A colleague of mine, an orthopedic surgeon I've worked with for about five years, called me last week. He'd just gotten his 2025 return back from his CPA. Everything was filed. Everything was accurate. And his exact words were, "Alright, that's done. See you in January."
-I asked him if he'd read it.
+          <t>Here's a conversation that illustrates the gap. A surgeon gets his 2025 return back from his CPA. Everything was filed. Everything was accurate. And his response: "Alright, that's done. See you in January."
+Ask that surgeon if he's read it.
 "Read it? My CPA read it. That's what I pay him for."
 He's not wrong about that. His CPA did exactly what a CPA is supposed to do: ensure compliance, file accurately, meet the deadline. But here's the thing. Your CPA reads your tax return the way a radiologist reads an image for a referring physician. They're looking for findings within their scope. They're not designing your treatment plan.
 You, as the surgeon, read the same image and see something different. You see the implications for the patient's function, mobility, quality of life. You see what the findings mean for the plan.
@@ -842,7 +842,7 @@
 Let me walk through them.
 ### Finding 1: Effective Tax Rate
 Where to find it: divide your total tax (line 24 on Form 1040, or the "total tax" figure your CPA provides) by your adjusted gross income (line 11).
-For a surgeon with AGI of $820,000, an effective rate of 36.3% ($298,000 in total tax) is in the range I commonly see. But it's not in the range it should be.
+For a surgeon with AGI of $820,000, an effective rate of 36.3% ($298,000 in total tax) is common at this income level. But it's not in the range it should be.
 An optimally structured surgeon at $820K AGI, one with a calibrated S-Corp salary, a fully funded cash balance plan, maximized retirement contributions, and proper deduction strategies, typically lands between 31% and 33%.
 The gap between 36.3% and 32% on $820,000 is roughly $35,000 per year. That's not a rounding error. That's the annual cost of a structural misalignment that shows up, in black and white, on a single line of your return.
 If your effective rate is above 34% at $800K+ in AGI, the return is telling you that your structure has room to improve. The treatment plan starts with the concepts we covered in Week 1 (entity design) and Week 2 (S-Corp salary calibration).
@@ -854,8 +854,8 @@
 If your QBI deduction is $0 or significantly below $20,000 at your income level, the return is diagnosing an S-Corp salary calibration issue. The treatment: recalibrate the salary for the current year, before the next quarterly payroll cycle.
 ### Finding 3: Retirement Contributions
 Where to find it: pull your W-2 Box 12 (retirement plan contributions), any SEP-IRA or cash balance plan contribution records, and your total retirement savings for the year.
-A surgeon I reviewed last month had total retirement contributions of $31,000 on his return. That's the 401(k) maximum (close to the 2025 limit). He was proud of it. "I maxed out my 401(k)," he told me.
-He did. But the available capacity was $203,000.
+Consider a surgeon whose return shows total retirement contributions of $31,000. That's the 401(k) maximum (close to the 2025 limit). A common reaction: "I maxed out my 401(k)."
+And technically, yes. But the available capacity was $203,000.
 At his age (54) and income level, he was eligible for 401(k) contributions of $30,500 (including the catch-up), employer profit-sharing of approximately $23,500, and cash balance plan contributions of up to $150,000. He was capturing $31,000 out of $203,000 in available tax-deferred space. That's 15% utilization.
 The $172,000 gap compounds every year. Over ten years at a 7% return, that's $2.4 million in retirement wealth that didn't accumulate, because the structure wasn't in place to capture it.
 If your retirement contribution total is below $100,000 and you're a practice owner over 45, the return is diagnosing a retirement plan design gap. The treatment: evaluate whether a cash balance plan (established alongside your existing 401(k)) could unlock the remaining capacity. This was the core concept from Week 1.
@@ -866,8 +866,8 @@
 For surgeons 3 to 5 years from practice transition, state tax strategy becomes a major variable. The difference between practicing (and selling) in a high-tax state versus a no-income-tax state can swing a practice exit by $300,000 to $700,000 in total tax savings. That doesn't mean you should move tomorrow. But it means the state line on your return is a finding worth investigating, especially as you approach transition.
 If your state tax burden exceeds $50,000, the return is telling you that state-level strategy deserves a seat at the planning table. The treatment: include state tax trajectory in any exit or transition planning conversation.
 ## The Diagnosis Nobody Made
-Here's what struck me about the surgeon who called me last week. His return contained every one of these findings. Effective rate above 35%. QBI deduction at $0. Retirement contributions at $34,000 against $200,000+ in available capacity. State tax of $63,000.
-His CPA filed a perfect return. Every number was accurate. Every form was correct. There was nothing wrong with the compliance work.
+Here's what makes this framework so powerful. Consider a return that contains every one of these findings. Effective rate above 35%. QBI deduction at $0. Retirement contributions at $34,000 against $200,000+ in available capacity. State tax of $63,000.
+The CPA filed a perfect return. Every number was accurate. Every form was correct. There was nothing wrong with the compliance work.
 But nobody read the return for strategy. Nobody looked at those four numbers and said, "Here's what this means for your wealth over the next decade." The return was treated as a historical document, a record of what happened, rather than a diagnostic tool that reveals what needs to change.
 It's the difference between filing an image and reading an image. Both are necessary. Only one changes the treatment plan.
 ## What to Do This Week
@@ -915,7 +915,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>WEEK 6 (APRIL 6–12)</t>
+          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
         </is>
       </c>
       <c r="B11" s="3" t="n"/>
@@ -929,7 +929,7 @@
     <row r="12" ht="200" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -949,16 +949,16 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Arrives in the week before April 15 when surgeons are deciding whether to fund prior-year IRA contributions. Challenges the reflexive "always do a backdoor Roth" habit by showing how OBBBA's permanent 37% rate changes the Roth vs. traditional calculus. Extends the April interpretation arc by turning the April 15 deadline from a single event into a three-decision framework. Builds on Week 5's "return as diagnostic" message by showing how the findings lead to specific, time-sensitive decisions.</t>
+          <t>Arrives in the two weeks before April 15 when surgeons are deciding whether to fund prior-year IRA contributions. Challenges the reflexive "always do a backdoor Roth" habit by showing how OBBBA's permanent 37% rate changes the Roth vs. traditional calculus. Extends the April interpretation arc by turning the April 15 deadline from a single event into a three-decision framework. Builds on Week 5's "return as diagnostic" message by showing how the findings lead to specific, time-sensitive decisions.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Last week I had a conversation with a surgeon (let's call her Dr. K) that I've had, in some variation, at least a dozen times every April.
-She had just come out of a meeting with her CPA, return filed, Q1 estimated payment calculated. Then she asked the question I was expecting: "Should I go ahead and fund my backdoor Roth before the fifteenth? I do it every year."
-I asked her a question back. "Why?"
-She paused. "Because I've always done it. My old advisor told me years ago to do a backdoor Roth every year, and I never stopped."
-That answer, the autopilot answer, is the one I hear most often. And for years, it was perfectly reasonable advice. But the tax landscape shifted in 2025, and a lot of surgeons haven't updated their thinking to match.
+          <t>Here's a conversation that plays out in planning offices across the country every April.
+A surgeon sits down with her advisor after meeting with her CPA. Return filed, Q1 estimated payment calculated. Then comes the question: "Should I go ahead and fund my backdoor Roth before the fifteenth? I do it every year."
+The advisor asks: "Why?"
+A pause. "Because I've always done it. My old advisor told me years ago to do a backdoor Roth every year, and I never stopped."
+That autopilot answer is remarkably common. And for years, it was perfectly reasonable advice. But the tax landscape shifted in 2025, and a lot of surgeons haven't updated their thinking to match.
 ## The Assumption That Stopped Being Automatic
 Here's the conventional wisdom: contribute to a traditional IRA, convert immediately to a Roth, pay the taxes now, and let the money grow tax-free forever. For high earners locked out of direct Roth contributions, the backdoor strategy has been a staple for over a decade.
 The logic depended on one critical assumption: that tax rates would go up. If you believed rates were heading higher, paying taxes now at a "lower" rate and withdrawing later tax-free was a clear win.
@@ -967,7 +967,7 @@
 ## The Decision Tree You Should Be Using
 Rather than defaulting to "always do the Roth," the better approach is to walk through a simple framework. There are three branches, and your answer depends on where you sit today and where you're heading.
 **Branch 1: Roth still makes sense.** If your current marginal rate is relatively low (maybe you're in a transition year with lower income, or you're early in practice and not yet at peak earnings), and you expect your retirement income to be higher than it is today, or estate planning is a top priority (Roth IRAs have no required minimum distributions and pass tax-free to heirs under the current $15 million per person estate exemption), then funding the Roth remains a strong move. The tax-free growth and flexible withdrawal rules are genuinely powerful tools in estate and legacy planning.
-**Branch 2: Traditional and cash balance contributions win.** This is where Dr. K landed. She's 55, earning north of $1.2 million, paying a combined federal and state rate of 42%. She plans to retire at 62 and move from a state with a 5% income tax to one with no income tax. Her expected retirement withdrawal rate will place her around 24% federal.
+**Branch 2: Traditional and cash balance contributions win.** Consider a surgeon in this position. She's 55, earning north of $1.2 million, paying a combined federal and state rate of 42%. She plans to retire at 62 and move from a state with a 5% income tax to one with no income tax. Her expected retirement withdrawal rate will place her around 24% federal.
 At 42% now versus 24% later, every dollar she converts to a Roth is taxed at nearly double the rate she'd pay in retirement. The backdoor Roth contribution of $7,500 has already been taxed at 42% on the way in. The growth is tax-free, yes. But on the contribution itself, there's no tax arbitrage. She's paying the high rate and gaining nothing on the principal.
 Now consider the alternative. That same $7,500, redirected toward increasing her cash balance plan contribution, gets sheltered from taxation entirely at 42%. That's $3,150 in immediate tax savings. Over 10 years of tax-deferred compounding at 6%, that single redirect grows to $5,640 in tax savings. And the cash balance plan allows contributions of $150,000 to $350,000 or more per year, depending on age and plan design, which dwarfs the $7,500 (or $8,600 with catch-up) IRA limit.
 The Roth gave her tax-free growth on $7,500. The cash balance redirect gave her $3,150 in immediate savings, years of deferred compounding, and a dramatically larger contribution ceiling. The math isn't close.
@@ -982,7 +982,7 @@
 If your return showed that you're paying an effective rate above 38% and you don't have a cash balance plan in place, the backdoor Roth is almost certainly not the highest-value use of your next dollar. If your return showed strong tax deferral, low effective rates, and a fully funded retirement structure, then the Roth becomes a useful complementary tool for estate planning and tax diversification.
 The point is that the decision should follow the data. Not the calendar. Not the habit. Not the advice you received five years ago under a different tax code.
 ## Why This Matters Beyond April
-There's a deeper principle here that extends well past the filing deadline. The surgeons I work with who build the most durable wealth are the ones who resist autopilot. They question assumptions, even comfortable ones. They update their strategies when the rules change. They treat every financial decision with the same rigor they bring to a complex surgical case: evaluate the current data, consider the alternatives, choose deliberately.
+There's a deeper principle here that extends well past the filing deadline. The surgeons who build the most durable wealth are the ones who resist autopilot. They question assumptions, even comfortable ones. They update their strategies when the rules change. They treat every financial decision with the same rigor they bring to a complex surgical case: evaluate the current data, consider the alternatives, choose deliberately.
 A backdoor Roth is a fine tool. But a tool used reflexively, without evaluating whether it's the right tool for the current situation, isn't strategy. It's routine. And routine, in the operating room or on the balance sheet, is where outcomes quietly erode.
 Before April 15, take twenty minutes. Pull up your return (or the diagnostic from last week). Look at your current marginal rate. Look at your expected retirement rate. Look at your state tax trajectory. Then decide, with fresh eyes and current math, whether the Roth is the best use of that contribution or whether the capital serves you better somewhere else.
 The answer isn't "always do the Roth." The answer is: model both and choose deliberately.
@@ -1081,7 +1081,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>WEEK 3 (MARCH 16–22)</t>
+          <t>WEEK 3 (MARCH 9–15)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -1095,7 +1095,7 @@
     <row r="3" ht="120" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -1149,7 +1149,7 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1208,7 +1208,7 @@
     <row r="5" ht="120" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -1263,7 +1263,7 @@
     <row r="6" ht="120" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1290,7 +1290,7 @@
         <is>
           <t>Most orthopedic practices track revenue closely. Far fewer benchmark the three overhead categories that determine how much of that revenue the surgeon actually keeps.
 If a 2.5% reimbursement cut costs your practice $32,000 a year, and a 2% overhead reduction recovers the same $32,000 with zero additional procedures, the question becomes: where does that 2% come from?
-In my experience, there are three line items that almost always have room:
+When you analyze orthopedic practice overhead, there are three line items that almost always have room:
 → Supply and vendor contracts. When was the last time your practice benchmarked implant pricing, surgical supplies, and office materials against peer practices? Most practices haven't renegotiated in years. A 5% reduction in supply costs alone can recover $10,000 to $20,000 annually.
 → Staffing ratios. And I want to be clear: this is not about cutting staff. Practices that have grown over time often carry staffing structures built for an earlier version of the practice. Aligning roles, scheduling workflows, and staffing ratios with current patient volume can reduce overhead 1% to 3% without reducing quality of care.
 → Facility utilization. If you own your space or hold a long-term lease, unused operatory time, underutilized square footage, and energy costs add up quietly. For surgeon-owned buildings, a cost segregation study can also accelerate depreciation deductions on top of the overhead savings.
@@ -1318,7 +1318,7 @@
     <row r="7" ht="120" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>There is a question I ask almost every surgeon I work with, usually within the first two meetings. It tends to land quietly, and then it stays with them.
+          <t>There is a question worth asking every surgeon who owns a practice. It tends to land quietly, and then it stays with them.
 Is your practice structured to build wealth, or just to generate revenue?
 Because those are two very different things.
 A practice that generates revenue puts money through the door. A practice that builds wealth makes sure the surgeon keeps as much of it as possible, in the most tax-efficient way, through the most intentional structure.
@@ -1372,7 +1372,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>WEEK 4 (MARCH 23–29)</t>
+          <t>WEEK 4 (MARCH 16–22)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
@@ -1386,7 +1386,7 @@
     <row r="10" ht="120" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1446,12 +1446,12 @@
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Q1 Revenue Is In. Ask About Your Keep Rate Before Anything Else.</t>
+          <t>As Q1 Wraps Up, Ask About Your Keep Rate Before Anything Else.</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1466,27 +1466,27 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Ties the effective hourly rate concept to the Q1 close, making the post timely and actionable. Introduces "keep rate" as a digestible metric surgeons can track quarterly. Positions revenue growth without structural improvement as a warning sign, not a celebration.</t>
+          <t>Ties the effective hourly rate concept to the upcoming Q1 close, making the post timely and actionable. Introduces "keep rate" as a digestible metric surgeons can track quarterly. Positions revenue growth without structural improvement as a warning sign, not a celebration.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Q1 revenue data is in. Before you celebrate (or panic), ask this: did your keep rate go up or down?
+          <t>Q1 is wrapping up. When your revenue data lands, before you celebrate (or panic), ask this: did your keep rate go up or down?
 Keep rate is simple. It's the percentage of gross revenue that actually flows to your personal wealth after overhead, taxes, debt service, and savings. If your practice collected $600K in Q1 and you kept $120K, your keep rate is 20%.
 Here's why this matters more than the top-line number.
-I see this pattern regularly: a practice grows revenue by 8% year over year, the surgeon feels good about the trajectory, but overhead crept up by 10%. Taxes increased because the additional income pushed into a higher marginal bracket. And the retirement plan wasn't restructured to capture the growth.
+This is a structural pattern that shows up frequently in surgeon-owned practices: a practice grows revenue by 8% year over year, the surgeon feels good about the trajectory, but overhead crept up by 10%. Taxes increased because the additional income pushed into a higher marginal bracket. And the retirement plan wasn't restructured to capture the growth.
 The result? Revenue went up. Keep rate went down. The practice got busier and more profitable on paper, and the surgeon's personal wealth-building actually slowed.
 Revenue growth without structural improvement means the practice generates more income for everyone except you. More for overhead. More for the IRS. More for lenders. The surgeon works harder, and the gap between collections and kept income widens.
 Your Q1 vital sign isn't revenue growth. It's keep rate direction.
 If revenue grew and keep rate grew with it, your structure is working. If revenue grew and keep rate stayed flat or declined, that's the signal to look under the hood before Q2 begins.
-One number. One question. That's your Q1 financial check-up.</t>
+One number. One question. That's your Q1 financial check-up when the numbers come in.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Primary Image
 Image type: Stat highlight card
-Rationale: The question-driven format creates engagement by prompting self-reflection. A simple keep rate metric on the card gives surgeons a framework they can immediately apply to their own Q1 data.
+Rationale: The question-driven format creates engagement by prompting self-reflection. A simple keep rate metric on the card gives surgeons a framework they can apply when their Q1 data comes in.
 AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with 80px side margins. Upper third: "Q1 Keep Rate" in Inter Medium, approximately 28pt, Warm Gray (#9AA3A8), centered, positioned at roughly 28% from top. Center: a large upward or downward arrow icon composed of two versions side by side (one pointing up in Antique Gold #B08D57, one pointing down in Blue Slate #5F7483), each approximately 80px tall, separated by 40px, centered horizontally at 50% vertical. Lower third: "Which direction is yours?" in Playfair Display SemiBold, approximately 40pt, Off-White (#F6F7F5), centered, positioned at roughly 72% from top. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, direct, serious. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
 Text overlay: "Q1 Keep Rate" in Inter Medium, ~28pt, Warm Gray (#9AA3A8), upper center. "Which direction is yours?" in Playfair Display SemiBold, ~40pt, Off-White (#F6F7F5), lower center.
 Platform and dimensions: LinkedIn, 1080x1080</t>
@@ -1501,7 +1501,7 @@
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1555,7 +1555,7 @@
     <row r="13" ht="120" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1610,7 +1610,7 @@
     <row r="14" ht="120" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1665,7 +1665,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>WEEK 5 (MARCH 30 – APRIL 5)</t>
+          <t>WEEK 5 (MARCH 23–29)</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
@@ -1679,7 +1679,7 @@
     <row r="17" ht="120" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Opens the April "Post-Filing Insights" month by reframing the tax return from a compliance document into a strategic diagnostic. Compresses the anchor blog's four-marker framework into a single, actionable LinkedIn post that positions the return as the most underread financial document a surgeon owns.</t>
+          <t>Leads into April's "Post-Filing Insights" month by reframing the tax return from a compliance document into a strategic diagnostic. Compresses the anchor blog's four-marker framework into a single, actionable LinkedIn post that positions the return as the most underread financial document a surgeon owns.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1732,7 +1732,7 @@
     <row r="18" ht="120" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1760,7 +1760,7 @@
           <t>A surgeon's return showed $31,000 in retirement contributions. The available capacity was $203,000. That $172,000 gap compounds every single year.
 Here is what that gap looks like in practice.
 A 401(k) with catch-up contributions for a surgeon over 50 allows $32,500 annually. Add a profit-sharing layer through an S-Corp, and you reach roughly $70,000. Layer in a cash balance plan, and the total available capacity can push past $200,000 in a single year, all tax-deferred.
-Most surgeons I see are using the 401(k) only. Some are maxing the employee contribution. Very few are using the profit-sharing component at all. Almost none have a cash balance plan in place.
+Most surgeons at this income level are using the 401(k) only. Some are maxing the employee contribution. Very few are using the profit-sharing component at all. Almost none have a cash balance plan in place.
 The result shows up on one line of the return: retirement plan contributions. And when that line reads $31,000 instead of $203,000, you are looking at the single largest structural gap in most surgical practices.
 This is not about being irresponsible. The surgeon in this example was disciplined, productive, and well-compensated. But the plan structure underneath was never built for an income at this level. A 401(k) designed for a $150,000 earner does not do the same work for someone earning $900,000.
 The tax return is where this shows up most clearly. One line. One number. And a gap that, over a decade, costs more than most people's houses.
@@ -1786,7 +1786,7 @@
     <row r="19" ht="120" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1817,7 +1817,7 @@
 For a surgeon earning $1.2M, the planning decisions available during the extension period can shift the tax outcome by $40,000 to $80,000. That is not a rounding error. That is the difference between a return that was filed and a return that was optimized.
 The catch is that most people treat the extension as extra time to gather documents. They file the extension in April, put the return out of mind, and scramble again in September. The six-month window closes without a single strategic decision being made.
 Used correctly, the extension period is when you sit down with your return (or last year's return, if this year's is still being prepared), identify the four diagnostic markers, and build a plan to close any structural gaps before October.
-If you filed an extension this year, you are not behind. You are in the strongest planning position of the calendar. The question is whether you will use the time.
+If you're planning to file an extension, or if you've already filed one, you are not behind. You are in the strongest planning position of the calendar. The question is whether you will use the time.
 What is one decision you could make before October 15 that would change next year's return?</t>
         </is>
       </c>
@@ -1840,7 +1840,7 @@
     <row r="20" ht="120" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1870,7 +1870,7 @@
 But here's where it gets interesting. The QBI deduction is one of the most misunderstood lines on a surgeon's return because its presence or absence is almost entirely determined by how your S-Corp salary is set.
 Pay yourself too much in W-2 salary relative to the practice's net income, and the qualified business income shrinks or disappears entirely. The deduction drops to zero. Pay yourself a reasonable but carefully calibrated salary, and the QBI deduction appears, sometimes worth $25,000 to $35,000.
 The line between those two outcomes is not luck. It is structure. Specifically, it is the ratio between your W-2 salary and your total S-Corp distributions, and whether anyone has looked at that ratio since you set up the entity.
-I've seen surgeons with nearly identical gross incomes file returns with a $30,000 difference in QBI deductions. Same specialty, same region, same revenue range. The only variable was how the S-Corp salary had been calibrated.
+Surgeons with nearly identical gross incomes can file returns with a $30,000 difference in QBI deductions. Same specialty, same region, same revenue range. The only variable is how the S-Corp salary has been calibrated.
 If your return shows a QBI deduction, check whether the amount reflects your full available capacity. If it shows zero, ask why. The answer usually points to a salary calibration conversation that should have happened a year ago.</t>
         </is>
       </c>
@@ -1893,7 +1893,7 @@
     <row r="21" ht="120" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1948,7 +1948,7 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>WEEK 6 (APRIL 6–12)</t>
+          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
         </is>
       </c>
       <c r="B23" s="3" t="n"/>
@@ -1962,7 +1962,7 @@
     <row r="24" ht="120" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -2017,7 +2017,7 @@
     <row r="25" ht="120" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -2072,7 +2072,7 @@
     <row r="26" ht="120" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -2126,7 +2126,7 @@
     <row r="27" ht="120" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -2181,7 +2181,7 @@
     <row r="28" ht="120" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -2303,7 +2303,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>WEEK 3 (MARCH 16–22)</t>
+          <t>WEEK 3 (MARCH 9–15)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -2317,7 +2317,7 @@
     <row r="3" ht="120" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -2342,11 +2342,11 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>I keep hearing from surgeons that the CMS reimbursement cuts feel like death by a thousand cuts.
+          <t>The CMS reimbursement cuts feel like death by a thousand cuts.
 They're not wrong.
 Every year, the per-procedure number gets a little smaller. And every year, the instinctive response is the same: work more, schedule more, add more cases to make up the difference.
 I understand why that feels like the answer. It's action. It's tangible. It looks like progress on a spreadsheet.
-But here's what I've noticed, working alongside surgeon-owned practices for years. The ones who respond to reimbursement pressure by adding volume end up running faster on the same treadmill. And the ones who pause, look at how their practice income actually flows, and tighten the system? They recover more, keep more, and spend fewer hours in the OR doing it.
+But here's the structural pattern. The practices that respond to reimbursement pressure by adding volume end up running faster on the same treadmill. And the ones that pause, look at how practice income actually flows, and tighten the system? They recover more, keep more, and the surgeons spend fewer hours in the OR doing it.
 The difference isn't how much revenue comes in. It's what happens to that revenue between the point where the practice collects it and the point where it reaches you.
 If that distinction feels worth exploring, we wrote something this week that walks through it in detail. Link in the comments.</t>
         </is>
@@ -2370,7 +2370,7 @@
     <row r="4" ht="120" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Story-driven post using an anonymized client composite to make the structural optimization argument tangible. While colleagues were working longer hours, this surgeon spent an afternoon reviewing practice overhead and recovered more than the reimbursement gap. Designed for mid-week (Wednesday) to build on the conceptual foundation laid in Facebook 1.</t>
+          <t>Story-driven post using an illustrative scenario to make the structural optimization argument tangible. While colleagues were working longer hours, this surgeon spent an afternoon reviewing practice overhead and recovered more than the reimbursement gap. Designed for mid-week (Wednesday) to build on the conceptual foundation laid in Facebook 1.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>I want to share a quick story (details changed for privacy, of course).
-A surgeon I work with came to me earlier this year, frustrated about the CMS reimbursement cut. Several of his partners and colleagues were already planning to add cases to their schedules. One was talking about picking up extra half-days every other week. Another was considering expanding into a new procedure just to fill the revenue gap.
-This surgeon didn't do any of that. Instead, he blocked out a Tuesday afternoon, sat down with his practice administrator, and pulled three reports: supply costs per procedure, staffing ratios, and their vendor contracts.
-What they found surprised them both. Two of their implant vendors hadn't been rebid in over four years. Their staffing ratio was running a full position above the MGMA benchmark for their practice size. And they were paying for a software subscription that had been auto-renewing since 2021 for a system they'd stopped using in 2023.
-Total savings once they made the adjustments? Just over $40,000 a year. More than the entire reimbursement gap, recovered without a single extra case, a single extra OR hour, or a single extra ounce of fatigue.
-His colleagues are working more. He's working the same amount and keeping more. That difference compounds every single year.</t>
+          <t>Here's a scenario that illustrates the opportunity sitting inside most practices.
+A surgeon hears about the CMS reimbursement cut. Several of his partners and colleagues are already planning to add cases to their schedules. One is talking about picking up extra half-days every other week. Another is considering expanding into a new procedure just to fill the revenue gap.
+But instead of adding volume, this surgeon blocks out a Tuesday afternoon, sits down with his practice administrator, and pulls three reports: supply costs per procedure, staffing ratios, and vendor contracts.
+What they find surprises them both. Two implant vendors haven't been rebid in over four years. The staffing ratio is running a full position above the MGMA benchmark for their practice size. And they're paying for a software subscription that has been auto-renewing since 2021 for a system they stopped using in 2023.
+Total savings once they make the adjustments? Just over $40,000 a year. More than the entire reimbursement gap, recovered without a single extra case, a single extra OR hour, or a single extra ounce of fatigue.
+The colleagues are working more. This surgeon is working the same amount and keeping more. That difference compounds every single year.</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2422,7 +2422,7 @@
     <row r="5" ht="120" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -2452,7 +2452,7 @@
 "What are our three highest supply costs per procedure, and when was the last time we benchmarked them?"
 That's it. You don't need to renegotiate anything today. You don't need to fire a vendor or overhaul your supply chain. Just ask the question and listen to the answer.
 Here's why. Most orthopedic practices set their vendor relationships years ago and haven't revisited them since. The rep is great, the products work, and nobody has time to shop around. I get it. But pricing drifts. Competitors introduce new options. And what was a competitive rate in 2021 may not be competitive in 2026.
-The surgeons I work with who have the most efficient practices aren't necessarily the ones who negotiate the hardest. They're the ones who ask the question regularly. That habit, by itself, tends to surface opportunities that would otherwise sit invisible in the overhead.
+The surgeons who run the most efficient practices aren't necessarily the ones who negotiate the hardest. They're the ones who ask the question regularly. That habit, by itself, tends to surface opportunities that would otherwise sit invisible in the overhead.
 One question. Five minutes. It might be the most productive thing you do for your bottom line this week.</t>
         </is>
       </c>
@@ -2475,7 +2475,7 @@
     <row r="6" ht="120" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -2501,11 +2501,11 @@
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Something I've been thinking about this week.
-The CMS reimbursement cut is real. Nobody enjoys earning less per procedure. But the more I look at the practices that are feeling it most, the more I notice a pattern: the cut didn't create a new problem. It made an existing one louder.
+The CMS reimbursement cut is real. Nobody enjoys earning less per procedure. But the more you look at the practices that are feeling it most, the clearer a pattern becomes: the cut didn't create a new problem. It made an existing one louder.
 Over the past couple of weeks, I've been writing about the structural gaps that quietly drain surgeon wealth. Things like an S-Corp salary that hasn't been recalibrated in years, retirement plans that aren't using their full capacity, depreciation strategies that were never implemented on a building the surgeon already owns.
 Those gaps existed before January 1. They were just easier to ignore when revenue was higher.
 The reimbursement cut is uncomfortable, but it's also clarifying. It's the financial equivalent of an imaging result you weren't expecting. You can be frustrated by the finding, or you can use it as a reason to look more carefully at the structure underneath.
-Most of the surgeons I work with, once they actually trace how their income flows from the practice to their personal balance sheet, find that the structural leaks are costing them far more than the CMS cut ever will.
+When surgeons actually trace how their income flows from the practice to their personal balance sheet, they typically find that the structural leaks cost far more than the CMS cut ever will.
 That's the real conversation worth having this quarter.</t>
         </is>
       </c>
@@ -2528,7 +2528,7 @@
     <row r="7" ht="120" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Week 3 (March 16–22)</t>
+          <t>Week 3 (March 9–15)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -2581,7 +2581,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>WEEK 4 (MARCH 23–29)</t>
+          <t>WEEK 4 (MARCH 16–22)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
@@ -2595,7 +2595,7 @@
     <row r="10" ht="120" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -2620,9 +2620,9 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>I've been working with surgeons long enough to know that most of them can quote their collections number off the top of their head. Ask them what they actually keep per hour of clinical work, though, and the room goes quiet.
-This week I sat down with a surgeon who was having a great year. Collections were up. Volume was strong. He felt like things were going well, and honestly, they were.
-Then we ran one calculation he'd never thought to run. We took his collections, subtracted overhead, taxes, retirement contributions, and debt service, then divided by the hours he actually spends doing clinical work.
+          <t>Most surgeons can quote their collections number off the top of their head. Ask them what they actually keep per hour of clinical work, though, and the room goes quiet.
+Here's a scenario that illustrates the gap. Consider a surgeon having a great year. Collections are up. Volume is strong. He feels like things are going well, and honestly, they are.
+Then he runs one calculation he's never thought to run. Take collections, subtract overhead, taxes, retirement contributions, and debt service, then divide by the hours actually spent doing clinical work.
 The number was $146 an hour.
 He had assumed it was somewhere north of $350. The gap between those two numbers wasn't a failure. It was a diagnosis. And like any good diagnosis, it pointed directly to where the treatment plan should focus.
 That gap is where your financial structure lives. And most surgeons have never looked at it.</t>
@@ -2647,7 +2647,7 @@
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -2667,14 +2667,14 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>End-of-month reflective wrap post. Closes the four-week Q1 Financial Health Check arc with a single takeaway that unifies Weeks 1 through 4. Brief, warm, designed to land gently rather than teach.</t>
+          <t>Reflective wrap post that closes the four-week Q1 Financial Health Check arc with a single takeaway that unifies Weeks 1 through 4. Brief, warm, designed to land gently rather than teach. Closes the four-week Q1 Financial Health Check arc with a single takeaway that unifies Weeks 1 through 4. Brief, warm, designed to land gently rather than teach.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>March is almost over. We've covered a lot this month: entity structure, S-Corp salary calibration, what happens when reimbursements shift, and (this week) the one number that ties it all together.
+          <t>We've covered a lot this month: entity structure, S-Corp salary calibration, what happens when reimbursements shift, and (this week) the one number that ties it all together.
 If you take one thing from the last four weeks, let it be this: the amount your practice earns and the amount you keep are two very different numbers. Understanding the gap between them is where real financial planning begins.
-You don't need to overhaul everything at once. You just need to know where you stand. And now, with a quarter of real data behind you, is a good time to look.</t>
+You don't need to overhaul everything at once. You just need to know where you stand. And as Q1 closes, when you have a quarter of real data in front of you, that's a good time to look.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -2696,7 +2696,7 @@
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -2722,10 +2722,10 @@
       <c r="F12" s="6" t="inlineStr">
         <is>
           <t>If you have 15 minutes this week, here's the most valuable thing you can do with them.
-Pull your Q1 collections. You probably already know this number, but write it down. Then subtract your overhead (your practice management software has this, or your office manager does). Subtract what you paid in estimated taxes. Subtract your retirement contributions. Subtract your debt service.
-Whatever is left, divide by the number of clinical hours you worked this quarter.
+As Q1 wraps up, pull your year-to-date collections. You probably already know this number, but write it down. Then subtract your overhead (your practice management software has this, or your office manager does). Subtract what you paid in estimated taxes. Subtract your retirement contributions. Subtract your debt service.
+Whatever is left, divide by the number of clinical hours you've worked so far this year.
 That's your effective hourly rate. It's what you actually kept for every hour you spent in the OR, in clinic, on call.
-Most surgeons I work with have never seen this number before. And almost all of them are surprised by it. Not because the number is bad, necessarily, but because the gap between what they assumed and what the math shows is wider than they expected.
+Most surgeons have never seen this number before. And almost all of them are surprised by it. Not because the number is bad, necessarily, but because the gap between what they assumed and what the math shows is wider than they expected.
 It takes about 15 minutes. And it changes how you think about everything else.</t>
         </is>
       </c>
@@ -2734,8 +2734,8 @@
           <t>Primary Image
 Image type: Quote/insight card
 Rationale: A clean card with the five-step framework compressed into a visual creates a "save this post" moment. The simplicity of the steps contrasts with the power of the result, which is the hook.
-AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: left-aligned text composition with 80px left margin and 60px top margin. Header text: "Your Effective Hourly Rate" in Playfair Display SemiBold, approximately 28pt, Antique Gold (#B08D57), left-aligned, positioned at the top of the text block. Below the header, with 32px spacing, five lines of text in Inter Regular, approximately 16pt, Off-White (#F6F7F5), left-aligned, with 20px vertical spacing between each line: "Q1 Collections", "− Overhead", "− Taxes", "− Retirement", "− Debt Service", "÷ Clinical Hours". A thin vertical accent line (2px, Antique Gold #B08D57) runs along the left edge of the text block, from the top of the header to the bottom of the last line, positioned 60px from the left edge. Below the last line, with 28px spacing, a horizontal rule (1px, Warm Gray #9AA3A8) spanning 50% of canvas width from the left margin. Below the rule, with 16px spacing: "= ?" in Playfair Display SemiBold, approximately 36pt, Antique Gold (#B08D57), left-aligned. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 24px from edges, approximately 60px wide. No imagery, no illustrations, no gradients, no drop shadows, no photographs. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no busy compositions. Mood: clear, inviting, purposeful. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Your Effective Hourly Rate" in Playfair Display SemiBold, ~28pt, Antique Gold (#B08D57), top-left. Five calculation steps in Inter Regular, ~16pt, Off-White (#F6F7F5), stacked below. "= ?" in Playfair Display SemiBold, ~36pt, Antique Gold (#B08D57), below the rule.
+AI image prompt: Create a 1200x630px landscape social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: left-aligned text composition with 80px left margin and 60px top margin. Header text: "Your Effective Hourly Rate" in Playfair Display SemiBold, approximately 28pt, Antique Gold (#B08D57), left-aligned, positioned at the top of the text block. Below the header, with 32px spacing, five lines of text in Inter Regular, approximately 16pt, Off-White (#F6F7F5), left-aligned, with 20px vertical spacing between each line: "Collections (YTD)", "− Overhead", "− Taxes", "− Retirement", "− Debt Service", "÷ Clinical Hours". A thin vertical accent line (2px, Antique Gold #B08D57) runs along the left edge of the text block, from the top of the header to the bottom of the last line, positioned 60px from the left edge. Below the last line, with 28px spacing, a horizontal rule (1px, Warm Gray #9AA3A8) spanning 50% of canvas width from the left margin. Below the rule, with 16px spacing: "= ?" in Playfair Display SemiBold, approximately 36pt, Antique Gold (#B08D57), left-aligned. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 24px from edges, approximately 60px wide. No imagery, no illustrations, no gradients, no drop shadows, no photographs. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no busy compositions. Mood: clear, inviting, purposeful. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Your Effective Hourly Rate" in Playfair Display SemiBold, ~28pt, Antique Gold (#B08D57), top-left. Five calculation steps (Collections YTD, overhead, taxes, retirement, debt service, clinical hours) in Inter Regular, ~16pt, Off-White (#F6F7F5), stacked below. "= ?" in Playfair Display SemiBold, ~36pt, Antique Gold (#B08D57), below the rule.
 Platform and dimensions: Facebook, 1200x630</t>
         </is>
       </c>
@@ -2748,7 +2748,7 @@
     <row r="13" ht="120" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -2774,7 +2774,7 @@
       <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Here's something I think about a lot.
-Every surgeon I know can tell you their collections. It shows up in practice reports, partner meetings, year-end summaries. Your practice tracks it. Your partners compare it. Your accountant files around it.
+Most surgeons can tell you their collections. It shows up in practice reports, partner meetings, year-end summaries. Your practice tracks it. Your partners compare it. Your accountant files around it.
 But nobody reports what you actually keep per hour of clinical work. It doesn't show up in any dashboard. No practice management system calculates it. No year-end report highlights it.
 And that's the problem. We measure what others report to us. Collections get tracked because someone else built a system to track them. Your keep rate doesn't get tracked because nobody built that system. It falls in the gap between your practice financials and your personal finances, a space that nobody owns.
 Which means the most important financial number in your life (the one that tells you whether your structure is actually working) is the one nobody is watching.
@@ -2800,7 +2800,7 @@
     <row r="14" ht="120" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Week 4 (March 23–29)</t>
+          <t>Week 4 (March 16–22)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -2851,7 +2851,7 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>WEEK 5 (MARCH 30 – APRIL 5)</t>
+          <t>WEEK 5 (MARCH 23–29)</t>
         </is>
       </c>
       <c r="B16" s="3" t="n"/>
@@ -2865,7 +2865,7 @@
     <row r="17" ht="120" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -2890,8 +2890,8 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Tax season confession: the first time I really looked at a surgeon client's return for strategy instead of compliance, I found $172,000 in unused retirement plan capacity. Every year. For years.
-They weren't doing anything wrong. Their CPA was solid. The return was accurate. Every number checked out.
+          <t>Here's a scenario worth sitting with. Take a surgeon's return and read it for strategy instead of compliance. What shows up? $172,000 in unused retirement plan capacity. Every year. For years.
+Nothing was wrong with the compliance work. The CPA was solid. The return was accurate. Every number checked out.
 But nobody had ever read it the way a surgeon reads an MRI, looking for what's not there as much as what is.
 That's the thing about tax returns. They're incredibly precise documents that almost nobody uses diagnostically. For most orthopedic surgeons earning $600K to $1.2M, the return gets filed, the refund or payment clears, and the whole thing goes in a drawer until next year.
 Meanwhile, four lines on that return can tell you more about the trajectory of your financial life than a quarter's worth of portfolio reports.
@@ -2917,7 +2917,7 @@
     <row r="18" ht="120" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -2937,15 +2937,15 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Normalizes the filing extension for surgeons who feel behind. Reframes the extension as a strategic window rather than a sign of procrastination. Positioned mid-week to catch surgeons who filed extensions in mid-March and may be second-guessing that decision.</t>
+          <t>Normalizes the filing extension for surgeons who feel behind. Reframes the extension as a strategic window rather than a sign of procrastination. Positioned mid-week to catch surgeons who are considering an extension or have filed one early and may be second-guessing that decision.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>If you filed an extension this year, you might be carrying a little guilt about it. I hear this from surgeons more than you'd expect.
+          <t>If you're planning to file an extension this year, or if you've already filed one, you might be carrying a little guilt about it. It's a more common reaction than you'd expect.
 Here's what I'd tell you over coffee: you didn't procrastinate. You gave yourself six months to optimize.
 An extension moves your filing deadline to October 15. It doesn't change when your taxes are due (that was still April 15), and it doesn't trigger any penalties as long as your estimated payment was reasonable. What it does give you is time. Time to fund a cash balance plan. Time to restructure entity elections. Time to finish a cost segregation study on that rental property you closed on in February.
-Most of the surgeons I work with who file extensions do so deliberately, because the strategy work takes longer than the compliance work.
+Surgeons who file extensions deliberately know something the others don't: the strategy work takes longer than the compliance work.
 So if you're sitting on an extension right now, treat these next six months as a planning window. What's one thing on your return you'd like to understand better before you file?</t>
         </is>
       </c>
@@ -2968,7 +2968,7 @@
     <row r="19" ht="120" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -2993,9 +2993,9 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>There's a moment I see fairly often in first meetings with surgeon clients. We pull up their most recent return, and I ask one question: "Do you know your effective tax rate?"
-Almost every time, the answer is their marginal bracket. "37 percent." Sometimes "40-something, with state."
-Then we do the actual math. Total tax divided by total income. And the number that comes back is usually lower than they expected. Sometimes significantly lower.
+          <t>Here's a question worth asking with your return in front of you: "Do you know your effective tax rate?"
+Most surgeons answer with their marginal bracket. "37 percent." Sometimes "40-something, with state."
+Then you do the actual math. Total tax divided by total income. And the number that comes back is usually lower than expected. Sometimes significantly lower.
 You'd think that would be good news. And it is, briefly. But then the next question lands: "Wait, if my effective rate is that low, does that mean my deductions are actually working? Or does it mean I'm missing something bigger?"
 That's the moment the return stops being a compliance document and starts being a diagnostic tool.
 If you want to find yours, it's a two-line calculation. Take your total tax (line 24 on your 1040) and divide it by your total income (line 15). That single percentage tells you more than your bracket ever will.
@@ -3021,7 +3021,7 @@
     <row r="20" ht="120" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -3049,7 +3049,7 @@
           <t>There's a line on your tax return that might read $0 when it could read $29,800. And if you've never heard of it, you're in good company.
 The QBI deduction (Qualified Business Income, Section 199A) allows certain pass-through business owners to deduct up to 20% of their qualified business income. For an orthopedic surgeon earning practice income through an S-corp or partnership, that can translate into a meaningful reduction in taxable income every single year.
 The catch? Surgeons often get told they "make too much" to qualify. And for some, that's true. But the income thresholds interact with filing status, entity structure, and how W-2 wages are set within the practice. The details matter, and they're not always intuitive.
-I've seen surgeons who assumed they were phased out discover, after a closer look at their entity setup, that they qualified all along.
+It's not uncommon for surgeons who assumed they were phased out to discover, after a closer look at their entity setup, that they qualified all along.
 Pull up your 1040 and look for Form 8995 or 8995-A. If it's missing entirely, that's worth a conversation with your tax advisor.
 Have you checked yours?</t>
         </is>
@@ -3073,7 +3073,7 @@
     <row r="21" ht="120" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Week 5 (March 30 – April 5)</t>
+          <t>Week 5 (March 23–29)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>March was about looking at the numbers. Your effective tax rate. Your retirement contributions. Your QBI deduction. Your state tax exposure. Four lines on a return that most people file and forget.
+          <t>This month we've been looking at the numbers. Your effective tax rate. Your retirement contributions. Your QBI deduction. Your state tax exposure. Four lines on a return that most people file and forget.
 If you followed along this month, you've already done something most surgeons never do: you treated your tax return like a diagnostic report instead of a receipt.
 That's a meaningful shift. And if it raised more questions than it answered, that's actually the point. A good diagnostic doesn't give you closure. It gives you clarity about where to look next.
 April is where we start interpreting. We'll get into what those numbers actually mean in the context of your broader financial picture, how they connect to your retirement timeline, your practice structure, and the decisions you're making (or putting off) about the next phase.
@@ -3125,7 +3125,7 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>WEEK 6 (APRIL 6–12)</t>
+          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
         </is>
       </c>
       <c r="B23" s="3" t="n"/>
@@ -3139,7 +3139,7 @@
     <row r="24" ht="120" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -3164,9 +3164,9 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>April 15 is next week. Quick reminder: it's more than a filing deadline.
+          <t>April 15 is two weeks away. Quick reminder: it's more than a filing deadline.
 It's also the last day to make a prior-year IRA contribution (up to $7,500 if you're over 50). And it's the due date for your Q1 estimated tax payment. Three decisions, one date.
-Most surgeons I work with are focused on the filing question. That's understandable. But I've watched the filing conversation crowd out the other two, and those two decisions often have a bigger impact on the year ahead.
+Most surgeons focus on the filing question. That's understandable. But the filing conversation tends to crowd out the other two, and those two decisions often have a bigger impact on the year ahead.
 Whether you file or extend, that's a process question. Whether you fund a prior-year IRA and how you calibrate your Q1 estimated payment? Those are strategy questions. They shape your tax position for the rest of 2026.
 If you're meeting with your CPA this week, bring all three to the table. Filing is one piece. The other two deserve their own conversation.</t>
         </is>
@@ -3190,7 +3190,7 @@
     <row r="25" ht="120" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -3216,7 +3216,7 @@
       <c r="F25" s="6" t="inlineStr">
         <is>
           <t>If you're filing an extension this year, I want you to hear something: that's a perfectly reasonable decision.
-More than half the surgeon clients I work with extend. The reason is simple. Complex returns take time, and rushing a return with multiple entities, retirement plan contributions, and K-1s waiting to arrive doesn't help anyone. An extension gives you until October 15 to file accurately and thoughtfully.
+More than half of high-income filers extend. The reason is simple. Complex returns take time, and rushing a return with multiple entities, retirement plan contributions, and K-1s waiting to arrive doesn't help anyone. An extension gives you until October 15 to file accurately and thoughtfully.
 Here's what most people miss about that window. The six months between April and October are some of the most valuable planning months of the year. Your Q1 income is visible. Your practice trajectory for the year is taking shape. You have real numbers to work with, not projections from last November.
 The surgeons who use the extension window well don't just file a better return. They make better decisions about estimated payments, retirement contributions, and entity distributions along the way.
 So if you extended, don't feel behind. You just gave yourself room to be more deliberate. Use it.</t>
@@ -3241,7 +3241,7 @@
     <row r="26" ht="120" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -3266,8 +3266,8 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>I've noticed something interesting in the conversations I have with surgeons this time of year.
-Almost every one of them funds a backdoor Roth IRA. It's on the annual checklist. Contribute $7,500 to a traditional IRA, convert it, move on. Many have been doing it for years without a second thought.
+          <t>There's an interesting pattern that surfaces this time of year.
+A large number of surgeons fund a backdoor Roth IRA every April. It's on the annual checklist. Contribute $7,500 to a traditional IRA, convert it, move on. Many have been doing it for years without a second thought.
 And for a long time, that was the right call. When the top rate was expected to sunset back to 39.6%, converting at a potentially lower rate today made strong mathematical sense.
 But the landscape shifted. Under OBBBA, the 37% top rate is now permanent. That changes the calculus. If you're paying 37% on the conversion today and you expect to be in a lower bracket in retirement, the backdoor Roth may actually cost you more than it saves.
 I'm not saying stop doing it. For many surgeons, the Roth still works. What I am saying is that a strategy you set up five years ago deserves a fresh look under the current rules.
@@ -3293,7 +3293,7 @@
     <row r="27" ht="120" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -3345,7 +3345,7 @@
     <row r="28" ht="120" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Week 6 (April 6–12)</t>
+          <t>Week 6 (March 30 – April 5)</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -3370,8 +3370,8 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>There's a particular kind of stress that builds in the days before April 15. I see it every year, even among surgeons who have everything organized, who have excellent CPAs, who are in great financial shape. The date itself carries weight.
-But here's something I've come to believe after years of working through this week with clients. April 15 is more useful as a decision point than as a deadline.
+          <t>There's a particular kind of stress that builds in the days before April 15. It shows up even among surgeons who have everything organized, who have excellent CPAs, who are in great financial shape. The date itself carries weight.
+But here's a perspective worth considering. April 15 is more useful as a decision point than as a deadline.
 A deadline asks: did you get it done? A decision point asks: are you on the right path?
 Filing is important. But the real value of this week is the chance to step back and look at the bigger picture. Did your financial structure serve you well over the past twelve months? Are the decisions you made last year still the right ones for this year? Is anything different enough to warrant a change?
 You operate on joints every day, making precise adjustments that compound over time. Your financial life works the same way. Small, well-timed decisions matter more than dramatic moves.

</xml_diff>

<commit_message>
Add podcast clip drafts (weeks 3-6) and update batch exporter
- Add 14 podcast clip drafts across weeks 3-6
- Update export script and batch summary spreadsheet

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/outputs/drafts/content-batch-2026-02-27/content-batch-summary-20260227.xlsx
+++ b/outputs/drafts/content-batch-2026-02-27/content-batch-summary-20260227.xlsx
@@ -8,13 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facebook" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podcast" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clips" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facebook" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Blog'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'LinkedIn'!$A$1:$H$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Facebook'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Podcast'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Clips'!$A$1:$H$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'LinkedIn'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Facebook'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1023,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1092,7 +1096,7 @@
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n"/>
     </row>
-    <row r="3" ht="120" customHeight="1">
+    <row r="3" ht="200" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Week 3 (March 9–15)</t>
@@ -1100,1146 +1104,1640 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>CMS Cut Your Reimbursement by 2.5%. Your Financial Advisor Probably Didn't Mention It.</t>
+          <t>Your Practice Makes Less Per Procedure Than It Did Last Year. Here's What to Do About It.</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Reimbursement Shift and Practice Wealth</t>
+          <t>The reimbursement shift and what it means for your wealth</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn Post</t>
+          <t>Video Podcast Script (uploaded to YouTube; audio distributed to podcast platforms)</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Opens the week's LinkedIn sequence by reframing the CMS 2.5% efficiency adjustment as a financial planning event rather than a practice management issue. Drives curiosity and positions Capable Wealth as the advisor who connects practice economics to personal wealth.</t>
+          <t>CMS's 2.5% "efficiency adjustment" on non-time-based orthopedic procedures has been active since January 1. Surgeons are now seeing 10+ weeks of reduced reimbursements reflected in their Q1 numbers. This episode reframes the reimbursement cut as a structural planning event, challenges the instinctive "do more volume" response, and walks through three concrete alternatives that protect personal wealth without requiring additional OR time. Builds on Weeks 1–2 (entity structure, S-Corp salary optimization) by extending the structural lens to practice economics.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>CMS cut your reimbursement by 2.5%. Your practice manager told you. Your financial advisor probably didn't.
-That gap matters.
-The 2.5% efficiency adjustment on non-time-based orthopedic codes has been active since January 1. If you perform 400 procedures a year at an average reimbursement of $3,200, the math is simple: $80 less per procedure, $32,000 less per year.
-Your practice manager sees a billing issue. Your accountant will see it in your year-end numbers. But the question nobody seems to be asking is what $32,000 in reduced revenue means for your retirement contributions, your tax positioning, and the long-term trajectory of your personal wealth.
-A reimbursement cut is a financial planning event. Every dollar your practice earns just became more valuable, which means how those dollars flow from your entity to your personal balance sheet matters more than it did six months ago.
-If your S-Corp salary hasn't been recalibrated since revenues dropped, you may be compounding the loss. If your retirement plan contributions haven't been reexamined in light of reduced income, you could be leaving additional tax-deferred growth on the table.
-The surgeons who absorb this cut without feeling it are the ones whose financial structure was already built for efficiency. The ones who feel it most are the ones who were already running at the margin.
-Which side of that line are you on?</t>
+          <t>## Clip Extraction Map
+### Clip 1
+- **Source segment:** Segment 2: The Volume Trap
+- **Timestamp markers:** "So those 10 additional procedures..." through "...You did 100% more work to get back 39% of what you lost."
+- **Hook line:** "Adding 10 procedures to offset a $32K revenue loss sounds logical. Here's why it costs you more than it recovers."
+- **Core insight:** The marginal cost of additional procedures consumes ~60% of the revenue, so 10 extra cases only recover $12,480 of a $32K gap. A 39% recovery rate for 100% more work.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~55 seconds
+### Clip 2
+- **Source segment:** Segment 3: Three Overhead Line Items
+- **Timestamp markers:** "The first is supply costs..." through "...Most practices just never use it."
+- **Hook line:** "Most orthopedic practices negotiate implant pricing once and never revisit it. That single habit could be costing you $40,000 a year."
+- **Core insight:** Implant pricing varies 15-30% across vendors for equivalent devices. A 10% reduction on $400K in annual supply spend saves $40K, more than the entire reimbursement gap.
+- **Platform tags:** [IG-REEL]
+- **Estimated duration:** ~65 seconds
+### Clip 3
+- **Source segment:** Segment 5: Revenue or Wealth?
+- **Timestamp markers:** "I work with two surgeons..." through "...Completely different financial outcomes."
+- **Hook line:** "Surgeon A collects $1.4 million. Surgeon B collects $1.35 million. Surgeon B takes home $80,000 more per year."
+- **Core insight:** Two surgeons with nearly identical revenue have an $80K/year wealth gap driven entirely by structural differences: implant contracts, staffing efficiency, and S-Corp salary calibration.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~55 seconds
+---
+## COLD OPEN (30–60 seconds)
+The most common response to the CMS reimbursement cut? More surgery.
+And I get it. The math feels intuitive. Revenue went down, so you do more procedures to make it up. That's how it should work, right?
+But think about it this way. If a patient comes to you with a stress fracture, you don't tell them to walk faster. You look at the structure. You look at the biomechanics that created the problem. And then you design a plan that addresses the root cause, not just the symptom.
+The same logic applies here. When your reimbursement drops by 2.5%, the instinctive response is more volume. But that instinct is expensive. And today I want to walk you through exactly why, and what to do instead.
+---
+## INTRO AND CONTEXT (1–2 minutes)
+Here's the situation. Since January 1, 2026, CMS has applied a 2.5% "efficiency adjustment" to reimbursement rates on non-time-based orthopedic procedures. If you do total joints, rotator cuff repairs, ACL reconstructions, spine fusions, anything that's billed on a procedure-based code rather than a time-based evaluation and management code, you are getting paid less per case than you were in December.
+Now, your practice manager probably told you about this. Maybe your billing department flagged it. But here's the question I keep asking: did your financial advisor call you about it?
+Because this is not just a practice management issue. This is a wealth-building issue. The amount you're reimbursed per procedure affects your gross revenue, which affects your take-home income, which affects how much flows into your retirement plans, your investments, your family's financial future.
+And yet the conversation almost always stays inside the four walls of the practice. It stays in the domain of "how do we keep collections up?" when the real question is, "how do we make sure the money we do collect gets kept as efficiently as possible?"
+That's what this episode is about. We're going to look at the actual math on this reimbursement cut, walk through why the most common response (adding volume) is also the most expensive response, and I'll share three specific structural adjustments that can recover the lost revenue without requiring a single additional hour in the OR.
+---
+## SEGMENT 1: What the 2.5% Cut Actually Means (3–5 minutes)
+Let's start with the numbers, because I think a lot of surgeons have heard "2.5%" and filed it away as a minor annoyance. Two and a half percent doesn't sound like much. Let me show you what it actually looks like in practice.
+Take a surgeon performing 400 procedures a year. That's a reasonable case volume for a busy orthopedic practice. And let's say the average reimbursement across those cases is $3,200. That's a blended number across your mix of total joints, scopes, fracture fixations, whatever your case mix looks like.
+Before the adjustment, that surgeon's procedural revenue is 400 times $3,200, which is $1,280,000. After the 2.5% cut, each procedure now reimburses $3,120. That's $80 less per case. Doesn't sound like a lot, right? Eighty dollars?
+But multiply that by 400 cases and you get $32,000 in annual revenue that just disappeared. Not because you did anything differently. Not because you lost patients or skills or referrals. The payer simply decided to pay you less for the same work.
+And here's the part that makes this more than a rounding error. That $32,000 comes straight off the top. It's the highest-margin revenue you had, because you were already doing those cases. The OR was already booked. The staff was already there. The overhead was already covered. That $32,000 was the revenue that flowed most directly into your personal income.
+Now, I want to put this in context. If you're a surgeon earning $800,000 a year and you lose $32,000 in top-line revenue, the after-tax impact (assuming a combined federal and state rate around 40%) is about $19,000 in reduced take-home pay. Almost $20,000 less in your pocket, from a cut you probably didn't spend more than five minutes thinking about.
+And this is just year one. I'll talk in a few minutes about why this particular cut is the beginning of a trend, not a one-time adjustment.
+But before we get there, let's look at the response that most surgeons default to. Because understanding why that response is so expensive is the key to finding a better one.
+---
+## SEGMENT 2: The Volume Trap (3–5 minutes)
+So the natural instinct when revenue drops is to do more. More cases, more procedures, more time in the OR. And that instinct makes sense on the surface. If each procedure now pays $80 less, you just need 10 more procedures to make up the $32,000 gap. Ten cases. That's less than one extra case per month. Easy, right?
+Except it's not easy. And it's not cheap.
+Here's what the "just add volume" math actually looks like. When you're already running a full surgical schedule and you add procedures at the margin, those additional cases carry real incremental costs. You need OR time, which means either extending your block time or competing for open slots. You need anesthesia coverage for those additional hours. You need surgical supplies, implants, disposables. You need pre-op and post-op nursing time. You need the front desk to schedule, the billing team to process, and the clinical staff to handle follow-ups.
+When you add it all up, the marginal cost of an additional procedure in a practice that's already operating near capacity is typically around 55% to 65% of the procedure's revenue. Let's use 60% as our number.
+So those 10 additional procedures at $3,120 each generate $31,200 in gross revenue. But the marginal cost at 60% is $18,720. Which means the net recovery is only $12,480. You added 10 cases to your surgical schedule, put in the extra hours, took on the additional clinical risk, and you recovered $12,480 of a $32,000 gap.
+That's a 39% recovery rate. You did 100% more work to get back 39% of what you lost.
+Let me say that differently, because I think this is the number that matters. For every additional hour you spend in the OR trying to make up for the reimbursement cut, you're earning significantly less per hour than you were on your existing cases. You're diluting your effective hourly rate (something we're going to talk about in detail next week) by chasing volume that doesn't carry its own overhead.
+And there's a compounding problem here. If you're adding cases, you're also adding fatigue, surgical risk, administrative burden, and time away from everything else. Time away from your family. Time away from the strategic work on your practice. Time away from the financial planning that could actually solve this problem more efficiently.
+Let's walk through what this looks like for a surgeon considering adding a half-day of surgery every other week to offset the CMS cut. The incremental revenue from those sessions, after accounting for the additional overhead, would net roughly $14,000 a year. That surgeon would give up 26 half-days (that's 13 full days, or about two and a half weeks of life) for $14,000. That's roughly $1,077 per day. For a surgeon earning $800,000 a year, that's well below what the time is worth on any rational analysis.
+The volume response feels productive. It feels like taking action. But it's the most expensive way to solve this problem. And there are alternatives that cost nothing in terms of additional time.
+---
+## SEGMENT 3: Three Overhead Line Items You've Probably Never Benchmarked (3–5 minutes)
+So if adding volume is the expensive response, what's the efficient one? The answer lives inside your practice's overhead structure. And specifically, inside three line items that most orthopedic practices have never benchmarked against industry data.
+Let me walk through each one.
+**The first is supply costs, and specifically implant pricing.**
+Most orthopedic practices negotiate implant pricing once (usually when they first establish their vendor relationships) and then never revisit it. The rep relationship feels solid, the products work well, and renegotiating feels like a distraction from clinical work.
+But here's the reality. Implant pricing varies by 15% to 30% across vendors for functionally equivalent devices. If your practice is spending $400,000 a year on implants and supplies (which is common for a busy orthopedic group), a 10% reduction through competitive bidding or renegotiation saves you $40,000 annually. That's more than the entire $32,000 reimbursement gap, recovered without touching your surgical schedule.
+And I want to be specific about how to approach this. You don't have to switch vendors. Often, the conversation starts with a simple request: "We'd like to see competitive pricing for equivalent products." Your current vendors will frequently match or beat competing offers to retain your business. The leverage is there. Most practices just never use it.
+**The second line item is staffing ratios.**
+The Medical Group Management Association publishes benchmarks for clinical and administrative staffing ratios in orthopedic practices. The benchmark for a well-run orthopedic group is approximately 4.5 to 5.0 total staff per full-time-equivalent physician. Many practices are running at 5.5 to 6.5.
+Now, I'm not suggesting you fire people. But understanding where your staffing ratio sits relative to the benchmark tells you something important about operational efficiency. Are there roles that could be restructured? Are there tasks being done manually that could be systematized or automated? Is there duplication across front-office and back-office functions?
+If your total staff compensation is $1.2 million and your ratio is one full position above the benchmark, that's roughly $55,000 to $70,000 in excess staffing cost. Even a partial correction (say, through attrition and role consolidation) could recover $25,000 to $35,000 annually. Again, more than enough to offset the reimbursement cut.
+**The third is facility utilization.**
+This one is less obvious but potentially the most impactful for practices that own or lease their space. Most orthopedic practices use their clinic and surgical facilities during standard business hours, roughly 8 a.m. to 5 p.m., Monday through Friday. That's 45 hours out of a potential 168 hours per week, which is about 27% utilization.
+Now, I'm not suggesting you start doing midnight clinics. But there's a realistic middle ground. Could you sublease unused clinic space to a physical therapy group two days a week? Could your ASC (if you have one) accommodate cases from outside surgeons on your off days? Could your imaging equipment generate revenue from after-hours referrals?
+These are revenue additions, not cost cuts. And they use assets you're already paying for. A practice that generates even $50,000 a year from improved facility utilization has more than replaced the CMS cut, and they've done it by making their existing infrastructure work harder, not by working harder themselves.
+Let me add these up. Implant renegotiation: $40,000. Staffing optimization: $25,000 to $35,000. Facility utilization: $30,000 to $50,000. Even implementing just one of these at the conservative end of the range recovers the full $32,000 gap. Implementing all three could generate $95,000 to $125,000 in annual savings or new revenue.
+The point is this: the money is already inside your practice. It's sitting in line items that nobody has looked at strategically, because the revenue was always high enough that nobody had to.
+---
+## SEGMENT 4: The Multi-Year Headwind (3–5 minutes)
+Now, everything I've said so far would be valuable even if this year's 2.5% cut were a one-time event. But it's not. And this is the part of the conversation that I think most surgeons haven't had with anyone yet.
+In 2025, the One Big Beautiful Bill Act (you'll hear it called OBBBA) became law. And buried inside that bill, alongside the tax provisions and the spending measures, is a formula that determines how Medicare physician payments will be updated going forward.
+Here's how the formula works. Starting in 2026, Medicare payment updates for physicians are tied to 75% of the Medicare Economic Index, which is the MEI. The MEI measures the cost of running a medical practice: rent, staff wages, malpractice insurance, supplies, all the things that get more expensive every year. Historically, the MEI runs somewhere around 2% to 3% annually.
+But the payment update only gives you 75% of that. So if practice costs go up 3%, your reimbursement goes up 2.25%. Every year, you fall a little further behind. Year after year after year.
+Let me put real numbers on this. If the MEI averages 2.5% over the next five years, your practice costs rise by a cumulative 13.1%. But your Medicare payments only rise by 9.8%. That's a 3.3 percentage point gap over five years. On a $1.3 million revenue base, that gap represents roughly $43,000 in purchasing power that has quietly evaporated.
+And that's on top of the 2.5% efficiency adjustment we've already talked about. These are additive pressures. The reimbursement is being compressed from two directions: an immediate cut and a structural formula that ensures you never quite keep up with rising costs.
+This is why I keep saying that the response has to be structural, not tactical. You can't outrun a compounding headwind with incremental volume. You have to look at the way your practice generates and retains income and redesign the system to be more efficient.
+Think of it this way. If you're a runner and the wind picks up, you have two choices. You can try to run faster (which burns more energy and eventually exhausts you), or you can change your form, lean into it, become more aerodynamic. The structural response is the financial equivalent of improving your form. It doesn't require more effort. It requires different effort.
+And for surgeons in the 45 to 65 age range, this matters on a very personal level. If you're 50 years old and planning to practice for another 10 to 15 years, this reimbursement headwind will be present for the remainder of your career. The decisions you make now about practice structure, overhead management, and income flow will compound across every remaining year. A 2% overhead reduction in year one doesn't just save you $26,000 this year. It saves you $26,000 every year for the next 12 years, which is over $310,000 in cumulative savings. And that's before you factor in what that money could have earned if it had been invested.
+---
+## SEGMENT 5: Revenue or Wealth? The Strategic Question (3–5 minutes)
+I want to step back for a moment and ask a question that ties everything in this episode together. Because the reimbursement cut, the volume trap, the overhead blind spots, the multi-year headwind, they all point to the same fundamental issue.
+Is your practice structured to build wealth, or is it structured to generate revenue?
+Those sound like the same thing, and for a long time in medicine, they were close enough. Revenue was high, overhead was manageable, and the gap between what the practice collected and what the surgeon kept was wide enough that structural inefficiency didn't matter much. You could have a bloated staff ratio, overpay for implants, leave your facility half-empty, and still take home $700,000 or $800,000 a year.
+But that margin is compressing. The reimbursement environment is getting tighter. Practice costs are rising faster than payments. And the gap between revenue and personal wealth is widening for surgeons who haven't updated their structure.
+Here's a way to think about this. Consider two surgeons with almost identical practices. Similar case volumes, similar specialties, similar geographic markets. Surgeon A collects $1.4 million in gross revenue. Surgeon B collects $1.35 million. So Surgeon A actually has higher revenue.
+But Surgeon B takes home $80,000 more per year. How? Three things. Surgeon B renegotiated implant contracts two years ago and saves about $35,000 annually. Surgeon B runs one fewer FTE than Surgeon A for the same patient volume, saving another $60,000. And Surgeon B's S-Corp salary is calibrated to maximize retirement plan contributions (which we talked about last week), adding another $25,000 in tax-deferred value.
+Surgeon A generates more revenue. Surgeon B builds more wealth. And over a decade, at $80,000 per year in structural advantage, plus the compounding on the tax-deferred savings, the gap between them will be somewhere north of a million dollars. Same specialty. Same market. Same training. Completely different financial outcomes.
+The reimbursement cut is a clarifying event. It forces a question that was always there but easy to ignore when revenue was plentiful: where is the money going between the point where the practice collects it and the point where it reaches your personal balance sheet?
+If you've never traced that flow, now is the time. Not because the sky is falling (it's not), but because the environment has shifted enough that the structural inefficiencies you could afford to ignore last year are now costing you real money.
+And the beautiful thing about structural improvements is that they don't require more time. They don't require more energy. They require a different kind of attention. The same kind of attention you already bring to surgical planning: deliberate, precise, informed by data, and focused on outcomes.
+---
+## LISTENER TAKEAWAY (1–2 minutes)
+Alright, let me bring this together with something concrete. If you take one action from this episode, here's what I'd recommend.
+This week, sit down with your practice financials (or ask your practice administrator to pull the numbers) and look at three things.
+First, calculate your per-procedure reimbursement trend. Pull the average reimbursement per case for Q1 2026 and compare it to Q1 2025. Quantify the actual dollar decline, not just the percentage. I want you to see the number.
+Second, look at your implant and supply spend as a percentage of revenue. If you don't know what it is, that itself is a finding. The MGMA benchmark for orthopedic supply costs is 8% to 12% of net revenue. If you're above 12%, there's almost certainly room to renegotiate.
+Third, count your staff-per-physician ratio. Total staff headcount divided by full-time-equivalent physicians. If you're above 5.0, you're likely carrying overhead that could be restructured over time through natural attrition and role consolidation.
+You can do all three of these in less than an hour. And what you'll have at the end is a diagnostic snapshot, a baseline that tells you where the structural opportunities are in your practice. You won't have solved anything yet, but you'll know where to look. And knowing where to look is how every good treatment plan starts.
+If you want to take it a step further, bring those three numbers to your next conversation with your financial advisor. If your advisor doesn't know what to do with them, or if you've never had a conversation about practice overhead as a wealth-building lever, that tells you something too.
+---
+## PHILOSOPHICAL CLOSE (1–2 minutes)
+I want to leave you with something that's been on my mind throughout this episode.
+You wouldn't treat every patient with the same implant regardless of the pathology. You wouldn't scope every knee and fuse every spine. You assess the individual case, you consider the options, and you choose the approach that fits the specific problem.
+Your financial life deserves that same precision.
+When revenue drops, the reflexive response is to work more. More hours, more procedures, more volume. And sometimes that's the right answer. But sometimes, the most productive thing you can do is stop, look at the structure, and ask whether the system itself is working as efficiently as it should.
+The surgeons who build the most wealth over the course of a career aren't necessarily the ones who operate the most. They're the ones who pay attention to the entire system: the revenue, the overhead, the entity structure, the tax strategy, the retirement plan design. They treat their financial life with the same rigor they bring to clinical practice.
+And I think that's the real lesson of the reimbursement cut. It's a signal. A diagnostic finding. And like any finding, it points you toward a treatment plan. The question is whether you'll address the underlying condition, or just try to outrun the symptoms.
+Thanks for spending this time with me today. Talk to you next week.</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The 2.5% number is the post's anchor data point and creates immediate recognition for any surgeon who has seen it in their Q1 statements. A bold stat card makes the number impossible to scroll past.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "2.5%" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper third of the canvas. Secondary text: "Your practice manager told you." in Inter Regular, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 32px below the primary text. Tertiary text: "Your financial advisor probably didn't." in Inter SemiBold, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 16px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: urgent, authoritative, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "2.5%" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), upper third center. "Your practice manager told you." in Inter Regular, ~22pt, Off-White (#F6F7F5), below primary. "Your financial advisor probably didn't." in Inter SemiBold, ~22pt, Off-White (#F6F7F5), below secondary.
-Platform and dimensions: LinkedIn, 1080x1080</t>
+Image type: Podcast cover art / YouTube thumbnail
+Rationale: The image must communicate the concept of declining per-procedure revenue and structural response. A clean, data-informed visual with a downward-trending line paired with authoritative text creates both urgency and credibility. The design should feel analytical and strategic, matching the episode's math-driven argument. Avoiding any imagery that could feel alarmist or clickbait is essential for the surgeon audience.
+AI image prompt: Create a 1400x1400px square podcast cover art image. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: text-dominant composition with content centered vertically and left-aligned with 100px left margin. Primary text: "Less Per Procedure" in Playfair Display SemiBold, approximately 100pt, Off-White (#F6F7F5), left-aligned, positioned in the upper-center area of the canvas. Secondary text: "What to Do About It" in Inter Regular, approximately 48pt, Warm Gray (#9AA3A8), positioned directly below primary text with 20px spacing, same left alignment. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 60% of the canvas width beneath the secondary text, starting from the left margin. Below the accent line, a subtle downward-angled line graph rendered in Antique Gold (#B08D57) at 50% opacity, suggesting a gradual decline over 5 data points, with no axis labels or grid lines, purely atmospheric. Bottom of canvas: "CAPABLE WEALTH" in Inter Medium, 24pt, Blue Slate (#5F7483), centered horizontally, 60px from bottom edge. No cartoons, no clip art, no stock photography, no illustrations of people, no medical imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No generic stock, no clickbait styling, no busy compositions. Mood: analytical, calm, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Less Per Procedure" in Playfair Display SemiBold, ~100pt, Off-White (#F6F7F5), upper-center left-aligned. "What to Do About It" in Inter Regular, ~48pt, Warm Gray (#9AA3A8), below primary text. "CAPABLE WEALTH" in Inter Medium, 24pt, Blue Slate (#5F7483), centered at bottom.
+Platform and dimensions: Podcast cover 1400x1400, YouTube thumbnail variant 1280x720 (text repositioned to center-left two-thirds, right third left open for subtle atmospheric texture)</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>week-3-linkedin-1.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="120" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Week 3 (March 9–15)</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Adding 10 Procedures to Offset a $32K Loss Sounds Logical. Here's Why It Costs You More Than It Recovers.</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Reimbursement Shift and Practice Wealth</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Builds on Post 1 by challenging the instinctive "do more procedures" response to reimbursement cuts. Uses marginal cost math to show that volume increases are the most expensive way to recover lost revenue, and introduces structural optimization as the more efficient alternative.</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Adding 10 procedures to offset a $32K revenue loss sounds logical. Here's why it costs you more than it recovers.
-The CMS 2.5% efficiency adjustment reduced your average reimbursement by about $80 per procedure. At 400 procedures a year, that's $32,000 in lost revenue.
-The instinctive response: add 10 cases at $3,200 each to close the gap.
-But each additional procedure carries marginal costs that your existing caseload has already absorbed. OR time, anesthesia, supplies, implants, staff hours. At the margin, those costs consume roughly 60% of the revenue from each extra case.
-Here's how it actually plays out:
-→ 10 additional procedures: $32,000 gross revenue
-→ Marginal costs at 60%: $19,200
-→ Net recovery: $12,800
-→ Additional OR time: 30 to 40 hours
-You just spent a month's worth of extra surgical hours to recover 40 cents on every dollar you lost.
-Now compare that to structural optimization. A 2% reduction in practice overhead (on a $1.6M practice) saves $32,000 directly. No additional procedures. No additional OR time. No additional marginal costs. Dollar-for-dollar recovery.
-Working harder recovers 40 cents on the dollar. Reducing overhead by 2% recovers 100 cents.
-At surgeon-level income, your time is the most expensive input you have. Before adding cases to the schedule, it's worth asking: is there a way to recover this revenue without spending more of it?</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
+          <t>week-3-podcast-less-per-procedure.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 4 (MARCH 16–22)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="200" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Before Q1 Closes: The One Number That Matters More Than Collections</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>The number that matters more than collections</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Video Podcast Script (uploaded to YouTube; audio distributed to podcast platforms)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>This is the capstone episode of the March arc. Weeks 1 through 3 diagnosed structural gaps (entity structure, S-Corp salary calibration, reimbursement cuts and overhead optimization). This episode synthesizes all three into a single metric, the effective hourly rate, that reveals what a surgeon actually keeps for each hour of clinical work. The timing is deliberate: Q1 is about to close, making this the ideal moment to equip surgeons with the framework so they can run the calculation as soon as the data is available. The episode closes the "diagnosis" phase of the quarterly content plan and sets up April's "interpretation" phase.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>## Clip Extraction Map
+### Clip 1
+- **Source segment:** Segment 3: Running the Calculation
+- **Timestamp markers:** "$480,000 divided by 2,600 hours equals $185 per hour." through "...That gap has consequences."
+- **Hook line:** "Your practice collected $2.4M last year. You kept $480K. Your effective hourly rate? $185."
+- **Core insight:** The effective hourly rate reveals the massive gap between perceived earnings and actual take-home. $185/hour for a surgeon collecting $2.4M exposes the structural leakage.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~50 seconds
+### Clip 2
+- **Source segment:** Segment 4: Structural Improvement Model
+- **Timestamp markers:** "$215 versus $185. That's $30 per hour more." through "...The only thing that changed is the structure."
+- **Hook line:** "A $30/hour difference doesn't sound like much. Over 2,600 clinical hours, it's $78,000 a year."
+- **Core insight:** Structural improvements (overhead reduction, entity optimization, cash balance plan) move the effective hourly rate from $185 to $215, worth $78K/year and over $1M over a decade.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~55 seconds
+### Clip 3
+- **Source segment:** Listener Takeaway
+- **Timestamp markers:** "Step one: Take your Q1 collections..." through "...It takes fifteen minutes."
+- **Hook line:** "Here's how to calculate your real hourly rate in 15 minutes. Five steps. One number that changes everything."
+- **Core insight:** A step-by-step walkthrough of the effective hourly rate calculation: collections, minus overhead, minus taxes, minus retirement, minus debt, divided by clinical hours.
+- **Platform tags:** [IG-REEL]
+- **Estimated duration:** ~75 seconds
+### Clip 4
+- **Source segment:** Segment 1: Why Collections Is a Vanity Metric
+- **Timestamp markers:** "Two surgeons, both collecting $2.4 million a year..." through "...Collections doesn't touch any of them."
+- **Hook line:** "Two surgeons. Same collections. $80,000 difference in what they keep. How?"
+- **Core insight:** Collections measures practice health, not surgeon wealth. The $80K gap between two identical-revenue surgeons sits in overhead, entity design, and tax strategy.
+- **Platform tags:** [YT-SHORT]
+- **Estimated duration:** ~45 seconds
+---
+## COLD OPEN (30–60 seconds)
+Most surgeons can tell you their practice's gross collections within $50K. Almost none of them can tell you their effective hourly rate.
+That's the actual dollar amount you earn for each hour spent in clinical work, after taxes, overhead, debt, and savings. The number that's left when everything else has been taken.
+And that gap, between what you think you make and what you actually keep, is where wealth disappears.
+Today I'm going to walk you through exactly how to calculate that number. We're going to use real math at surgeon-level income, and I think some of what we find is going to surprise you. We'll also talk about the three levers that can move the number by $30 an hour or more, which at full-time clinical hours translates to $78,000 a year.
+If you've been following along this month, we've covered entity structure, S-Corp salary optimization, and the reimbursement landscape. This episode ties all of it together into one metric. One number. The number I think matters more than collections.
+Let's get into it.
+---
+## INTRO AND CONTEXT (1–2 minutes)
+So here's why I wanted to do this episode right now, in mid-March.
+Q1 closes at the end of this month. In about two weeks, if you're running a practice, you'll have three months of revenue data, expense data, and clinical hours logged. You'll have enough information to run a real calculation, not a hypothetical, not a projection. An actual number based on actual data from the first quarter of this year. I want you to have the framework in hand before that data arrives.
+And here's a pattern that shows up frequently in surgeon-owned practices. Almost every surgeon can tell you what their practice collected last quarter. That number lives in their head. It comes up in partner meetings, in conversations with the practice manager, sometimes even over dinner with colleagues.
+But ask, "What did you actually take home per hour of clinical work after everything?" and the answer is usually silence. Or a rough guess that's almost always too high.
+Collections is a practice metric. It tells you how the business is doing. That's valuable, obviously. But it doesn't tell you how the surgeon is doing. It doesn't tell you whether your time, your most finite resource, is being compensated in a way that reflects the skill you bring, the training you invested, and the life you're trying to build.
+The effective hourly rate answers that question. And for most surgeons, the answer is uncomfortable the first time they see it.
+I'm not saying that to be dramatic. I'm saying it because this is a structural pattern that shows up frequently in surgeon-owned practices. When a surgeon runs this calculation for the first time, the reaction is predictable. There's a pause. There's a recalculation. And then there's a very productive conversation about what to do about it.
+That's what this episode is for.
+---
+## SEGMENT 1: Why Collections Is a Vanity Metric for the Surgeon (3–5 minutes)
+Let me be clear about what I mean when I say collections is a vanity metric. I'm not saying it doesn't matter. I'm saying it measures the wrong thing if what you're trying to understand is your personal financial health.
+Collections tells you how much revenue the practice generated. That's important for the entity. It's important for your practice manager, your lender, your partners if you have them. But it tells you almost nothing about what you, as the surgeon, actually kept.
+Think about it this way. Two surgeons, both collecting $2.4 million a year. Same specialty, similar case volume. One takes home $480K. The other takes home $560K. Same collections, $80,000 difference in what they keep.
+How? The difference sits in everything that happens between the top line and the bottom line. Overhead structure, entity design, tax strategy, retirement plan contributions, debt load. Those are the variables that determine your real compensation. Collections doesn't touch any of them.
+And here's what makes this tricky: collections is the number that gets talked about. In partner meetings, in benchmarking surveys, at conferences, at dinner. Nobody asks, "What's your effective hourly rate?" They ask, "What did you collect?" or "What's your comp?" And "comp" usually means the number before taxes, which is a very different thing from the number after taxes.
+So surgeons end up anchoring on a number that flatters them. $800K in compensation sounds fantastic. And it is. But $800K before a 40% effective tax rate, before retirement contributions, before debt service on practice loans? That's a very different picture.
+Consider a surgeon who feels like he should have more to show for fifteen years of practice at his income level. When you run the numbers for someone in this position, the feeling is often justified. The practice is collecting well. Compensation looks strong. But the effective hourly rate, what the surgeon is actually keeping for each hour of clinical work, can be lower than expected by $100 an hour or more.
+That's the gap. And you can't see it if you're only looking at collections.
+The first step is simply acknowledging that collections and compensation and take-home and effective hourly rate are four different numbers. They're related, but they measure different things. And the one that matters most for your personal wealth trajectory is the last one.
+---
+## SEGMENT 2: The Five Components of Your Effective Hourly Rate (4–5 minutes)
+So let's build this number from the ground up. There are five components that determine your effective hourly rate, and I want to walk through each one, because understanding the components is what tells you which levers you can actually pull.
+Component one: gross revenue. This is the starting point. For the math we'll use today, I'm going to use $2.4 million in annual practice collections. That's a realistic number for an orthopedic surgeon with a mature, busy practice. If your number is higher or lower, the ratios and percentages still apply. The absolute dollars will shift, but the structure of the calculation doesn't change.
+Component two: overhead. This is everything the practice spends before the surgeon gets paid. Staff salaries, rent, supplies, insurance, billing, equipment leases, all of it. For orthopedic practices, overhead typically runs between 50% and 60% of collections. The national average for surgical specialties hovers around 55%. We'll use 55% for our baseline, which on $2.4 million in collections means $1.32 million in overhead, leaving $1.08 million as the surgeon's gross income.
+Now, I want to pause here because this is where Week 3's conversation becomes relevant. We spent that entire episode talking about the CMS reimbursement cut and why the instinctive response (doing more procedures) is more expensive than the structural response (optimizing overhead). If your overhead is running at 55% and you can bring it to 52%, that's $72,000 in additional income on $2.4 million in collections. Without doing a single additional case. That overhead number matters enormously in this calculation.
+Component three: taxes. At $1.08 million in surgeon income, the effective tax rate, combining federal, state, and the net investment income tax, typically lands around 38% to 42% depending on your state and your deduction profile. I'll use 40% for our example, which means $432,000 goes to taxes. That brings us from $1.08 million down to $648,000 after tax.
+And this is where Week 1's entity structure conversation comes back. Your entity structure, your S-Corp election, your salary calibration, your QBI deduction, all of those directly affect this tax number. A surgeon with an optimized structure might have an effective rate closer to 37% or 38%. A surgeon with an unoptimized structure might be closer to 42% or 43%. At this income level, each percentage point is roughly $10,800. So the difference between a well-structured and a poorly-structured entity can be $30,000 to $50,000 a year, right here in this one component.
+Component four: retirement contributions. This includes 401(k) contributions, any cash balance plan funding, and employer matches. For our baseline surgeon, let's say $72,000, which would be a 401(k) with catch-up contributions plus a modest employer match. That brings us from $648,000 down to $576,000.
+Now, retirement contributions are interesting because they reduce your take-home today, but they're building your wealth for tomorrow. They're not "lost" money. They're redirected money. But they do reduce what lands in your checking account this year, and that matters for this calculation.
+Component five: debt service. Practice loans, equipment financing, building mortgage if you own the facility. For a surgeon with a practice loan and some equipment financing, $96,000 a year in debt service payments is common. That brings us from $576,000 down to $480,000.
+So the waterfall looks like this: $2.4 million in collections, minus $1.32 million in overhead, minus $432,000 in taxes, minus $72,000 in retirement contributions, minus $96,000 in debt service. What's left is $480,000.
+That's what the surgeon keeps. Out of $2.4 million.
+---
+## SEGMENT 3: Running the Calculation, and What the Number Reveals (4–5 minutes)
+Now we divide.
+$480,000 in take-home, divided by the number of hours you spend in clinical work. And this is the part where I need you to be honest with yourself about the denominator.
+Clinical hours means time in the OR, time in clinic, time rounding, time on call that actually produces patient care. For most full-time orthopedic surgeons, that number falls between 2,200 and 2,800 hours per year. Some of you work more. A few of you work less. But the range is consistent.
+For our example, I'll use 2,600 hours. That's roughly 50 hours a week of clinical activity across 52 weeks with a couple of weeks off.
+$480,000 divided by 2,600 hours equals $185 per hour.
+Let that sit for a moment.
+$185 per hour. For a surgeon who trained for over a decade. Who carries the liability of surgical outcomes. Who runs a practice collecting $2.4 million a year.
+Now, I want to be careful here. $185 an hour is not a small number in the broader economy. I'm not trying to suggest that surgeons are underpaid in some absolute sense. What I am saying is that the gap between what a surgeon thinks they earn per hour and what they actually keep per hour is almost always larger than they expect. And that gap has consequences.
+Because here's what happens when you know your effective hourly rate. Every financial decision starts to have a time cost attached to it. That $96,000 in debt service? That's 519 hours of your clinical time. More than ten weeks of work, just servicing debt. The overhead difference between 55% and 52%? That's 389 hours of your time being consumed by structural inefficiency.
+Suddenly, the abstract concepts we've been discussing all month, entity structure, S-Corp salary, overhead optimization, they aren't abstract anymore. They have a direct connection to the hours of your life.
+And remember that Jose Mujica quote I come back to all the time: "We're not paying with money. We're paying with the time from our lives we had to spend to earn that money." Your effective hourly rate makes that real. It converts every dollar of waste, every structural gap, into hours of clinical work that you're doing for free, essentially.
+So here's the question I want you to ask yourself. When Q1 closes and you have the data in front of you, what will this number be?
+You'll have the information. You'll know your Q1 collections. You can estimate your overhead percentage. You know your tax situation, or close enough. You know your retirement contributions and your debt service payments. And you know how many hours you spent in clinical work.
+Run the number. It takes fifteen minutes.
+When Q1 closes, annualize your data (multiply by four if your Q1 is representative, or adjust for seasonality if it's not). Walk through the five components. Do the division.
+And then write the number down. Because you're going to want to compare it to what it could be.
+---
+## SEGMENT 4: What the Number Could Be, the Structural Improvement Model (4–5 minutes)
+So we've established the baseline: $2.4 million in collections, $480,000 take-home, $185 per hour. Now let's model what happens when you apply the structural improvements we've discussed over the last three weeks.
+Lever one: overhead optimization. This is the Week 3 lever. If the surgeon reduces overhead from 55% to 52%, that changes the overhead number from $1.32 million to $1.248 million. That's $72,000 more flowing to the surgeon. And remember, we showed in Week 3 that a 2-3% overhead reduction is realistic for most practices. It doesn't require firing staff or cutting quality. It usually comes from renegotiating supply contracts, auditing vendor relationships, and improving facility utilization. Three things most practices have never systematically benchmarked.
+Lever two: entity and tax structure optimization. This is the Week 1 and Week 2 lever combined. Optimizing your S-Corp salary calibration (getting the balance right between payroll tax, retirement plan capacity, and the QBI deduction), adding a cash balance plan, and ensuring your entity structure supports wealth accumulation rather than just compliance. In our model, this brings the effective tax rate from 40% down to 37.5%, and it increases retirement plan contributions from $72,000 to $135,000 (because the cash balance plan unlocks an additional $63,000 in annual tax-deferred contributions).
+Now, you might look at that and think, "Wait, higher retirement contributions reduce my take-home." And they do, in the near term. But they reduce your taxes more than they reduce your take-home, because every dollar going into the cash balance plan is pre-tax. So the net effect on your after-everything take-home is positive. You're sheltering more, paying less tax, and building more wealth, even though the contribution number went up.
+Let me run the waterfall with these adjustments.
+$2.4 million in collections. Overhead at 52%: $1.248 million. Surgeon gross income: $1.152 million. Taxes at 37.5% effective rate: $432,000. (Notice, the tax bill is the same dollar amount, even though the income is higher, because the rate dropped from 40% to 37.5%. That's the structure working.) Retirement contributions at $135,000, including the cash balance plan. Debt service still at $96,000.
+Take-home: $1.152 million minus $432,000 minus $135,000 minus $96,000 equals $489,000.
+Hmm. $489,000 versus $480,000. Only $9,000 more in take-home? That doesn't seem like much.
+But here's where the full picture matters. You're now sheltering $135,000 a year in retirement accounts instead of $72,000. That additional $63,000 in tax-deferred contributions is growing at, let's say conservatively, 6% per year. Over ten years, that single change produces over $830,000 in additional retirement wealth. And you funded it largely with tax savings, not out of pocket.
+When you factor retirement wealth accumulation into total compensation (which you should, because that money is yours, just deferred), the picture changes dramatically. Your total annual compensation, take-home plus retirement contributions, goes from $552,000 ($480K + $72K) to $624,000 ($489K + $135K). That's $72,000 more in total wealth creation per year.
+And your effective hourly rate on total compensation? $624,000 divided by 2,600 hours equals $240 per hour, up from $212 ($552K divided by 2,600).
+But even if we just look at liquid take-home and model the more aggressive overhead reduction scenario (let's say you get overhead to 51% through disciplined cost management and the structural tax rate to 37%), the waterfall produces about $560,000 in take-home. Divide that by 2,600 hours, and you get $215 per hour.
+$215 versus $185. That's $30 per hour more. Across 2,600 clinical hours, that's $78,000 per year. In additional take-home. From structural changes, not from doing more surgery, not from working harder, not from seeing more patients. From fixing the plumbing.
+$78,000 a year. Over a ten-year career horizon, with modest investment returns, that's over a million dollars in additional wealth. From the same collections, the same clinical hours, the same practice. The only thing that changed is the structure between the top line and the bottom line.
+That's why I keep saying: the structure is the strategy.
+---
+## SEGMENT 5: The Three Levers and the March Arc (3–4 minutes)
+So let me pull the camera back and connect the dots across the entire month.
+We've spent four weeks building a case for something specific. The amount you collect is less important than the amount you keep, and the amount you keep is determined by three structural levers.
+Lever one is your entity and tax structure. That was Week 1. We talked about the three structural gaps that cost the most: the S-Corp salary misalignment, the missing cash balance plan, and the absent cost segregation study. The combined annual cost of those three gaps, at surgeon-level income, ranges from $85,000 to $130,000 per year.
+Lever two is your salary calibration. That was Week 2. We walked through the three-variable balancing act of payroll tax, retirement plan contributions, and the QBI deduction. The insight was that your S-Corp salary isn't one number serving one purpose. It's one number that interacts with three different optimization targets, and getting it wrong in either direction costs real money.
+Lever three is your overhead and practice economics. That was Week 3. The CMS reimbursement cut was the catalyst, but the real lesson was broader: when revenue per procedure declines, the instinctive response (more volume) is the most expensive response. Optimizing overhead by 2-3% recovers more revenue than adding ten procedures, with none of the marginal cost.
+Today, in Week 4, we've taken those three levers and fed them into a single output metric. The effective hourly rate. One number that tells you whether those three levers are working for you or against you.
+And what I hope you take away from this month is that these aren't three separate conversations. They're three parts of the same conversation. Your entity structure determines your tax rate. Your tax rate determines your take-home. Your overhead determines how much revenue reaches you in the first place. And your effective hourly rate captures all of it in a single, honest number.
+When a surgeon calculates this rate for the first time, it changes the nature of every financial conversation that follows. Because now, every structural improvement has a unit of measurement: hours of your life.
+Reduce overhead by 2%? That's 389 hours of clinical work you just freed up, or $72,000 more in your pocket, however you want to think about it. Optimize your S-Corp salary and add a cash balance plan? That's another 280 hours of value. Accelerate depreciation through a cost segregation study? Another 80 to 160 hours.
+Those aren't abstract improvements. Those are days and weeks and months of your life that you're either capturing or losing, depending on whether the structure is right.
+---
+## LISTENER TAKEAWAY (1–2 minutes)
+Here's what I want you to do this week. One thing. Fifteen minutes.
+Calculate your effective hourly rate as soon as Q1 closes at month-end.
+Step one: Take your Q1 collections and annualize them. If Q1 was $600,000, your annualized collections estimate is $2.4 million.
+Step two: Subtract your overhead. If you don't know your exact overhead percentage, ask your practice manager. If you can't get it this week, use 55% as a starting estimate for an orthopedic practice. You can refine later.
+Step three: From the surgeon income that remains, subtract your effective tax rate. If you don't know your exact effective rate, use 40%. Again, refine later.
+Step four: Subtract your annual retirement contributions and your annual debt service.
+Step five: Divide what's left by your annual clinical hours. If you're not sure, use 2,400 to 2,600 as a reasonable range for full-time clinical practice.
+Write the number down.
+Then ask yourself two questions.
+First: is this number higher or lower than what I assumed?
+Second: which of the three levers (entity structure, salary calibration, overhead optimization) is most likely dragging this number down?
+You don't have to fix everything today. You just have to know the number. Because you can't improve what you haven't measured. And for most surgeons, this is the one measurement that's never been taken.
+If the number surprises you, and for most people it does, that's not a problem. That's a diagnosis. And like any good diagnosis, it points directly to the treatment plan.
+---
+## PHILOSOPHICAL CLOSE (1–2 minutes)
+You measure outcomes in the OR because you know that what gets measured gets improved. Every procedure has metrics. Every patient has benchmarks. You track range of motion, infection rates, revision rates, patient-reported outcomes. You do this because you understand, at a fundamental level, that precision and measurement are what separate good outcomes from mediocre ones.
+The same principle applies to your finances.
+If you've never calculated your effective hourly rate, the real measure of what your time is worth, this is the week to do it. Not because the number will be comfortable, but because it will be true.
+And there's something powerful about knowing the true number. Because once you know it, you stop guessing. You stop assuming. You stop anchoring on collections or compensation or whatever number happens to get mentioned at the partner meeting. You have a number that is yours, that reflects your specific structure, your specific overhead, your specific tax situation, and your specific hours.
+From that number, every decision gets clearer. Is the structure right? Is the overhead where it should be? Are you sheltering enough? Are you working the right number of hours, or are you trading time for money at a rate that doesn't reflect the value you bring?
+These are not comfortable questions. But they're the right questions. And they start with one number.
+You've spent this whole month learning about the levers. The entity structure that determines your tax rate. The salary calibration that unlocks your retirement contributions. The overhead optimization that recovers revenue without adding cases. Now you have the tool to see whether those levers are working.
+Run the calculation. Know the number. And if it's not where you want it to be, that's not a failure. That's the beginning of a very productive conversation.
+Capably yours.</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The 40-cents-on-the-dollar recovery figure is the post's most memorable data point. Isolating it as a stat card creates a scannable, shareable visual that captures the core argument without requiring the reader to process the full math.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "40¢" in Playfair Display SemiBold, approximately 108pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "recovered per dollar lost" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "when you add procedures to offset a cut" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: precise, authoritative, thought-provoking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "40¢" in Playfair Display SemiBold, ~108pt, Antique Gold (#B08D57), center. "recovered per dollar lost" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "when you add procedures to offset a cut" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below secondary.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>week-3-linkedin-2.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="120" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Week 3 (March 9–15)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>OBBBA Tied Medicare Physician Payments to 75% of the MEI. Here's What That Number Means in Your Pocket.</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Reimbursement Shift and Practice Wealth</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Zooms out from the immediate 2.5% cut to the broader legislative context. The One Big Beautiful Bill Act (OBBBA) pegged Medicare physician payment updates to 75% of the Medicare Economic Index, creating a permanent structural gap between rising practice costs and reimbursement growth. This post frames the shift as long-term and structural, requiring a financial response beyond single-year adjustments.</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>OBBBA tied Medicare physician payments to 75% of the Medicare Economic Index in 2026. Here's what that number means in your pocket.
-The Medicare Economic Index tracks how much it actually costs to run a medical practice: staff wages, rent, malpractice, supplies, everything. When those costs go up 4%, the MEI reflects that increase.
-Before OBBBA, physician payment updates were set year by year through temporary legislative patches, usually at or near 0%. The new law replaced that system with an automatic annual update tied to 75% of the MEI.
-On the surface, that sounds like progress. And compared to a decade of flat or negative updates, it is.
-But 75% is a permanent structural gap. If your practice costs rise 4%, your Medicare reimbursement rises 3%. Every year, the difference compounds. Over five years, that gap between costs and reimbursement becomes meaningful. Over ten years, it reshapes practice economics.
-For a surgeon collecting $1.6M annually with 40% of revenue from Medicare, even a 1% annual gap means roughly $6,400 in lost ground per year. That's not dramatic in year one. By year five, the cumulative shortfall is over $30,000. By year ten, it's approaching $70,000.
-This is the important part: a structural shift requires a structural response. Adjusting your surgical schedule year by year won't close a gap that's built into the payment formula itself.
-What will close it: reducing overhead systematically, optimizing how your income flows from the practice to your personal wealth, and building a financial structure that doesn't depend on reimbursement growth to function.
-The payment formula changed. Has your financial plan?</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
+Image type: Podcast cover art / YouTube thumbnail
+Rationale: The thumbnail must communicate the "one number" concept with visual clarity at both podcast cover and YouTube thumbnail scale. A bold numerical contrast (the collections number versus the effective hourly rate) creates immediate curiosity. The design uses the financial advisory aesthetic that resonates with orthopedic surgeons 45-65: clean, authoritative, zero clickbait energy.
+AI image prompt: Create a 1400x1400px square podcast cover art image. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: text-dominant composition, vertically centered. Primary text: "$185/hr" in Playfair Display SemiBold, approximately 140pt, Antique Gold (#B08D57), horizontally centered. Secondary text: "Your Real Rate" in Inter Medium, approximately 48pt, Off-White (#F6F7F5), centered directly below the primary text with 20px spacing. Tertiary text: "CAPABLE WEALTH" in Inter SemiBold, approximately 24pt, Warm Gray (#9AA3A8), letterspaced at 200%, positioned near the bottom of the canvas with 80px bottom margin, horizontally centered. A thin horizontal rule (2px, Antique Gold #B08D57, 40% canvas width) separates the primary and secondary text, centered horizontally. Subtle background texture: a very faint grid of thin lines in Blue Slate (#5F7483) at 8-10% opacity, suggesting a spreadsheet or calculation aesthetic without being literal. No cartoons, no clip art, no illustrations, no people, no stock photography. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: precise, revelatory, grounded. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$185/hr" in Playfair Display SemiBold, ~140pt, Antique Gold (#B08D57), centered. "Your Real Rate" in Inter Medium, ~48pt, Off-White (#F6F7F5), below primary text. "CAPABLE WEALTH" in Inter SemiBold, ~24pt, Warm Gray (#9AA3A8), letterspaced, near bottom.
+Platform and dimensions: Podcast cover 1400x1400, YouTube thumbnail variant 1280x720</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>week-4-podcast-one-number.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 5 (MARCH 23–29)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+    </row>
+    <row r="9" ht="200" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>How to Read Your Tax Return Like a Surgeon Reads an MRI</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Video Podcast Script (uploaded to YouTube; audio distributed to podcast platforms)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Companion piece to the Week 5 anchor blog. While the blog presents the four diagnostic markers as a framework, this podcast walks through them conversationally, with extended examples and more personal reflection. Builds on four weeks of structural diagnosis (entity, salary, reimbursement, hourly rate) by showing surgeons how their tax return confirms or reveals each gap. The MRI metaphor bridges clinical expertise to financial literacy.</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>## Clip Extraction Map
+### Clip 1
+- **Source segment:** Segment 4: Finding Three, the Retirement Contribution Gap
+- **Timestamp markers:** "So let's do the math on Dr. K..." through "...nearly $2 million in retirement wealth."
+- **Hook line:** "A surgeon contributed $31,000 to retirement last year. The available capacity was $203,000. That $172,000 gap compounds every single year."
+- **Core insight:** The retirement contribution gap ($31K contributed vs. $203K available) represents the single largest missed opportunity on most surgeon returns. Over 10 years, the difference is nearly $2M in retirement wealth.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~55 seconds
+### Clip 2
+- **Source segment:** Segment 2: Finding One, the Effective Tax Rate
+- **Timestamp markers:** "So what does 'normal' look like?" through "...it compounds to something considerably north of half a million dollars."
+- **Hook line:** "Your effective tax rate should be between 30% and 33% at $800K. If it's 36%+, your structure is leaking $35K a year."
+- **Core insight:** A 4.3 percentage point gap in effective tax rate means $35K-$40K per year in excess taxes. Over a decade, that compounds to over $500K.
+- **Platform tags:** [YT-SHORT]
+- **Estimated duration:** ~50 seconds
+### Clip 3
+- **Source segment:** Segment 6: The Treatment Plan
+- **Timestamp markers:** "The combined potential impact of all four treatments..." through "...And the only input required was reading the return."
+- **Hook line:** "Four findings on a tax return. Four structural fixes. Combined impact: $120,000 to $156,000 per year. No additional OR time."
+- **Core insight:** The four diagnostic markers (effective rate, QBI, retirement gap, state tax) together represent $120K-$156K in annual optimization, all from structural adjustments.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~50 seconds
+### Clip 4
+- **Source segment:** Segment 3: Finding Two, the QBI Deduction
+- **Timestamp markers:** "Now, when the QBI line shows zero..." through "...From a single calibration adjustment."
+- **Hook line:** "Your QBI deduction is zero. That's the financial equivalent of an ACL that should be intact but isn't. One number on your S-Corp setup could save you $17,000 a year."
+- **Core insight:** A zero QBI deduction on a surgeon's S-Corp return reveals a salary calibration issue. Adjusting one number can generate $11K-$17K in annual tax savings.
+- **Platform tags:** [IG-REEL]
+- **Estimated duration:** ~65 seconds
+---
+## COLD OPEN (30–60 seconds)
+You spent 10 or more years learning to read diagnostic images. You can look at an MRI and see what everyone else misses. You can spot a subtle meniscal tear, a stress reaction in the subchondral bone, an early avascular necrosis that a general practitioner would walk right past.
+But I'm willing to bet you've never looked at your own tax return with that same diagnostic eye.
+You hand it to your CPA. They file it. You move on. Maybe you glance at the refund line or the amount due. Maybe you wince. But the actual findings on that 30-page document? Nobody's reading them.
+And here's the thing: your tax return is trying to tell you something. It contains four specific diagnostic markers that reveal whether your financial structure is working or leaking. And today, I'm going to walk you through each one the same way you'd walk a resident through an imaging study. Finding by finding. With what "normal" looks like, what a concerning reading means, and what the treatment plan should be.
+---
+## INTRO AND CONTEXT (1–2 minutes)
+So here's the situation. We're in late March, which means April 15 is a few weeks away. Some of you have already filed your 2025 return. Others are in the final stretch of preparation. And some of you are planning to file an extension (which, by the way, is perfectly fine and something we'll talk about in a future episode).
+Whichever camp you're in, you either have a return in hand already or you will very soon. And that document represents the single most comprehensive snapshot of your financial life from the past 12 months. Your income, your deductions, your entity structure, your retirement funding, your state tax exposure. It's all there, on paper, in black and white.
+The problem is that most surgeons treat their tax return the way most patients treat their discharge paperwork. They glance at the summary, maybe ask one or two questions, and then put it in a drawer. The return gets filed as a compliance exercise. The CPA did their job. Box checked. Move on.
+But over the last four weeks, we've been building a framework for thinking about your financial structure with the same rigor you bring to clinical practice. We started with entity structure in Week 1. Then S-Corp salary calibration. Then the reimbursement environment and what it means for your practice economics. Last week, we talked about the one number that matters more than collections: your effective hourly rate.
+This week, we're going to pull all of those threads together. Because your tax return is the document that confirms or reveals every single one of those structural gaps. Think of it as the post-op imaging study on your financial year. The surgery (your financial decisions from last year) is done. The return shows you the results.
+And I'm going to build a hypothetical return, based on the kind of profile that's common at surgeon-level income, to walk through exactly what to look for.
+---
+## SEGMENT 1: The Case Study, and Why Most Surgeons Miss the Findings (3–5 minutes)
+Let me build a hypothetical profile to walk through. We'll call her Dr. K. She's 52 years old, practices orthopedic surgery in a mid-size metro area, and runs her practice through an S-Corp. She's busy. Clinically excellent. Her patients love her. She takes home a strong income by any reasonable standard.
+In a scenario like this, the typical reaction is, "Everything looks normal. My CPA said we're in good shape."
+And from a compliance standpoint, her CPA was right. The return was accurately prepared. Every number was correct. Every form was attached. No red flags for audit. From a compliance standpoint, it was a clean return.
+But compliance and strategy are two very different things.
+Here are the headline numbers from Dr. K's return. Adjusted gross income: $820,000. Total federal and state tax: $298,000. Effective tax rate: 36.3%. QBI deduction: zero. Total retirement contributions: $31,000. State income tax: $52,000.
+Now, if you're a surgeon and those numbers feel roughly familiar, that's because they're common. Returns with this profile are common at surgeon-level income. The income is high. The tax bill is large but feels "about right" given the income. The CPA confirms everything is in order. And the surgeon moves on, because nothing looks obviously broken.
+But let me show you what a diagnostic reading of this return actually reveals. Because when I look at those five numbers through a structural lens, I see four distinct findings, each pointing to a specific treatment recommendation.
+Think about it this way. When you look at an MRI of a knee, you don't just see "a knee." You systematically evaluate each structure: the menisci, the cruciate ligaments, the articular cartilage, the bone marrow signal. Each finding tells a story. Some findings are normal. Some are incidental. And some require intervention.
+Your tax return works the same way. So let's go through it, finding by finding.
+---
+## SEGMENT 2: Finding One, the Effective Tax Rate (3–5 minutes)
+The first thing I look at on any surgeon's return is the effective tax rate. This is total tax paid divided by adjusted gross income. It's the single number that tells you what percentage of every dollar you earned actually went to taxes.
+On Dr. K's return, that number is 36.3%. She earned $820,000 and paid $298,000 in combined federal and state tax.
+So what does "normal" look like? For a surgeon earning $800,000 to $900,000, a well-structured return typically shows an effective rate between 30% and 33%. I'm not talking about the marginal rate (the rate on your last dollar of income, which is 37% under the permanent OBBBA framework). I'm talking about the blended, all-in rate across every dollar from the first to the last, including state taxes.
+When I see 36.3%, that's a high reading. It tells me that several structural optimizations are likely missing. The return is paying close to the marginal rate on a blended basis, which means there isn't enough happening between gross income and taxable income to create meaningful separation.
+Let me put a number on that. If Dr. K's effective rate were 32% instead of 36.3%, her total tax bill would be $262,400 instead of $298,000. That's a difference of $35,600. Not a deduction. Not a credit. Just the mathematical consequence of having a more efficiently structured financial picture.
+And here's why this matters beyond the single year. If that 4.3 percentage point gap persists (and it will, if nothing changes structurally), we're talking about $35,000 to $40,000 per year in excess taxes. Over a 10-year period, that's $350,000 to $400,000. Invested at a reasonable rate of return, it compounds to something considerably north of half a million dollars.
+The effective tax rate is the vital sign of your return. It doesn't tell you exactly what's wrong, but a high reading tells you to keep looking. And in Dr. K's case, it pointed me directly to the next three findings.
+---
+## SEGMENT 3: Finding Two, the QBI Deduction (3–5 minutes)
+The second diagnostic marker is the Qualified Business Income deduction, or QBI. Under current law (made permanent by OBBBA), S-Corp owners can deduct up to 20% of their qualified business income. For surgeons running their practice through an S-Corp, this deduction is potentially worth tens of thousands of dollars.
+On Dr. K's return, the QBI deduction was zero.
+Now, when the QBI line shows zero for a surgeon operating through an S-Corp, that's a significant finding. It's the financial equivalent of seeing an ACL that should be intact but isn't. Something structural has happened.
+So why was Dr. K's QBI deduction zero? The answer lives in how her S-Corp salary was calibrated. Remember, the QBI deduction applies to the pass-through income from the S-Corp, not the W-2 salary. The more income that flows through as salary, the less qualifies for QBI.
+Dr. K's CPA had set her W-2 salary at $550,000. The remaining $270,000 flowed through as distributions. But at that salary level, combined with the income thresholds and phase-out calculations for specified service trades (which includes medical practices), the deduction phased out entirely.
+This is a calibration issue. Her salary wasn't wrong in the sense that it was unreasonable or indefensible. It was defensible. But it wasn't optimized. A salary in the range of $350,000 to $400,000 (still reasonable for an orthopedic surgeon of her experience and production, and well within IRS guidelines) would have increased the pass-through income and, depending on the interaction with the phase-out thresholds, generated a QBI deduction of approximately $30,000 to $45,000.
+Let me say that more plainly. By adjusting one number on her S-Corp setup, a number that most surgeons never revisit after their CPA initially sets it, Dr. K could reduce her taxable income by $30,000 to $45,000 per year. At her marginal rate, that's $11,000 to $17,000 in annual tax savings. From a single calibration adjustment.
+And this connects directly to what we talked about in Week 2. Your S-Corp salary is one of the most consequential financial decisions you make, and most surgeons set it once and never think about it again. The QBI line on your return is the diagnostic marker that tells you whether that calibration is working.
+If your QBI deduction is zero and you run an S-Corp, that's a finding. It deserves a follow-up conversation with your advisor.
+---
+## SEGMENT 4: Finding Three, the Retirement Contribution Gap (3–5 minutes)
+This is the finding that tends to land hardest. It's the one that makes the math impossible to ignore, the same way the effective hourly rate calculation from last week changed the entire picture.
+On Dr. K's return, total retirement contributions were $31,000. That's the 2025 401(k) employee deferral maximum (including catch-up, since she's over 50, it could have been $32,500, but she contributed $31,000). She funded her 401(k). She felt good about it. Her CPA confirmed it was maxed out.
+But "maxed out" is a misleading phrase. Because the 401(k) employee deferral is only one layer of the retirement contribution architecture available to an S-Corp surgeon.
+Here's what the full picture looks like in 2026. The 401(k) employee deferral is $24,500, with an $8,000 catch-up if you're 50 or older (and a $11,250 super catch-up if you're 60 to 63, which is new). The employer profit-sharing contribution can bring the total defined contribution up to $72,000. And then there's the cash balance plan, which, depending on your age, can shelter an additional $150,000 to $350,000 or more per year in tax-deductible contributions.
+So let's do the math on Dr. K. She contributed $31,000. The total available capacity, if she had a properly structured retirement plan architecture with a cash balance plan layered on top, would have been approximately $203,000.
+That's a gap of $172,000.
+Let me make that tangible. At her marginal rate of roughly 40% (combining federal and state), that $172,000 in additional contributions would have reduced her current-year tax bill by approximately $69,000. Sixty-nine thousand dollars. In one year. And the money doesn't disappear. It goes into her retirement account, where it compounds tax-deferred.
+If Dr. K makes that change and maintains it for 10 years (she's 52, planning to practice until at least 62), the cumulative tax-deferred contributions total $1.72 million. At a modest 6% annual return, the compounded value is approximately $2.4 million. Compared to what she's currently doing ($310,000 over 10 years, compounding to roughly $430,000), the difference is nearly $2 million in retirement wealth.
+From one structural change. On one line of the return.
+This is why I call the retirement contribution line the loudest finding on most surgeon returns. The gap between what was contributed and what was available is almost always the single largest missed opportunity. And it's sitting right there on the return, in plain view, every single year.
+Now, I want to be clear about something. Setting up a cash balance plan requires intention. It requires plan design, actuarial calculations, and ongoing administration. Your CPA may not bring it up, because it's outside their core compliance work. Your 401(k) provider won't bring it up, because they don't offer it. It typically requires a conversation with an advisor who understands how to layer defined benefit plans on top of defined contribution plans for high-income practice owners.
+But the first step is just seeing the gap. And your return shows it to you.
+---
+## SEGMENT 5: Finding Four, the State Tax Burden (3–5 minutes)
+The fourth diagnostic marker is one that surgeons often overlook entirely, because it feels fixed. It feels like a fact of geography rather than a planning variable. But for a surgeon earning $800,000 or more, state taxes deserve the same structural analysis as any other line on the return.
+Dr. K paid $52,000 in state income tax. She practices in a state with a top marginal rate of about 6.5%. On $820,000 of income, that comes out to roughly $52,000. Straightforward math.
+But here's the question worth asking: is that $52,000 a necessary cost of doing business, or is it a wealth drag that could be mitigated?
+Now, I want to be careful here. I'm not going to tell you to move to Florida or Texas. That's the lazy version of this conversation, and it ignores everything that makes your life work: your practice, your referral network, your community, your family's roots. Uprooting your life to save on state taxes is rarely the right answer, and frankly, it's rarely necessary.
+But there are structural strategies within a high-tax state that most surgeons never explore. For example, if Dr. K has investment income (rental properties, portfolio income, business interests outside her practice), the sourcing of that income matters. Some states tax all income regardless of source. Others allow favorable treatment for certain types of passive or investment income. The structure of her entities, the location of her investments, and the allocation of income across entities can all influence the state tax line without requiring a change of address.
+There's also the question of trajectory. If Dr. K is planning to retire in 8 to 10 years and relocate to a lower-tax state at that point, the timing of certain income events (selling a practice interest, triggering capital gains, taking large retirement distributions) can be strategically planned around the move. A $52,000 annual state tax bill, multiplied by the remaining years in a high-tax state, is a planning variable worth quantifying.
+And for surgeons who split time between states, who do locum work in different jurisdictions, or who have practice interests in multiple locations, the state tax picture gets more complex and more optimizable. Thoughtful state tax planning can reduce the burden by $15,000 to $30,000 annually without requiring a change of address.
+The point here is not that $52,000 in state tax is "wrong." The point is that it's a finding worth investigating. Just like a radiological finding that may be incidental or may be clinically significant, the state tax line deserves a focused look. And for many surgeons, it reveals options they didn't know they had.
+---
+## SEGMENT 6: The Treatment Plan, Turning Findings Into Actions (3–5 minutes)
+Alright, so we've walked through the four diagnostic markers on Dr. K's return. Let me bring them together, because a diagnosis without a treatment plan is just a list of findings. And you'd never hand a patient a radiology report and say, "Good luck."
+Here's the treatment plan, one action per finding.
+**Finding one: effective tax rate at 36.3%.** Treatment: schedule a structural review with your financial advisor before Q3. The goal is to identify which specific structural gaps (S-Corp salary, retirement plan architecture, deduction strategy) are contributing to the elevated rate and model the impact of correcting each one. Target: an effective rate of 31% to 33%, which at $820,000 represents $25,000 to $40,000 in annual tax savings.
+**Finding two: QBI deduction of zero.** Treatment: request an S-Corp salary analysis from your CPA or advisor. The question is specific: "At what salary level does my QBI deduction phase in, and what is the optimal range that balances payroll tax savings against QBI eligibility?" This is a quantitative exercise, not a judgment call. The math will give you a clear answer. Potential impact: $11,000 to $17,000 per year.
+**Finding three: retirement contributions of $31,000 versus $203,000 available.** Treatment: explore adding a cash balance plan to your existing retirement plan architecture. This requires a conversation with an actuary and a retirement plan specialist, not just your 401(k) provider. The key question: "Given my age, income, and planned retirement timeline, how much additional tax-deferred contribution capacity is available to me?" Potential impact: $69,000 in current-year tax reduction, with compounding benefits of $1.5 to $2 million over the next decade.
+**Finding four: state tax of $52,000.** Treatment: request a state tax exposure analysis. Ask your advisor to map your income sources and evaluate whether entity structuring, income sourcing, or retirement timing adjustments could reduce your state tax burden. This is especially important if you're within 10 years of a planned relocation or if you have income sources outside your primary practice. Potential impact: $15,000 to $30,000 annually, depending on circumstances.
+Now, here's what I want you to notice about this treatment plan. None of these actions require you to earn more money. None of them require additional OR time. None of them require you to take on more patients or more risk. Every single one is a structural adjustment to how the money you already earn flows through your financial life.
+The combined potential impact of all four treatments for Dr. K? Conservatively, $120,000 to $156,000 per year in reduced taxes and increased retirement funding. And the only input required was reading the return.
+---
+## LISTENER TAKEAWAY (1–2 minutes)
+Alright, here's what I'd like you to do this week. And I mean this week, because if you've already filed or if you're about to, the return is fresh and available.
+Pull out your 2025 tax return. Or ask your CPA to send you the final copy. And look at four numbers.
+First, calculate your effective tax rate. Total tax paid (line 24 on Form 1040, plus your state return) divided by your adjusted gross income (line 11 on Form 1040). If that number is above 33%, circle it.
+Second, look for your QBI deduction. It's on line 13 of Form 1040. If it's zero and you operate through an S-Corp, circle it.
+Third, find your total retirement contributions. This may require looking at your W-2 (box 12, code D for 401(k) deferrals) and any additional contributions reported on your S-Corp return. Compare what you contributed to the $72,000 defined contribution limit, and, if you're over 45, to the additional $150,000 to $350,000 available through a cash balance plan. Calculate the gap.
+Fourth, add up your state income tax. It's on your state return, and it's also reflected in the SALT deduction on Schedule A. Write down the number.
+You can do this in 15 minutes. You don't need to solve anything today. You just need to see the findings. Because once you see them, you can't unsee them. And that's when the real planning conversation starts.
+If you want to take this further, bring those four numbers to your next conversation with your financial advisor. If they don't know what to do with them, or if they've never walked you through your return as a diagnostic document, that tells you something important about whether your advisory relationship is built for compliance or strategy.
+---
+## PHILOSOPHICAL CLOSE (1–2 minutes)
+I want to close with something that's been on my mind throughout this episode.
+You've spent your career developing a skill that very few people in the world possess: the ability to look at complex diagnostic information and see what it means. To look at an MRI and see, not just anatomy, but a story. A story about what happened, what's happening now, and what will happen next if you don't intervene.
+That skill transfers. It transfers directly to your financial life.
+A diagnosis without a treatment plan is just information. The same is true for your tax return. The return tells you what happened. What you do with it determines what happens next.
+And the surgeons who build the most wealth over the course of a career are the ones who bring that diagnostic rigor to their financial documents. They don't just file and forget. They read, they interpret, and they act. The same way they do in the clinic every single day.
+Your tax return is not a compliance document. It's a diagnostic report. And nobody should be better at reading diagnostic reports than you.
+Thanks for spending this time with me today. Talk to you next week.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: The 75% figure is the post's central data point and captures the structural gap in a single number. Presenting it as a bold stat card creates immediate visual impact and makes the legislative change feel concrete rather than abstract.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "75%" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "of cost increases covered" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "Medicare physician payment update, 2026 forward" in Inter Regular, approximately 15pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: clear, sobering, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "75%" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), center. "of cost increases covered" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "Medicare physician payment update, 2026 forward" in Inter Regular, ~15pt, Warm Gray (#9AA3A8), below secondary.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>week-3-linkedin-3.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="120" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Week 3 (March 9–15)</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Three Overhead Line Items Most Practices Never Benchmark</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Reimbursement Shift and Practice Wealth</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Extends the week's reimbursement theme into actionable territory. Posts 1 through 3 established why structural optimization matters more than volume increases. This post gives surgeons three specific overhead categories to examine, making the "2% overhead reduction" concept from the anchor blog concrete and immediately actionable.</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Most orthopedic practices track revenue closely. Far fewer benchmark the three overhead categories that determine how much of that revenue the surgeon actually keeps.
-If a 2.5% reimbursement cut costs your practice $32,000 a year, and a 2% overhead reduction recovers the same $32,000 with zero additional procedures, the question becomes: where does that 2% come from?
-When you analyze orthopedic practice overhead, there are three line items that almost always have room:
-→ Supply and vendor contracts. When was the last time your practice benchmarked implant pricing, surgical supplies, and office materials against peer practices? Most practices haven't renegotiated in years. A 5% reduction in supply costs alone can recover $10,000 to $20,000 annually.
-→ Staffing ratios. And I want to be clear: this is not about cutting staff. Practices that have grown over time often carry staffing structures built for an earlier version of the practice. Aligning roles, scheduling workflows, and staffing ratios with current patient volume can reduce overhead 1% to 3% without reducing quality of care.
-→ Facility utilization. If you own your space or hold a long-term lease, unused operatory time, underutilized square footage, and energy costs add up quietly. For surgeon-owned buildings, a cost segregation study can also accelerate depreciation deductions on top of the overhead savings.
-None of these require adding a single case to your schedule. All three are within your control.
-The reimbursement environment is tightening. The practices that absorb it best are the ones that know exactly where their overhead sits relative to their peers.
-When was the last time your practice ran that comparison?</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
+Image type: Podcast cover art / YouTube thumbnail
+Rationale: The image must communicate the intersection of clinical diagnostic skill and financial analysis. A clean, authoritative design pairing the language of medical imaging with financial documents creates immediate recognition for the surgeon audience. The visual should feel analytical and precise, matching the episode's diagnostic walkthrough tone. Avoiding any literal medical imagery (no actual MRI scans or stethoscopes) keeps the design in the financial advisory space while the text carries the clinical metaphor.
+AI image prompt: Create a 1400x1400px square podcast cover art image. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: text-dominant composition with content centered vertically and left-aligned with 100px left margin. Primary text: "Your Tax Return" in Playfair Display SemiBold, approximately 90pt, Off-White (#F6F7F5), left-aligned, positioned in the upper-center area of the canvas. Secondary text: "Is a Diagnostic Report" in Inter Regular, approximately 48pt, Warm Gray (#9AA3A8), positioned directly below primary text with 20px spacing, same left alignment. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 60% of the canvas width beneath the secondary text, starting from the left margin. Below the accent line, four short horizontal bar segments of varying lengths arranged vertically (suggesting diagnostic readings or chart findings), rendered in Antique Gold (#B08D57) at 40% opacity, with subtle spacing between them. The bars decrease in length from top to bottom, evoking a waterfall chart or diagnostic marker readout. Bottom of canvas: "CAPABLE WEALTH" in Inter Medium, 24pt, Blue Slate (#5F7483), centered horizontally, 60px from bottom edge. No cartoons, no clip art, no stock photography, no illustrations of people, no medical imagery, no MRI scans. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No generic stock, no clickbait styling, no busy compositions. Mood: analytical, calm, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Your Tax Return" in Playfair Display SemiBold, ~90pt, Off-White (#F6F7F5), upper-center left-aligned. "Is a Diagnostic Report" in Inter Regular, ~48pt, Warm Gray (#9AA3A8), below primary text. "CAPABLE WEALTH" in Inter Medium, 24pt, Blue Slate (#5F7483), centered at bottom.
+Platform and dimensions: Podcast cover 1400x1400, YouTube thumbnail variant 1280x720 (text repositioned to center-left two-thirds, right third left open for subtle atmospheric texture)</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>week-5-podcast-tax-return-mri.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n"/>
+      <c r="C11" s="3" t="n"/>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="200" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>The Three April 15 Decisions Hiding in Plain Sight</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta — filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Video Podcast Script (uploaded to YouTube; audio distributed to podcast platforms)</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Companion piece to the Week 6 anchor blog. While the blog focuses on the backdoor Roth decision tree, this podcast widens the lens to cover all three April 15 decisions (file/extend, IRA contribution, estimated payment) and how they interact. Timing is critical: this episode must be available before April 15 to have maximum impact. Builds on Week 5's diagnostic framework by showing how the return's findings lead to specific, time-sensitive decisions at the April 15 deadline.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>## Clip Extraction Map
+### Clip 1
+- **Source segment:** Cold Open
+- **Timestamp markers:** "Most surgeons think April 15 is about one thing..." through "...That's not a strategy. That's inertia dressed up as a deadline."
+- **Hook line:** "April 15 has three decisions hidden inside it. Most surgeons see only one."
+- **Core insight:** April 15 bundles three distinct decisions: file/extend, prior-year IRA contribution, and Q1 estimated payment. Most surgeons only address the first consciously.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~50 seconds
+### Clip 2
+- **Source segment:** Segment 2: Decision Two, The Prior-Year IRA Contribution
+- **Timestamp markers:** "But OBBBA changed that calculation..." through "...April 15 should trigger a deliberate analysis, not a reflexive deposit."
+- **Hook line:** "You've been funding a backdoor Roth every year because someone told you to. OBBBA changed the math. Here's why."
+- **Core insight:** With the 37% top rate made permanent, paying 40%+ now to avoid 22-24% later may be the most expensive way to save $7,500. A cash balance plan redirect saves $3,150 immediately.
+- **Platform tags:** [BOTH]
+- **Estimated duration:** ~55 seconds
+### Clip 3
+- **Source segment:** Segment 1: Decision One, File or Extend
+- **Timestamp markers:** "Here's the reality. More than half of high-income taxpayers file extensions." through "...I'll take that trade every time."
+- **Hook line:** "The extension isn't procrastination. More than half of high-income taxpayers file extensions. Here's why it might be the smarter move."
+- **Core insight:** Extensions give time for late K-1s, complex modeling, and current-year planning. The cost of overpaying by $5K for six months is ~$100 in forgone interest.
+- **Platform tags:** [IG-REEL]
+- **Estimated duration:** ~70 seconds
+---
+## COLD OPEN (30–60 seconds)
+Most surgeons think April 15 is about one thing: taxes. File or extend. Pay what you owe. Move on.
+But April 15 is actually three separate financial decisions compressed into one day. And most surgeons make only one of them consciously.
+Here's what I mean. On April 15, you're not just deciding whether to file your return. You're also deciding whether to make a prior-year IRA contribution (which for many of you means the backdoor Roth question). And you're making your Q1 estimated tax payment for 2026, which is either calibrated to your actual income trajectory or it's a guess based on last year's numbers.
+Three decisions. One date. And the way most surgeons handle it is: they deal with the filing, let their CPA autopilot the estimated payment, and either fund the Roth because they always have or skip it because they forgot. That's not a strategy. That's inertia dressed up as a deadline.
+Today I want to walk through all three decisions, show you how they interact with each other, and give you a protocol you can run through with your advisor before April 15 arrives.
+---
+## INTRO AND CONTEXT (1–2 minutes)
+Last week, I talked about reading your tax return like a diagnostic report. Four findings, four treatment recommendations. If you listened to that episode, you now have a clearer picture of where your financial structure is working and where it's leaking.
+This week is about what you do with that diagnosis. Because April 15 is the first action point. The return told you what happened last year. April 15 is where you start shaping what happens this year.
+And here's the thing that makes April 15 unusual. Most financial deadlines involve one decision. Should I rebalance my portfolio? Should I adjust my 401(k) contribution? Should I fund the HSA? One question, one answer, move on.
+April 15 bundles three distinct decisions together, and they interact with each other in ways that most surgeons (and honestly, most advisors) don't think through carefully. Filing status affects your Roth contribution timing. Your Roth decision affects how much cash you have available for the estimated payment. Your estimated payment strategy affects your cash flow for the rest of the quarter.
+If you optimize each of these in isolation, you'll get a decent outcome. If you think about them as a system, you'll get a meaningfully better one.
+So let's take them one at a time, and then I'll show you how they connect.
+---
+## SEGMENT 1: Decision One, File or Extend (3–5 minutes)
+The first decision is the one everybody thinks about: do you file your return by April 15, or do you file an extension and push the deadline to October 15?
+Most people assume that filing an extension is a bad thing. It feels like procrastination. It feels like you're behind. And there's a vague sense that extensions attract audit attention, which (for the record) is not true. The IRS has said explicitly that filing an extension does not increase audit risk.
+Here's the reality. More than half of high-income taxpayers file extensions. This is not a fringe behavior. It is the norm for people with complex financial lives. And for surgeons in particular, there are real strategic reasons to extend.
+Let me walk through when extending makes sense.
+First, if you have K-1 income from partnerships, surgical centers, or real estate investments, those K-1s frequently arrive late. Sometimes March. Sometimes April. Sometimes later. Filing before all your K-1s are in means filing an incomplete return and then amending later, which is more work, more cost, and more headache than extending in the first place.
+Second, if your financial picture changed significantly in the prior year (you started a new practice, sold a piece of a surgery center, changed entity structures, took a distribution from a retirement plan), an extension gives your CPA and your advisor time to model the return correctly rather than rushing through it under deadline pressure. Tax preparation done under time pressure is tax preparation that misses things.
+Third, and this is the one most surgeons don't consider: if you're evaluating major financial moves for the current year (establishing a cash balance plan, recalibrating your S-Corp salary, evaluating a Roth conversion), the extension window gives you six months to make those decisions with better information. By July or August, you have a much clearer picture of your 2026 income than you do in April. And some of those decisions require the prior year's return to be finalized before they can be fully analyzed.
+Now, here's the critical nuance. Filing an extension extends your filing deadline. It does not extend your payment deadline. If you owe taxes on your 2025 return, that payment is still due April 15 even if you extend. You estimate what you owe, send the payment, and file the return later.
+For a surgeon earning $900,000 with a potential balance due of, say, $15,000 to $25,000, the extension calculus is straightforward. You send a payment of $25,000 on April 15 (round up to be safe, because underpayment penalties are more expensive than having a small overpayment refunded later). Then you use the next six months to file a complete, fully optimized return rather than a rushed one.
+The cost of overpaying by $5,000 for six months? At the current fed funds rate of 3.50% to 3.75%, you're forgoing roughly $100 in interest. That's the price of getting your return right. I'll take that trade every time.
+---
+## SEGMENT 2: Decision Two, The Prior-Year IRA Contribution (3–5 minutes)
+The second decision embedded in April 15 is one that a lot of surgeons make on autopilot, and it deserves more thought than it typically gets.
+April 15 is the last day you can make an IRA contribution for the prior tax year. For 2025 contributions, the limit is $7,500 (or $8,600 if you're 50 or older and using the catch-up provision). And for surgeons earning well above the Roth IRA income limits, this usually means the backdoor Roth strategy: you contribute to a traditional IRA with after-tax dollars, then convert it to a Roth IRA.
+I wrote about this in detail in this week's blog post, so I won't repeat the full decision tree here. But let me hit the key points that matter for the April 15 decision.
+The backdoor Roth has been the default recommendation for high-income earners for years. And for years, it made sense. The logic was simple: pay taxes now at today's rate, let the money grow tax-free, and withdraw it in retirement with no taxes owed. If tax rates go up in the future, you win because you locked in today's lower rate.
+But OBBBA changed that calculation. The One Big Beautiful Bill Act made the 37% top marginal rate permanent. Before OBBBA, there was an argument that rates might revert to 39.6% or higher, which made paying 37% now look like a bargain. That argument is substantially weaker today.
+So here's the question you need to ask: what will your marginal tax rate be when you withdraw this money?
+If you're a 52-year-old surgeon earning $1.1 million, you're paying a combined federal and state rate of roughly 40% to 42% on your last dollar of income. When you contribute $7,500 to a backdoor Roth, that money has already been taxed at 40%+ on the way in.
+Now fast-forward to retirement. If your retirement income drops to, say, $250,000 a year from Social Security, pension, and required minimum distributions, your effective federal rate might be 22% to 24%. If you've moved to a no-income-tax state (Florida, Texas, Tennessee, Wyoming), the combined rate drops further.
+In that scenario, you paid 40%+ going in for the privilege of not paying 22% to 24% coming out. The growth is tax-free, which has real value on a $7,500 contribution. But over 10 years at 7% growth, that $7,500 becomes roughly $14,750. The tax-free growth component is worth about $1,700 to $2,400 in avoided taxes. Meaningful, but not transformative.
+Compare that to redirecting the same $7,500 into a cash balance plan increase (if your plan allows it) or a donor-advised fund contribution. In the cash balance plan, the full $7,500 goes in pre-tax, saving you $3,150 in taxes immediately at a 42% combined rate. In a DAF, the charitable deduction generates a similar immediate tax benefit while accomplishing philanthropic goals.
+The point is not that the backdoor Roth is wrong. For some surgeons (particularly those with estate planning priorities, since Roth IRAs have no required minimum distributions and pass to heirs tax-free), it remains the right call. The point is that April 15 should trigger a deliberate analysis, not a reflexive deposit.
+And here's where this interacts with Decision One. If you file an extension, your prior-year IRA contribution deadline stays April 15. The extension doesn't change it. So even if you're extending your return, you still need to make the Roth decision by the 15th. Which means this decision can't wait for the extension period. It has to happen now.
+---
+## SEGMENT 3: Decision Three, The Q1 Estimated Tax Payment (3–5 minutes)
+The third decision is the one that gets the least attention, and it might matter the most over the course of the year.
+Your Q1 estimated tax payment for 2026 is due April 15. And for most surgeons, this payment is calculated using one of two methods: either your CPA set up quarterly vouchers based on last year's total tax liability divided by four, or you're using the "safe harbor" method, which means paying 110% of last year's tax divided into four installments.
+Both of these methods are designed to avoid underpayment penalties. Neither of them is designed to optimize your cash flow.
+Let me give you a specific example. Say you earned $950,000 in 2025 and your total federal tax liability was $280,000. The safe harbor amount (110% of prior year) is $308,000, divided into four quarterly payments of $77,000 each.
+But what if your 2026 income is tracking differently? Maybe you changed your case mix. Maybe your practice added a partner and your revenue share shifted. Maybe you started a cash balance plan in January that will shelter $200,000 in contributions. Your actual 2026 tax liability could be materially different from $308,000.
+If you're overpaying your quarterlies, you're essentially giving the IRS an interest-free loan. On a $20,000 overpayment across four quarters, at 3.5% interest, that's roughly $350 to $700 in forgone returns over the year. Not catastrophic, but not nothing either, and it adds up when compounded across years.
+If you're underpaying, you'll face penalties at the IRS underpayment rate, which currently runs around 7% to 8% annually. That penalty is non-deductible, meaning you're losing money with zero tax benefit.
+The right approach is to treat each quarterly payment as a calibration point. Not just "pay the voucher and move on," but "does this number still reflect my actual 2026 situation?"
+Here's what I recommend. Before you write that April 15 check, spend 20 minutes with your advisor or CPA reviewing three things.
+First, your year-to-date income. Is Q1 2026 tracking above or below your 2025 pace? If you've had a slower surgical quarter (maybe you took time off in February, or a few cases got rescheduled), your actual tax liability for the year may be lower than the safe harbor assumes.
+Second, your retirement contributions pacing. If you're funding a 401(k) at $24,500, a cash balance plan at $200,000+, and an HSA, those pre-tax contributions reduce your taxable income. Are your estimated payments reflecting those deductions, or are they calculated on gross income?
+Third, any structural changes. Did you recalibrate your S-Corp salary? Change your entity structure? Start a new investment that generates losses or deductions? Any of these can shift your estimated tax obligation.
+The surgeon who reviews these three inputs and adjusts the Q1 payment accordingly is making a strategic decision. The surgeon who autopilots the voucher amount from last year is flying blind. Both of them will end up paying approximately the same total tax for the year. But the first surgeon will have better cash flow throughout the year, more capital available for investment, and fewer surprises when the return gets filed.
+---
+## SEGMENT 4: How the Three Decisions Interact (3–5 minutes)
+Now here's where this gets interesting, and why I wanted to cover all three decisions in one episode rather than splitting them up.
+These decisions don't exist in isolation. They influence each other in ways that create second-order effects.
+Let me walk through a few examples.
+**The extension and the Roth contribution.** If you're planning to extend, you might assume that the Roth decision can wait too. It can't. April 15 is the deadline for prior-year IRA contributions regardless of whether you extend your filing. So if you're extending but haven't made the 2025 IRA contribution, you need to decide now. And here's the tension: if you haven't finished reviewing your 2025 return, you may not have the full picture you need to make the Roth decision optimally. You might not know your exact effective tax rate, your state tax burden, or whether a cash balance plan change would have been a better use of the dollars. The extension buys you time on the filing but not on the contribution. That asymmetry catches people.
+**The Roth contribution and the estimated payment.** If you decide to fund the backdoor Roth at $7,500 (or $8,600 if you're 50+) on April 15, that cash comes out of the same pool you're using for your estimated tax payment. For a surgeon writing a $77,000 estimated tax check and a $7,500 Roth contribution on the same day, the total outflow is $84,500. That's not a problem if your cash reserves are strong. But if your Q1 was lighter than expected, or if you have a major expense coming (a tuition payment, a home project, a practice equipment purchase), the combined outflow could strain your liquidity. The question becomes: do you fund the Roth fully, partially, or skip it this year and redirect the cash toward a better-calibrated estimated payment?
+**The estimated payment and the extension.** If you extend your return, your estimated payment takes on additional importance. Here's why. When you file by April 15, your return reconciles your estimated payments against your actual liability. You either owe a balance or get a refund. That feedback loop is relatively quick. But if you extend, that reconciliation doesn't happen until October. Which means your estimated payment strategy for Q2, Q3, and Q4 is running without a confirmed baseline for eight months. If your Q1 payment was miscalibrated, the error compounds across the remaining quarters.
+This is why I encourage surgeons to treat the extension not as a deferral of attention but as a commitment to increased attention. If you extend, you should be reviewing your estimated payment pacing at least quarterly with your advisor. Not just paying the voucher, but checking whether the voucher still makes sense.
+**A quick scenario to tie these together.** Consider a 54-year-old orthopedic surgeon earning $1.2 million. She's filing an extension because her surgery center K-1 hasn't arrived yet. She has $85,000 in cash reserves. Her Q1 estimated payment voucher says $82,000. She hasn't made her 2025 IRA contribution yet.
+If she pays the full estimated payment and funds the backdoor Roth at $8,600 (she's over 50), her total April 15 outflow is $90,600. That brings her cash reserves to negative territory, which means she'd need to pull from investments or a line of credit.
+The better approach: she reviews her Q1 income pacing with her advisor. It turns out her 2026 income is tracking about 8% below the 2025 safe harbor baseline because she cut back her surgical schedule in January to attend a conference and mentor a resident. Her advisor recalculates the Q1 estimated payment at $75,000 (still above the minimum to avoid penalties, but closer to reality). She funds the backdoor Roth at $8,600 because her estate plan prioritizes Roth assets for her children.
+Total outflow: $83,600. Cash reserves post-payment: $1,400. Tight, but manageable, and she has a surgical schedule in April that will rebuild the reserve within two weeks.
+Without looking at all three decisions together, she would have either overpaid the estimated tax, skipped the Roth reflexively, or strained her liquidity unnecessarily. Seeing them as a system let her optimize the whole package.
+---
+## SEGMENT 5: The One-Hour April 15 Protocol (3–5 minutes)
+Alright, let me give you something concrete you can use. I call this the one-hour April 15 protocol, and it's a checklist you can run through with your financial advisor or CPA in a single meeting before the deadline.
+Set aside an hour. Bring your most recent pay stubs or practice revenue reports, your 2025 return (or draft return, or whatever version you have), and your current estimated tax vouchers. Here's what you cover.
+**First fifteen minutes: the filing decision.**
+Ask three questions. Are all your K-1s in? (If not, you should probably extend.) Have there been any major financial events in 2025 that your CPA hasn't fully modeled yet? (Practice sale, real estate transaction, large charitable gift, significant capital gains.) Is there a planning benefit to the extension window? (Are you considering a cash balance plan, entity restructuring, or Roth conversion strategy that would benefit from more time?)
+If any of those answers point toward extending, extend. And remember: send your estimated balance-due payment on April 15 even if you're extending the filing.
+**Second fifteen minutes: the IRA contribution.**
+Work through a three-question decision tree. First, what is your current combined marginal tax rate (federal plus state)? At surgeon-level income, this is typically 37% federal plus your state rate, putting you somewhere between 37% and 50% combined depending on where you practice.
+Second, what do you expect your effective tax rate to be in retirement? If you're planning to draw $200,000 to $300,000 annually and move to a low-tax or no-tax state, your effective rate could drop to 18% to 24%.
+Third, do you have estate planning goals that favor Roth assets? Roth IRAs have no required minimum distributions during the owner's lifetime and pass to heirs income-tax-free. If leaving tax-free assets to the next generation is a priority, the backdoor Roth makes sense even when the rate arithmetic is unfavorable.
+If your current rate is much higher than your expected retirement rate and you don't have a strong estate planning reason, consider redirecting the $7,500 to $8,600 toward a cash balance plan increase, a DAF contribution, or simply keeping it liquid for the estimated payment.
+If you decide to fund the Roth, execute the backdoor: contribute to the traditional IRA, then convert to Roth. Do both steps before April 15 if possible, or at minimum make the contribution by April 15 and convert shortly after.
+**Third fifteen minutes: the estimated payment.**
+Review your Q1 2026 income against your annualized safe harbor projection. Is your income pacing above, below, or in line with the number your voucher is based on?
+Check whether your retirement contributions for 2026 are on pace. If you're front-loading your 401(k) or making early-year cash balance plan contributions, those reduce taxable income and should reduce your estimated payment.
+Confirm whether any structural changes (S-Corp salary adjustment, new entity, change in partnership income) have been reflected in the estimated payment calculation. If not, adjust.
+The goal is to pay enough to avoid penalties while keeping excess cash in your own accounts rather than at the IRS. For most surgeons, this means paying at or slightly above the safe harbor minimum, and then refining the number each quarter as more income data comes in.
+**Last fifteen minutes: document and schedule.**
+Write down the three decisions you made and the rationale for each. Set a calendar reminder for June 15 (Q2 estimated payment) to repeat the estimated payment calibration exercise. And if you extended, set a reminder for late August to begin preparing the return for October 15 filing.
+That's it. One hour. Three decisions. Each one deliberate rather than reflexive.
+---
+## LISTENER TAKEAWAY (1–2 minutes)
+If you take one thing from this episode, let it be this: April 15 is not one deadline. It's three decision points sharing the same calendar square.
+The surgeons who treat it as one thing ("get my taxes handled") will file or extend, write a check, and move on. And they'll be fine. They won't face penalties. They won't miss the filing deadline.
+But the surgeons who treat it as three things will ask better questions. Should I file or would extending give me a strategic advantage? Is the backdoor Roth still the best use of this $7,500, or has the math changed since OBBBA? Is my estimated payment calibrated to my actual 2026 income, or am I running on autopilot from last year?
+Those questions are worth about an hour of your time. And the answers, when you add up the cash flow optimization, the tax positioning, and the liquidity management, can easily be worth $10,000 to $30,000 across a single tax year.
+If you haven't already, download this week's blog post where I go deeper on the backdoor Roth decision tree specifically. And bring both pieces (this episode's protocol and the blog's decision framework) to your next advisor meeting. If your advisor looks at you like you're speaking a different language, that itself is a data point worth paying attention to.
+---
+## PHILOSOPHICAL CLOSE (1–2 minutes)
+I want to leave you with something I've been thinking about.
+We treat deadlines as obligations. Something we have to get through. File the return, pay the bill, check the box. And then we exhale and go back to work.
+But the most important moments in your financial life aren't the deadlines. They're the decisions embedded inside those deadlines. The deadline tells you when. The decision determines what.
+April 15 feels like a deadline. And it is one, technically. But it's also a decision point. Three of them, actually. And the quality of your financial life is determined not by the deadlines you meet, but by the decisions you make at each one.
+In surgery, the most critical moment in a procedure isn't the one everyone expects. It's the quiet decision two steps before: the angle of approach, the plane of dissection, the choice that shapes everything that follows. By the time the dramatic moment arrives, the outcome was already determined by the deliberate choice nobody saw.
+April 15 works the same way. The filing, the payment, the contribution. Those are the visible actions. But the decisions behind them (should I extend? should I fund the Roth or redirect? should I adjust my quarterly pacing?) are the quiet choices that shape the next twelve months of your financial life.
+Make them deliberately. Make them with good data. And make all three of them, not just the one that's loudest.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Primary Image
-Image type: Stat highlight card
-Rationale: A clean card listing the three benchmark categories creates a scannable, saveable reference that surgeons can screenshot or forward to their practice manager. The list format matches the post's actionable, checklist-style tone.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: left-aligned text composition with generous margins (120px top and bottom, 100px left, 80px right). Header text: "3 line items to benchmark" in Playfair Display SemiBold, approximately 36pt, Off-White (#F6F7F5), left-aligned, positioned in the upper quarter of the canvas. A thin horizontal rule (1px, Antique Gold #B08D57) spans 50% of the canvas width, left-aligned with the header text, positioned 24px below the header. Three list items below the rule, each in Inter Medium, approximately 22pt, Off-White (#F6F7F5), left-aligned, with 36px vertical spacing between items. Item 1: "Supply &amp; vendor contracts". Item 2: "Staffing ratios". Item 3: "Facility utilization". A small square bullet (6px, Antique Gold #B08D57) precedes each item with 16px horizontal spacing. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: actionable, organized, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "3 line items to benchmark" in Playfair Display SemiBold, ~36pt, Off-White (#F6F7F5), upper quarter left. Three list items in Inter Medium, ~22pt, Off-White (#F6F7F5), with Antique Gold (#B08D57) bullet squares.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>week-3-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="120" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Week 3 (March 9–15)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Is Your Practice Structured to Build Wealth, or Just to Generate Revenue?</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Reimbursement Shift and Practice Wealth</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Closes the week's LinkedIn sequence with a reflective, strategic-level post that ties the reimbursement theme back to the broader Q2 arc. Connects Week 3's external pressure (reimbursement cuts) to Weeks 1 and 2's internal structural gaps (entity structure, S-Corp salary, retirement plans), reinforcing the cumulative argument that financial structure determines how much of what you earn you actually keep.</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>There is a question worth asking every surgeon who owns a practice. It tends to land quietly, and then it stays with them.
-Is your practice structured to build wealth, or just to generate revenue?
-Because those are two very different things.
-A practice that generates revenue puts money through the door. A practice that builds wealth makes sure the surgeon keeps as much of it as possible, in the most tax-efficient way, through the most intentional structure.
-Over the past few weeks, we've looked at what happens when that structure has gaps. An S-Corp salary that hasn't been recalibrated in years can cost you $25,000 annually in misallocated self-employment tax. A missing cash balance plan leaves $45,000 to $80,000 per year in tax-deferred growth on the table. And now, a 2.5% reimbursement cut takes another $32,000 off the top.
-These are not separate problems. They compound. A surgeon earning $800,000 with all three gaps is losing over $100,000 a year to structural inefficiency. Over a decade, that's a seven-figure difference in personal wealth.
-And every one of those gaps is fixable. The S-Corp salary is adjustable. The cash balance plan can be established this year. The overhead can be benchmarked and reduced. The reimbursement cut, the one thing you can't control, becomes the smallest variable in the equation once the structure is right.
-You spent years building a practice that generates excellent revenue. The question worth sitting with is whether that practice is also structured to turn that revenue into lasting wealth.</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: The central question of the post works as a bold typographic statement that prompts self-reflection. Presenting it as a clean quote-style card creates a thumb-stopping moment in the feed and invites engagement.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "Revenue is what you bill." in Playfair Display Regular, approximately 32pt, Off-White (#F6F7F5), centered horizontally, positioned above the vertical center of the canvas. Secondary text: "Wealth is what you keep." in Playfair Display SemiBold, approximately 38pt, Antique Gold (#B08D57), centered horizontally, positioned 28px below the primary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, positioned 48px below the secondary text. Tertiary text: "Are you structured for both?" in Inter Regular, approximately 18pt, Warm Gray (#9AA3A8), centered horizontally, positioned 24px below the rule. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: reflective, composed, forward-looking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Revenue is what you bill." in Playfair Display Regular, ~32pt, Off-White (#F6F7F5), above center. "Wealth is what you keep." in Playfair Display SemiBold, ~38pt, Antique Gold (#B08D57), below primary. "Are you structured for both?" in Inter Regular, ~18pt, Warm Gray (#9AA3A8), below rule.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>week-3-linkedin-5.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>WEEK 4 (MARCH 16–22)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-    </row>
-    <row r="10" ht="120" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Week 4 (March 16–22)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Your Effective Hourly Rate Is the Number That Actually Matters</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>The Number That Matters More Than Collections</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Introduces the "surgeon effective hourly rate" concept as the true measure of financial health. Anchors the week's theme by contrasting collections (a practice metric) with effective hourly rate (a personal wealth metric), using real math to make the gap visceral.</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Your practice collected $2.4M last year. You kept $480K. Your effective hourly rate? $185.
-That number surprises most surgeons when they see it for the first time. And it should.
-Collections measure practice health. They tell you the business is generating revenue, the billing team is performing, and payers are reimbursing. Those are all good things to know.
-But collections don't tell you what you actually kept. And they definitely don't tell you what each hour of your time was worth after overhead, taxes, debt service, and retirement contributions came out.
-Here's the math on a $2.4M practice:
-→ 55% overhead: $1,320,000 gone before you see a dollar
-→ Federal and state taxes on the remainder
-→ Student loan payments, if applicable
-→ Retirement contributions (assuming you're maxing them)
-→ What's left: roughly $480,000
-Divide that by 2,600 clinical and administrative hours per year. You land at $185/hr.
-That's your effective hourly rate. The number that tells you what your time is actually producing for your family's wealth.
-Most surgeons have calculated their collections per case, their RVUs per quarter, their overhead percentage. Almost none have calculated this number. And yet this is the one that determines whether you're building wealth or just building a practice.
-If you've never run this calculation, this is the week to do it. The gap between what you collect and what you keep is where the real planning starts.</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: The stark contrast between $2.4M collections and $185/hr effective rate creates immediate cognitive dissonance, which drives engagement. A clean stat card communicates the math at a glance and stops the scroll.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: vertically stacked text composition, centered horizontally with 80px side margins. Top section (upper 40%): "$2.4M collected" in Inter Regular, approximately 36pt, Warm Gray (#9AA3A8), centered, positioned at roughly 30% from top. A thin horizontal divider line (2px, Blue Slate #5F7483, 60% canvas width) separates the top and bottom sections, centered vertically. Bottom section (lower 40%): "$185/hr kept" in Playfair Display SemiBold, approximately 56pt, Antique Gold (#B08D57), centered, positioned at roughly 65% from top. Subtle thin-line downward arrow icon (Antique Gold #B08D57, 2px stroke) between the two text blocks, centered, approximately 40px tall. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: contemplative, precise, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "$2.4M collected" in Inter Regular, ~36pt, Warm Gray (#9AA3A8), upper center. "$185/hr kept" in Playfair Display SemiBold, ~56pt, Antique Gold (#B08D57), lower center.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>week-4-linkedin-1.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="120" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Week 4 (March 16–22)</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>As Q1 Wraps Up, Ask About Your Keep Rate Before Anything Else.</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>The Number That Matters More Than Collections</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Ties the effective hourly rate concept to the upcoming Q1 close, making the post timely and actionable. Introduces "keep rate" as a digestible metric surgeons can track quarterly. Positions revenue growth without structural improvement as a warning sign, not a celebration.</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Q1 is wrapping up. When your revenue data lands, before you celebrate (or panic), ask this: did your keep rate go up or down?
-Keep rate is simple. It's the percentage of gross revenue that actually flows to your personal wealth after overhead, taxes, debt service, and savings. If your practice collected $600K in Q1 and you kept $120K, your keep rate is 20%.
-Here's why this matters more than the top-line number.
-This is a structural pattern that shows up frequently in surgeon-owned practices: a practice grows revenue by 8% year over year, the surgeon feels good about the trajectory, but overhead crept up by 10%. Taxes increased because the additional income pushed into a higher marginal bracket. And the retirement plan wasn't restructured to capture the growth.
-The result? Revenue went up. Keep rate went down. The practice got busier and more profitable on paper, and the surgeon's personal wealth-building actually slowed.
-Revenue growth without structural improvement means the practice generates more income for everyone except you. More for overhead. More for the IRS. More for lenders. The surgeon works harder, and the gap between collections and kept income widens.
-Your Q1 vital sign isn't revenue growth. It's keep rate direction.
-If revenue grew and keep rate grew with it, your structure is working. If revenue grew and keep rate stayed flat or declined, that's the signal to look under the hood before Q2 begins.
-One number. One question. That's your Q1 financial check-up when the numbers come in.</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: The question-driven format creates engagement by prompting self-reflection. A simple keep rate metric on the card gives surgeons a framework they can apply when their Q1 data comes in.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with 80px side margins. Upper third: "Q1 Keep Rate" in Inter Medium, approximately 28pt, Warm Gray (#9AA3A8), centered, positioned at roughly 28% from top. Center: a large upward or downward arrow icon composed of two versions side by side (one pointing up in Antique Gold #B08D57, one pointing down in Blue Slate #5F7483), each approximately 80px tall, separated by 40px, centered horizontally at 50% vertical. Lower third: "Which direction is yours?" in Playfair Display SemiBold, approximately 40pt, Off-White (#F6F7F5), centered, positioned at roughly 72% from top. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, direct, serious. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Q1 Keep Rate" in Inter Medium, ~28pt, Warm Gray (#9AA3A8), upper center. "Which direction is yours?" in Playfair Display SemiBold, ~40pt, Off-White (#F6F7F5), lower center.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>week-4-linkedin-2.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="120" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Week 4 (March 16–22)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>The Five Components of Your Effective Hourly Rate</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>The Number That Matters More Than Collections</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Framework post that breaks the effective hourly rate into five actionable components. Gives surgeons a mental model for understanding which variables they can influence, shifting the conversation from "I need to earn more" to "I need to optimize what flows through." Supports the anchor blog's core math.</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Your effective hourly rate has five components. You can influence four of them.
-Here's what sits between your gross collections and what each hour of your time actually produces:
-→ Gross Revenue: the total your practice collects. Largely driven by case volume, payer mix, and reimbursement rates. You have some control here, but the ceiling is set by how many hours you're willing to work.
-→ Overhead: the operating cost of the practice. Staffing, supplies, rent, insurance, billing. For most orthopedic practices, this runs between 50% and 60%. Even a 3-point reduction on $2.4M in collections frees up $72,000.
-→ Taxes: federal, state, self-employment, and payroll. This is where entity structure, S-Corp salary optimization, and deduction strategies make their biggest impact. The spread between a poorly structured and well-structured surgeon at the same income level can be $40,000 or more.
-→ Debt Service: student loans, practice acquisition debt, equipment financing. The interest rate, repayment timeline, and tax treatment of this debt all affect your hourly rate. Refinancing or restructuring can move the needle meaningfully.
-→ Retirement Savings: the money you're setting aside for future wealth. This is the one component where spending more actually improves your long-term hourly rate. Maximizing tax-deferred vehicles (401(k), cash balance plans) reduces your current tax burden and compounds over decades.
-The key insight: most surgeons try to improve their rate by increasing the first component. Working more hours, adding cases, negotiating higher rates. But the largest opportunity usually lives in components two through five, the structural side of the equation.</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: A clean numbered list on a card format makes the five components instantly scannable and shareable. The visual framework reinforces the teaching structure and gives surgeons a reference they'll return to.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: left-aligned text composition with 80px left margin and 80px right margin. Top section: "Your Effective Hourly Rate" in Playfair Display SemiBold, approximately 36pt, Off-White (#F6F7F5), left-aligned, positioned at roughly 15% from top. Below the title (starting at roughly 30% from top), five lines of text stacked vertically with 36px spacing between each line: "1. Gross Revenue" in Inter Medium, 24pt, Antique Gold (#B08D57). "2. Overhead" in Inter Medium, 24pt, Off-White (#F6F7F5). "3. Taxes" in Inter Medium, 24pt, Off-White (#F6F7F5). "4. Debt Service" in Inter Medium, 24pt, Off-White (#F6F7F5). "5. Retirement Savings" in Inter Medium, 24pt, Off-White (#F6F7F5). A thin vertical accent line (3px, Antique Gold #B08D57) runs along the left edge from the first item to the last item, positioned at 60px from the left edge. Bottom: "Which ones can you move?" in Inter Regular, 20pt, Warm Gray (#9AA3A8), left-aligned, positioned at roughly 85% from top. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: structured, educational, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Your Effective Hourly Rate" in Playfair Display SemiBold, ~36pt, Off-White (#F6F7F5), top left. Five numbered items in Inter Medium, ~24pt, stacked vertically. "Which ones can you move?" in Inter Regular, ~20pt, Warm Gray (#9AA3A8), bottom left.
-Platform and dimensions: LinkedIn, 1080x1080</t>
+Image type: Podcast cover art / YouTube thumbnail
+Rationale: The image must communicate the concept of three distinct financial decisions converging on a single date. A clean, structured visual with the number three and the date April 15 creates intellectual curiosity and signals strategic depth. The design should feel deliberate and analytical, matching the episode's decision-framework argument. The composition avoids urgency or deadline-panic styling in favor of calm authority.
+AI image prompt: Create a 1400x1400px square podcast cover art image. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: text-dominant composition with content centered vertically and left-aligned with 100px left margin. Primary text: "Three Decisions" in Playfair Display SemiBold, approximately 100pt, Off-White (#F6F7F5), left-aligned, positioned in the upper-center area of the canvas. Secondary text: "April 15" in Inter Regular, approximately 48pt, Warm Gray (#9AA3A8), positioned directly below primary text with 20px spacing, same left alignment. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 60% of the canvas width beneath the secondary text, starting from the left margin. Below the accent line, three small squares (24x24px each) arranged horizontally with 20px spacing, each filled with Antique Gold (#B08D57) at 80% opacity, representing the three decisions. Bottom of canvas: "CAPABLE WEALTH" in Inter Medium, 24pt, Blue Slate (#5F7483), centered horizontally, 60px from bottom edge. No cartoons, no clip art, no stock photography, no illustrations of people, no medical imagery, no calendar or clock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No generic stock, no clickbait styling, no busy compositions. Mood: deliberate, strategic, calm authority. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Three Decisions" in Playfair Display SemiBold, ~100pt, Off-White (#F6F7F5), upper-center left-aligned. "April 15" in Inter Regular, ~48pt, Warm Gray (#9AA3A8), below primary text. "CAPABLE WEALTH" in Inter Medium, 24pt, Blue Slate (#5F7483), centered at bottom.
+Platform and dimensions: Podcast cover 1400x1400, YouTube thumbnail variant 1280x720 (text repositioned to center-left two-thirds, right third left open for subtle atmospheric texture)</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>week-4-linkedin-3.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="120" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Week 4 (March 16–22)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>From $185 to $215 Per Hour Without Adding a Single Case</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>The Number That Matters More Than Collections</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Connects the entire March content arc (entity structure, S-Corp salary, reimbursement response, effective hourly rate) into a single proof of concept. Shows that the $30/hr improvement ($78K/year) comes from structural changes discussed over the prior three weeks, reinforcing that structure, not effort, drives the gap.</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>$185 per hour to $215 per hour. Same collections. Same hours. Same number of cases.
-The difference? $78,000 per year. And it comes entirely from structural improvements, not from working harder or seeing more patients.
-Over the past month, I've been walking through the specific changes that move this number. Here's how they add up for a surgeon collecting $2.4M annually:
-→ Entity structure optimization (proper S-Corp election, clean entity separation): reduces self-employment tax exposure and opens planning flexibility. Typical impact: $15,000 to $25,000.
-→ S-Corp salary calibration (setting reasonable compensation at the right level, not just the level your CPA defaulted to years ago): balances payroll tax savings against retirement contribution capacity and QBI deduction. Typical impact: $10,000 to $20,000.
-→ Proactive reimbursement response (restructuring overhead and revenue mix when payer rates shift): protects margins before they erode. Typical impact: $15,000 to $30,000 in preserved income.
-→ Retirement plan maximization (adding or optimizing a cash balance plan on top of a 401(k)): converts current taxable income into tax-deferred compounding. Typical impact: $20,000 to $40,000 in annual tax savings.
-None of these require you to operate on one more patient. None require a longer workday. They require a coordinated financial structure that's designed for surgeon-level income.
-The move from $185 to $215 per hour is a structural outcome. And it's available to most practice-owning orthopedic surgeons who haven't had this conversation yet.</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: The before/after hourly rate comparison creates a clear visual payoff for the month's content arc. The $78K annual difference translates the per-hour improvement into a number that commands attention.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered composition with 80px side margins. Upper section (roughly 25% from top): "Same hours. Same cases." in Inter Regular, approximately 24pt, Warm Gray (#9AA3A8), centered. Center section: two large numbers side by side, separated by a rightward-pointing arrow. Left number: "$185/hr" in Playfair Display SemiBold, approximately 48pt, Blue Slate (#5F7483), positioned at roughly 40% from left, vertically centered. Right arrow: a simple rightward arrow (→) in Antique Gold (#B08D57), approximately 36pt, centered between the two numbers. Right number: "$215/hr" in Playfair Display SemiBold, approximately 48pt, Antique Gold (#B08D57), positioned at roughly 65% from left, vertically centered. Lower section (roughly 75% from top): "+$78,000/year" in Inter SemiBold, approximately 32pt, Off-White (#F6F7F5), centered. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: confident, precise, compelling. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Same hours. Same cases." in Inter Regular, ~24pt, Warm Gray (#9AA3A8), upper center. "$185/hr → $215/hr" in Playfair Display SemiBold, ~48pt, center. "+$78,000/year" in Inter SemiBold, ~32pt, Off-White (#F6F7F5), lower center.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>week-4-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="120" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Week 4 (March 16–22)</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Four Weeks, One Message: Structure Determines What You Keep</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>The Number That Matters More Than Collections</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>End-of-month synthesis post that wraps the entire March Q1 Financial Health Check arc into a single philosophical takeaway. Provides narrative closure across all four weeks while creating a soft, natural bridge toward a coordinated review before the April 15 tax deadline.</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Four weeks. Four topics. One message.
-In the first week of March, we looked at entity structure: why the way your practice is organized determines your tax exposure, your liability protection, and your ability to build wealth through the business.
-In week two, we examined S-Corp salary calibration: the single number inside your entity that interacts with self-employment tax, retirement contributions, and the QBI deduction simultaneously.
-In week three, we addressed reimbursement cuts: how to respond structurally when payer rates decline, rather than simply absorbing the hit or working more hours to compensate.
-And this week, we put a number on all of it. Your effective hourly rate. The figure that tells you what each hour of your professional life actually produces for your family's wealth. For many surgeons, the structural improvements from weeks one through three move that rate from $185 to $215 per hour. That's $78,000 per year, with no additional cases and no longer days.
-The thread connecting all four weeks is simple: structure determines what you keep.
-You can't out-earn a broken structure. You can't out-save it either. At surgeon-level income, the difference between a well-designed financial structure and one that was never coordinated is six figures per year. Every year.
-April 15 is three weeks away. If you haven't looked at your entity, your salary, your retirement plan, and your effective hourly rate as a connected system, this is the window. A coordinated review before tax season closes can set the structure for the rest of the year.
-The work you put into your craft deserves a financial structure that matches.</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: A clean typographic card with the arc's core message serves as a capstone visual for the month. The philosophical framing elevates the post beyond tactical advice and gives it lasting shareability.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with 100px side margins. Single block of text vertically centered on the canvas: "Structure determines what you keep." in Playfair Display SemiBold, approximately 44pt, Off-White (#F6F7F5), centered horizontally, line-broken naturally if needed for balance. A thin horizontal accent line (2px, Antique Gold #B08D57, approximately 120px wide) centered below the text with 24px spacing. Below the accent line: "Q1 Financial Health Check" in Inter Regular, approximately 18pt, Warm Gray (#9AA3A8), centered, with 16px spacing from the line. Small "CAPABLE WEALTH" wordmark in Inter Medium, approximately 12pt, Blue Slate (#5F7483), centered at the bottom of the canvas with 60px bottom margin. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, authoritative, calm. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "Structure determines what you keep." in Playfair Display SemiBold, ~44pt, Off-White (#F6F7F5), centered. "Q1 Financial Health Check" in Inter Regular, ~18pt, Warm Gray (#9AA3A8), below accent line. "CAPABLE WEALTH" in Inter Medium, ~12pt, Blue Slate (#5F7483), bottom center.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>week-4-linkedin-5.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>WEEK 5 (MARCH 23–29)</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="120" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Week 5 (March 23–29)</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Your Tax Return Is a 30-Page Diagnostic Report. Nobody Read It for Strategy.</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Your tax return is a diagnostic report</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Leads into April's "Post-Filing Insights" month by reframing the tax return from a compliance document into a strategic diagnostic. Compresses the anchor blog's four-marker framework into a single, actionable LinkedIn post that positions the return as the most underread financial document a surgeon owns.</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Your tax return is a 30-page diagnostic report. Your CPA read it for compliance. Nobody read it for strategy.
-That is a problem worth fixing.
-Buried in those pages are four line items that tell you whether your financial structure is working or leaking. Your effective tax rate reveals whether you are actually paying what you think you are paying, or something significantly more. Your QBI deduction shows whether your S-Corp salary is calibrated correctly. Your retirement contributions tell you how much of your available tax-sheltered capacity you are using. And your state tax line tells you whether your entity geography is costing you money.
-For a surgeon earning $900,000, the spread between a well-structured return and a poorly structured one can exceed $120,000 in a single year. That is the difference between a return that was filed and a return that was read.
-Most CPAs are excellent at making sure you file correctly and on time. That is their job. But the question of whether your return reflects a financial structure that is actually optimized for your income, your practice, and your goals requires a different lens.
-Your return already has the answers. The question is whether anyone is asking the right questions of it.
-If you filed in the past two weeks, pull it back out. Look at those four lines. What do they tell you?</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: The "30-page diagnostic report" framing is the post's central reframe. Presenting it as a bold typographic statement creates an immediate pattern interrupt for any surgeon scrolling past tax season content.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "30 Pages" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper third of the canvas. Secondary text: "Your CPA read it for compliance." in Inter Regular, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 32px below the primary text. Tertiary text: "Nobody read it for strategy." in Inter SemiBold, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 16px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: authoritative, provocative, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "30 Pages" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), upper third center. "Your CPA read it for compliance." in Inter Regular, ~22pt, Off-White (#F6F7F5), below primary. "Nobody read it for strategy." in Inter SemiBold, ~22pt, Off-White (#F6F7F5), below secondary.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>week-5-linkedin-1.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="120" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Week 5 (March 23–29)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>A Surgeon's Return Showed $31,000 in Retirement Contributions. The Available Capacity Was $203,000.</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Your tax return is a diagnostic report</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Isolates the most visceral diagnostic marker from the anchor's four-line framework: the retirement contribution gap. Lets the numbers speak directly and positions the tax return as the document that exposes how much tax-sheltered capacity a surgeon is leaving unused every year.</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>A surgeon's return showed $31,000 in retirement contributions. The available capacity was $203,000. That $172,000 gap compounds every single year.
-Here is what that gap looks like in practice.
-A 401(k) with catch-up contributions for a surgeon over 50 allows $32,500 annually. Add a profit-sharing layer through an S-Corp, and you reach roughly $70,000. Layer in a cash balance plan, and the total available capacity can push past $200,000 in a single year, all tax-deferred.
-Most surgeons at this income level are using the 401(k) only. Some are maxing the employee contribution. Very few are using the profit-sharing component at all. Almost none have a cash balance plan in place.
-The result shows up on one line of the return: retirement plan contributions. And when that line reads $31,000 instead of $203,000, you are looking at the single largest structural gap in most surgical practices.
-This is not about being irresponsible. The surgeon in this example was disciplined, productive, and well-compensated. But the plan structure underneath was never built for an income at this level. A 401(k) designed for a $150,000 earner does not do the same work for someone earning $900,000.
-The tax return is where this shows up most clearly. One line. One number. And a gap that, over a decade, costs more than most people's houses.
-What does your retirement contribution line say?</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph (photorealistic, people)
-Rationale: The $172,000 retirement gap is fundamentally about a surgeon who doesn't realize the capacity available to them. A photorealistic image of a senior surgeon reviewing financial documents creates an immediate sense of "that could be me" and grounds the abstract gap in a concrete, relatable moment.
-AI image prompt: Create a 1080x1080px square photorealistic image. A male surgeon in his late 50s, wearing a tailored charcoal sport coat over a white open-collar dress shirt, seated at a clean modern walnut desk. He is reviewing a multi-page printed financial document, one hand resting on the pages, the other holding a pair of reading glasses. The setting is a private office with a large window behind and to the right, soft late-afternoon natural light illuminating the desk surface and the side of his face. Background softly out of focus: a few books on a minimal shelf, neutral gray wall. His expression is thoughtful and focused, slightly furrowed brow, as if discovering something unexpected in the numbers. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field, sharp focus on his hands and the document. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no handshakes, no stethoscope on money). Mood: sobering, precise, introspective. Photorealistic editorial photography style suitable for a financial advisory brand serving orthopedic surgeons ages 45-65.
-Text overlay: None (photorealistic image, no text)
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>week-5-linkedin-2.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="120" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Week 5 (March 23–29)</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>The Extension Isn't Procrastination. It's a Strategy, If You Use It Right.</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Your tax return is a diagnostic report</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Extends the anchor's "return as diagnostic" message to surgeons who haven't filed yet. Reframes the extension from a sign of disorganization into the most valuable planning window of the year, creating a bridge between the April 15 deadline and the October 15 opportunity.</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>The extension isn't procrastination. It's a strategy, if you use it right.
-More than half of high-income taxpayers file extensions every year. There is a reason for that, and it has nothing to do with being behind.
-The six months between April 15 and October 15 represent the most valuable planning window on the tax calendar. During that period, you can finalize retirement plan contributions, restructure entity elections, establish or fund a cash balance plan, and make S-Corp salary adjustments that affect your current-year return.
-For a surgeon earning $1.2M, the planning decisions available during the extension period can shift the tax outcome by $40,000 to $80,000. That is not a rounding error. That is the difference between a return that was filed and a return that was optimized.
-The catch is that most people treat the extension as extra time to gather documents. They file the extension in April, put the return out of mind, and scramble again in September. The six-month window closes without a single strategic decision being made.
-Used correctly, the extension period is when you sit down with your return (or last year's return, if this year's is still being prepared), identify the four diagnostic markers, and build a plan to close any structural gaps before October.
-If you're planning to file an extension, or if you've already filed one, you are not behind. You are in the strongest planning position of the calendar. The question is whether you will use the time.
-What is one decision you could make before October 15 that would change next year's return?</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Simple infographic
-Rationale: The six-month planning window from April to October is a timeline-driven insight that benefits from a clean visual timeline rather than static text. A branded horizontal timeline shows the extension period as a deliberate strategic runway, making the abstract "six months" feel concrete and structured.
-AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (100px all sides). A horizontal timeline runs across the center of the canvas from left to right. Left endpoint: a small filled circle (12px, Deep Muted Blue #243A4B) with the label "April 15" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), positioned above the circle. Right endpoint: a small filled circle (12px, Antique Gold #B08D57) with the label "October 15" in Inter SemiBold, 16pt, Antique Gold (#B08D57), positioned above the circle. The timeline bar connecting them: 3px, Blue Slate (#5F7483). Three evenly spaced milestone markers along the timeline (small open circles, 8px, Blue Slate #5F7483). Below each milestone, labels in Inter Regular, 13pt, Charcoal (#1E2428): "Fund cash balance plan", "Restructure entity elections", "Finalize retirement contributions". Headline above the timeline: "6 Months of Planning Capacity" in Playfair Display SemiBold, 28pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper third. Below the timeline, a supporting line: "The extension is a strategy, not a delay." in Inter Regular, 15pt, Blue Slate (#5F7483), centered, positioned 48px below the timeline. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows, no chart junk. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: strategic, organized, empowering. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: "6 Months of Planning Capacity" in Playfair Display SemiBold, ~28pt, Deep Muted Blue (#243A4B), upper third. Timeline labels and milestones in Inter, various sizes, Charcoal and Blue Slate.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>week-5-linkedin-3.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="120" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Week 5 (March 23–29)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>There's a Deduction on Your Tax Return That's Either Worth $29,800 or $0. Which One Is Yours?</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Your tax return is a diagnostic report</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Zooms into one specific diagnostic marker from the anchor's four-line framework: the QBI deduction. Expands on the anchor's finding that QBI presence or absence reveals whether S-Corp salary calibration is correct, giving surgeons a concrete line item to find on their own returns.</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>There's a deduction on your tax return that's either worth $29,800 or $0. Which one is yours?
-The QBI deduction allows a 20% deduction on qualified business income. For a surgeon with $149,000 in S-Corp flow-through income, that translates to roughly $29,800 in deductions. At a 37% marginal rate, the tax savings approach $11,000 in a single year.
-But here's where it gets interesting. The QBI deduction is one of the most misunderstood lines on a surgeon's return because its presence or absence is almost entirely determined by how your S-Corp salary is set.
-Pay yourself too much in W-2 salary relative to the practice's net income, and the qualified business income shrinks or disappears entirely. The deduction drops to zero. Pay yourself a reasonable but carefully calibrated salary, and the QBI deduction appears, sometimes worth $25,000 to $35,000.
-The line between those two outcomes is not luck. It is structure. Specifically, it is the ratio between your W-2 salary and your total S-Corp distributions, and whether anyone has looked at that ratio since you set up the entity.
-Surgeons with nearly identical gross incomes can file returns with a $30,000 difference in QBI deductions. Same specialty, same region, same revenue range. The only variable is how the S-Corp salary has been calibrated.
-If your return shows a QBI deduction, check whether the amount reflects your full available capacity. If it shows zero, ask why. The answer usually points to a salary calibration conversation that should have happened a year ago.</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph (photorealistic, environment)
-Rationale: The QBI deduction is a hidden lever buried in the tax return. A photorealistic image of a calm, modern professional environment with a tax document visible on the surface creates a contemplative mood that pairs with the "look closer" message of the post without revealing the answer on the image itself.
-AI image prompt: Create a 1080x1080px square photorealistic image. A clean, modern executive desk surface shot from above at a slight angle. On the desk: a neatly printed multi-page tax return (1040 form partially visible), a fine-point pen resting on the pages, and a small potted succulent in the upper-left corner. The desk is walnut or dark wood grain. Soft natural light from a window on the right side casts gentle shadows across the surface. The background beyond the desk is softly out of focus: a neutral gray wall with a hint of a framed credential. No people visible, just the desk and documents suggesting someone has been studying the return. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field with sharp focus on the pen and the center of the document. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: precise, contemplative, quietly provocative. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
-Text overlay: None (photorealistic image, no text)
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>week-5-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="120" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Week 5 (March 23–29)</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Four Weeks of Structural Diagnosis. One Document That Confirms Everything.</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Your tax return is a diagnostic report</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Month-closing synthesis that bookends the transition from March's structural diagnosis arc to April's post-filing interpretation. Connects every prior week's insight (entity design, S-Corp salary, reimbursement pressure, effective hourly rate) to the tax return as the single validating document, reinforcing the cumulative argument built across the entire March content arc.</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Four weeks of structural diagnosis. One document that confirms everything.
-Over the past month, we've walked through the major structural levers in a surgical practice. Week by week, piece by piece.
-In Week 1, we looked at entity structure: whether your practice is organized as a sole proprietorship, an S-Corp, or something else entirely, and what that choice costs you in taxes every year. For surgeons earning above $500,000, the wrong entity election can mean $30,000 or more in unnecessary self-employment tax.
-In Week 2, we examined S-Corp salary calibration: the ratio between your W-2 and your distributions, and how that ratio determines whether you qualify for the QBI deduction, how much you pay in payroll taxes, and how much capacity you have for tax-deferred retirement contributions.
-In Week 3, the conversation shifted to external pressure. The CMS 2.5% efficiency adjustment reduced reimbursement for non-time-based orthopedic codes, making every dollar your practice earns more valuable and every structural inefficiency more costly.
-In Week 4, we reframed the entire picture through the effective hourly rate: the number that shows what you actually earn per hour of clinical work after taxes, overhead, and structural drag.
-Now here is the connection. Every one of those insights shows up on your tax return. Your entity election, your salary split, your retirement contributions, your effective rate. The return is the document that validates or contradicts everything.
-If the last four weeks prompted even one question about your financial structure, your tax return is where the answer lives.
-Have you looked at yours with fresh eyes?</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Data visualization
-Rationale: The post synthesizes four weeks of content into one closing argument. A convergence diagram showing four diagnostic threads flowing into a single document creates a visual summary that makes the cumulative narrative feel inevitable, rewarding readers who followed the arc while standing alone for new viewers.
-AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "4 Weeks. 1 Document." in Playfair Display SemiBold, 28pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, four horizontal rounded-rectangle boxes (approximately 300px wide x 48px tall each) stacked vertically with 20px spacing, centered horizontally. Each box has a 2px border in Blue Slate (#5F7483) with Off-White fill. Labels inside each box in Inter Medium, 15pt, Deep Muted Blue (#243A4B), centered: Box 1: "Entity Structure", Box 2: "S-Corp Salary", Box 3: "Reimbursement Pressure", Box 4: "Effective Hourly Rate". From the right edge of each box, a thin connecting line (2px, Antique Gold #B08D57) curves downward and converges to a single point below all four boxes. At the convergence point, a larger rounded rectangle (320px wide x 56px tall) with a solid Deep Muted Blue (#243A4B) fill. Label inside: "Your Tax Return" in Inter SemiBold, 16pt, Off-White (#F6F7F5), centered. Below the bottom box, 24px of spacing, then: "Every answer is on one document." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: composed, authoritative, clarifying. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: "4 Weeks. 1 Document." in Playfair Display SemiBold, ~28pt, Deep Muted Blue. Four labeled boxes and convergence to "Your Tax Return" box.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>week-5-linkedin-5.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="120" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Week 6 (March 30 – April 5)</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>You've Been Funding a Backdoor Roth Every Year Because Someone Told You To. Here's Why the Math Might Have Changed.</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Opens the week's LinkedIn sequence by challenging the reflexive backdoor Roth habit. OBBBA made the 37% top rate permanent, which fundamentally changes the Roth calculus for high-income surgeons who expect lower rates in retirement. Distills the anchor blog's central argument into a provocative, shareable one-liner that positions Capable Wealth as the advisor who questions conventional wisdom with math.</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>You've been funding a backdoor Roth every year because someone told you to. Here's why the math might have changed.
-The backdoor Roth IRA became a reflex for high-income physicians sometime around 2015. Fund the non-deductible IRA, convert immediately, pay the tax, and enjoy tax-free growth forever. Simple, clean, and almost universally recommended.
-But the tax landscape shifted when OBBBA made the 37% top rate permanent. That changes the equation in a way most surgeons haven't reconsidered.
-Here's the core question: are you paying 37% on your Roth contribution today, and do you expect to withdraw at a rate lower than 37% in retirement?
-If the answer is yes to both, the backdoor Roth may be the most expensive way to save $7,500.
-Consider the math. A surgeon earning $1.2M contributes $7,500 to a backdoor Roth at a 37% federal rate (plus state taxes in most cases). That contribution costs roughly $2,775 in tax today, paid on dollars that could have been directed to a pre-tax vehicle like a cash balance plan, where the same $7,500 would generate an immediate deduction.
-The Roth makes sense when you expect your future tax rate to be the same or higher. For a 55-year-old surgeon planning to retire at 65 with a significantly lower income, that assumption deserves scrutiny.
-This is not an argument against Roth accounts. They have real value in the right circumstances. But "I've always done it" is a habit, not a strategy. And at surgeon-level income, a habit that costs an extra $2,775 per year in unnecessary tax is worth reexamining.
-Before April 15, it's worth asking: does the Roth still earn its place in your plan, or are you funding it out of momentum?</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Stat highlight card
-Rationale: The 37% rate is the post's anchor data point and creates immediate recognition for any surgeon who sees it on their pay stub. A bold stat card makes the tax rate impossible to scroll past and frames the Roth question as a math problem, not a default decision.
-AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "37%" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "tax on every Roth dollar" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "Is that still the right move?" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: precise, thought-provoking, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
-Text overlay: "37%" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), center. "tax on every Roth dollar" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "Is that still the right move?" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below secondary.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>week-6-linkedin-1.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="120" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Week 6 (March 30 – April 5)</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Estimated Taxes Aren't a Quarterly Bill. They're a Quarterly Strategy Session.</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Extends the April 15 theme from the Roth question to the broader estimated tax strategy. Reframes Q1 estimated tax payments from an obligation into an opportunity, introducing a "quarterly financial vital signs" framework that positions each payment as a recalibration point for withholding, income timing, and retirement contribution pacing.</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Estimated taxes aren't a quarterly bill. They're a quarterly strategy session.
-Most surgeons treat their Q1 estimated payment (due April 15) the same way they treated it last year: same amount, same calculation, same assumptions. Write the check, move on.
-But your income probably changed. Your practice revenue may have shifted with the CMS efficiency adjustment. Your retirement contributions may be pacing differently. And OBBBA changed the rate structure in ways that affect how much you should be setting aside.
-Every estimated tax payment is a chance to recalibrate three things at once.
-First, your withholding accuracy. If you're consistently getting large refunds, you're lending the government money interest-free. If you're consistently underpaying, you're setting yourself up for penalties. The target is 100% of last year's liability or 110% of adjusted gross income, whichever applies. At surgeon income levels, the difference between those two thresholds can be meaningful.
-Second, your retirement contribution pacing. Q1 is 25% of the year. Are your 401(k) contributions on pace to max out ($24,500, plus $8,000 catch-up if you're 50 or older)? Is your cash balance plan funded proportionally? Falling behind in Q1 means compressing contributions into later quarters, which can create cash flow pressure.
-Third, your income timing. If you control the timing of distributions from your practice entity, the Q1 payment is a natural checkpoint to evaluate whether your current distribution schedule still makes sense given year-to-date revenue.
-One payment. Three strategic decisions embedded inside it.
-Before you write the April 15 check this year, it's worth spending 30 minutes asking whether the number on that check still reflects your current reality.</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph (photorealistic, people)
-Rationale: The post reframes estimated tax payments as quarterly strategy sessions. A photorealistic image of a surgeon and financial advisor reviewing numbers together conveys the proactive, collaborative relationship the post advocates, moving the image from an abstract number to a tangible moment of financial intentionality.
-AI image prompt: Create a 1080x1080px square photorealistic image. Two professionals seated across from each other at a clean, modern conference table in a well-lit office. One is a male surgeon in his mid-50s wearing a navy blazer over an open-collar white shirt; the other is a female financial advisor in her 40s wearing a charcoal blazer. Between them on the table: a printed financial summary, a laptop angled toward the advisor, and two ceramic coffee cups. The advisor is pointing at a line on the printed document while the surgeon leans in slightly, expression engaged and focused. The setting is a modern office with floor-to-ceiling windows, natural afternoon light creating soft highlights. Background softly out of focus: a cityscape or green campus visible through the windows. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field, sharp focus on the two professionals and the document between them. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no posed handshakes, no pointing at charts on a whiteboard). Mood: strategic, composed, collaborative. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
-Text overlay: None (photorealistic image, no text)
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>week-6-linkedin-2.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="120" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Week 6 (March 30 – April 5)</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>The April 15 Deadline Has Three Decisions Hidden Inside It. Most Surgeons See Only One.</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Unifying post that connects all three April 15 decisions into a single framework. Most surgeons see April 15 as a filing deadline. This post reveals that it is simultaneously the Q1 estimated payment deadline, the prior-year IRA contribution deadline, and the implicit start of the extension planning window. Positions Capable Wealth as the advisor who sees the full picture.</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>The April 15 deadline has three decisions hidden inside it. Most surgeons see only one.
-Everyone knows April 15 is the tax filing deadline. But for a surgeon with a practice entity, retirement plans, and estimated tax obligations, that single date carries two additional decisions that are just as consequential.
-Here's what's actually on the table:
-Decision 1: File or extend. If your return is straightforward and your numbers are final, filing by April 15 makes sense. If your practice financials are still being reconciled, or if there are planning opportunities that need more time (cost segregation studies, entity restructuring, retirement plan amendments), an extension to October 15 buys you six months of runway. An extension is not a red flag. It is a planning tool.
-Decision 2: Make your Q1 estimated tax payment. This is due April 15 regardless of whether you file or extend. The amount you choose should reflect your 2026 income trajectory, not just last year's numbers. Underpaying triggers penalties. Overpaying ties up cash that could be working elsewhere.
-Decision 3: Make your prior-year IRA contribution. You have until April 15, 2026 to fund a 2025 IRA contribution (up to $7,000, or $8,000 if you were 50 or older in 2025). If you haven't contributed yet and you're planning a backdoor Roth conversion, this is your last window.
-Three decisions, one date, and they interact with each other. Your filing status affects your estimated tax calculation. Your IRA contribution affects your Roth conversion timing. Your extension decision affects how much planning flexibility you have for the rest of the year.
-Which of these three have you addressed?</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Simple infographic
-Rationale: The post reveals three decisions hidden inside a single deadline. A clean three-panel infographic makes the framework immediately scannable and creates a saveable reference visual that surgeons can revisit as April 15 approaches.
-AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "April 15: Three Decisions, One Date" in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, three vertical panels arranged side by side with 24px spacing between them, each approximately 260px wide x 420px tall. Each panel has a 2px top border only (no sides or bottom). Panel 1 top border: Deep Muted Blue (#243A4B). Inside Panel 1: number "1" in Playfair Display SemiBold, 48pt, Deep Muted Blue (#243A4B), centered, at top. Below: "File or Extend" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Process decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Panel 2 top border: Antique Gold (#B08D57). Inside Panel 2: number "2" in Playfair Display SemiBold, 48pt, Antique Gold (#B08D57), centered, at top. Below: "Prior-Year IRA" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Strategy decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Panel 3 top border: Blue Slate (#5F7483). Inside Panel 3: number "3" in Playfair Display SemiBold, 48pt, Blue Slate (#5F7483), centered, at top. Below: "Q1 Estimated Tax" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Strategy decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Below all three panels, 32px spacing, then: "Which of these three have you addressed?" in Inter Regular, 15pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: clarifying, organized, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: "April 15: Three Decisions, One Date" headline. Three numbered panels with decision labels and types.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>week-6-linkedin-3.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="120" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Week 6 (March 30 – April 5)</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>$7,500 Into a Roth at 42% Tax, or $7,500 Into a Cash Balance Plan at 0% Tax. Same Money. Very Different Math.</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Zooms into the specific math comparison from the anchor blog, isolating the backdoor Roth vs. cash balance plan decision as a direct side-by-side. At surgeon income levels, the opportunity cost of a backdoor Roth contribution compared to redirecting those dollars to a cash balance plan is measurable and significant. This post makes the comparison visceral and concrete.</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>$7,500 into a backdoor Roth at a 42% combined tax rate, or $7,500 into a cash balance plan at 0% tax. Same money. Very different math.
-Let's walk through what's actually happening with each dollar.
-The backdoor Roth: You contribute $7,500 of after-tax dollars to a non-deductible IRA and convert to Roth. Because the money was already taxed at your marginal rate (37% federal plus 5% state in most states with income tax), you paid roughly $3,150 in tax to get those dollars into the Roth. The upside: tax-free growth and tax-free withdrawals in retirement.
-The cash balance plan: You contribute $7,500 of pre-tax dollars to a defined benefit plan. That contribution generates an immediate deduction at your marginal rate, saving you the same $3,150 in tax this year. The money grows tax-deferred and is taxed at your retirement rate when you withdraw it.
-Here's where the math gets interesting.
-If you expect your retirement tax rate to be 24% (a reasonable estimate for a surgeon drawing $300,000 to $400,000 annually from retirement accounts), the cash balance plan lets you defer $3,150 in tax today and eventually pay roughly $1,800 on the same $7,500 at withdrawal. Net savings: $1,350 on a single year's contribution.
-Over 10 years of making this choice, the cumulative tax savings from redirecting to a cash balance plan instead of a Roth can exceed $13,000, before accounting for the additional compounding on those deferred tax dollars.
-And cash balance plans allow contributions far beyond $7,500. For surgeons over 50, annual contributions can range from $150,000 to $350,000 or more, depending on plan design.
-The Roth is a good tool. But at your income level, is it the best use of the next $7,500?</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Data visualization
-Rationale: The post's entire argument is a side-by-side math comparison. A branded bar chart showing the tax treatment of the same $7,500 in two vehicles makes the opportunity cost immediately visible and creates a visual that surgeons can share with colleagues to illustrate the point.
-AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "Same $7,500. Very Different Math." in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, two vertical bar chart columns centered on the canvas with 80px horizontal spacing between them. Left bar: tall (approximately 340px height), filled with Blue Slate (#5F7483). Labeled above the bar: "42%" in Inter SemiBold, 28pt, Deep Muted Blue (#243A4B). Labeled below the bar in two lines: "Backdoor Roth" in Inter SemiBold, 15pt, Deep Muted Blue (#243A4B), then "Tax on contribution" in Inter Regular, 12pt, Blue Slate (#5F7483). Right bar: very short (approximately 20px height, representing near-zero), filled with Antique Gold (#B08D57). Labeled above the bar: "0%" in Inter SemiBold, 28pt, Antique Gold (#B08D57). Labeled below the bar in two lines: "Cash Balance Plan" in Inter SemiBold, 15pt, Deep Muted Blue (#243A4B), then "Immediate deduction" in Inter Regular, 12pt, Blue Slate (#5F7483). A thin Warm Gray (#9AA3A8) baseline (1px) connects the base of both bars. Below the chart, 40px spacing, then: "At surgeon income levels, the opportunity cost compounds." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows, no chart junk. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: precise, comparative, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
-Text overlay: "Same $7,500. Very Different Math." headline, "42%" and "0%" bar labels, vehicle names and descriptions below bars.
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>week-6-linkedin-4.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="120" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Week 6 (March 30 – April 5)</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Every Quarter, Four Numbers Tell You Whether Your Financial Plan Is on Track. Most Surgeons Check Zero of Them.</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn Post</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Closes the week's LinkedIn sequence by extending the estimated tax discussion into a broader quarterly discipline. Introduces a "quarterly vital signs" framework that gives surgeons four specific numbers to check each quarter, transforming a reactive tax compliance exercise into a proactive wealth-building habit. Positions Capable Wealth as the advisor who builds systems, not just solves problems.</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Every quarter, four numbers tell you whether your financial plan is on track. Most surgeons check zero of them.
-You check vital signs on every patient. You assess labs, imaging, and functional progress at regular intervals because waiting until something goes wrong is not a strategy. Your financial plan deserves the same discipline.
-Here are the four numbers worth reviewing every quarter:
-1. Year-to-date income vs. annual projection. Is your practice revenue tracking where you expected? If you're running 10% ahead, your tax obligations are higher than planned. If you're 10% behind (perhaps from the CMS efficiency adjustment), your retirement contributions and distributions may need adjusting.
-2. Retirement contribution pacing. At the end of Q1, you should be roughly 25% of the way to your annual maximum. For 2026, that means about $6,125 of your $24,500 401(k) limit (or $8,125 including catch-up contributions). If your cash balance plan calls for $200,000 this year, about $50,000 should be funded or committed.
-3. Estimated tax adequacy. Compare your Q1 payment to your projected annual liability. If your income is tracking higher than last year and your estimated payments haven't changed, you're building a shortfall that compounds each quarter. Better to catch it in April than discover it in January.
-4. Cash reserve level. How many months of personal and practice expenses can you cover without touching investments? The target for most surgeon households is three to six months of personal expenses and two to three months of practice overhead. If a large tax payment or equipment purchase just drew down your reserves, this is the quarter to rebuild.
-Four numbers. Fifteen minutes per quarter. The surgeons who check these consistently are the ones who never get surprised.
-Which of these four have you looked at this quarter?</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Primary Image
-Image type: Conceptual photograph (photorealistic, environment)
-Rationale: The post introduces a quarterly discipline framework using a clinical vital-signs analogy. A photorealistic image of a modern medical office environment evokes the clinical rigor the post advocates, connecting the surgeon's professional world to their financial discipline without being literal or heavy-handed.
-AI image prompt: Create a 1080x1080px square photorealistic image. A modern, well-lit medical office corridor viewed from a slight angle, early morning natural light filtering through large windows on the right side. The corridor is clean, minimal, and empty, with polished light-gray floors and white walls. A glass-walled conference room is partially visible on the left, with a clean table and two chairs inside, suggesting a structured meeting space. A single potted green plant sits at the far end of the corridor, providing a subtle touch of warmth. The overall feeling is one of order, discipline, and calm professionalism. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field with the far end of the corridor softly out of focus. No people, no text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: organized, professional, forward-looking. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
-Text overlay: None (photorealistic image, no text)
-Platform and dimensions: LinkedIn, 1080x1080</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>week-6-linkedin-5.md</t>
+          <t>week-6-podcast-april-15-decisions.md</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="85" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Strategic Context</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Visual Asset Brief</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Source File</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 3 (MARCH 9–15)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="120" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>You Did 100% More Work to Get Back 39%</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>The reimbursement shift and what it means for your wealth</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Isolates the volume trap math from the full episode into a self-contained clip that challenges the most common instinct surgeons have when reimbursement drops. The 39% recovery stat is a scroll-stopping number that reframes "do more cases" from productive to expensive, earning the click to the full episode.</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Adding 10 procedures to offset a $32K revenue loss sounds logical. Here's why it costs you more than it recovers.
+When you add procedures at the margin, those additional cases carry real incremental costs. OR time, anesthesia coverage, surgical supplies, implants, pre-op and post-op nursing, billing, follow-ups.
+The marginal cost of an additional procedure in a practice already operating near capacity is typically around 60% of the procedure's revenue.
+So those 10 additional procedures at $3,120 each generate $31,200 in gross revenue. But the marginal cost at 60% is $18,720. The net recovery is only $12,480.
+You added 10 cases to your surgical schedule, put in the extra hours, took on the additional clinical risk, and you recovered $12,480 of a $32,000 gap.
+That's a 39% recovery rate. You did 100% more work to get back 39% of what you lost.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The 39% stat is the clip's gut-punch number and must be the dominant visual element to stop the scroll and provoke the question "39% of what?"
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "39% Recovery" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "100% more work to get back 39% of what you lost." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: sobering, precise, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "39% Recovery" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "100% more work to get back 39% of what you lost." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>week-3-clip-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>$40,000 Hiding in Your Implant Contracts</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>The reimbursement shift and what it means for your wealth</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Extracts the most immediately actionable segment from the episode: implant renegotiation as a one-conversation recovery of the entire reimbursement gap. This clip delivers a concrete dollar amount and a specific first step, making it highly shareable among practice partners and administrators. Optimized for Instagram Reels where the slightly longer format allows the full vendor conversation framing.</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Most orthopedic practices negotiate implant pricing once and never revisit it. That single habit could be costing you $40,000 a year.
+Here's the reality. Implant pricing varies by 15% to 30% across vendors for functionally equivalent devices. If your practice is spending $400,000 a year on implants and supplies (which is common for a busy orthopedic group), a 10% reduction through competitive bidding or renegotiation saves you $40,000 annually.
+That's more than the entire $32,000 reimbursement gap, recovered without touching your surgical schedule.
+And you don't have to switch vendors. Often, the conversation starts with a simple request: "We'd like to see competitive pricing for equivalent products." Your current vendors will frequently match or beat competing offers to retain your business.
+The leverage is there. Most practices just never use it.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The $40,000 savings figure is the clip's core value proposition and directly answers the reimbursement gap. Leading with the dollar amount creates immediate relevance for any surgeon aware of the CMS cut.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$40,000/Year" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Hiding in the implant contracts you never revisited." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: revealing, direct, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$40,000/Year" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "Hiding in the implant contracts you never revisited." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>week-3-clip-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Less Revenue, $80,000 More Wealth</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>The reimbursement shift and what it means for your wealth</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Captures the episode's philosophical core in a single comparison that redefines success. The Surgeon A vs. Surgeon B contrast is immediately graspable and challenges the assumption that higher revenue equals better financial outcomes. The million-dollar decade gap is a powerful curiosity driver to the full episode.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Surgeon A collects $1.4 million. Surgeon B collects $1.35 million. Surgeon B takes home $80,000 more per year.
+How? Three things. Surgeon B renegotiated implant contracts two years ago and saves about $35,000 annually. Surgeon B runs one fewer FTE than Surgeon A for the same patient volume, saving another $60,000. And Surgeon B's S-Corp salary is calibrated to maximize retirement plan contributions, adding another $25,000 in tax-deferred value.
+Surgeon A generates more revenue. Surgeon B builds more wealth. And over a decade, at $80,000 per year in structural advantage, plus the compounding on the tax-deferred savings, the gap between them will be somewhere north of a million dollars.
+Same specialty. Same market. Same training. Completely different financial outcomes.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The side-by-side revenue vs. wealth comparison is the clip's central tension. Leading with the counterintuitive outcome (lower revenue, higher wealth) creates immediate cognitive friction that earns the view.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$1.35M vs. $1.4M" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Less revenue. $80,000 more wealth per year." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: provocative, clarity-driven, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$1.35M vs. $1.4M" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "Less revenue. $80,000 more wealth per year." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>week-3-clip-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 4 (MARCH 16–22)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>$185 an Hour: The Number Your Collections Report Hides</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>The number that matters more than collections</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>This clip isolates the most visceral reveal from the podcast: a surgeon collecting $2.4M keeps $185/hour. The math shock works as a standalone scroll-stop because it requires zero setup and reframes how the viewer thinks about their own compensation.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Your practice collected $2.4 million last year. You kept $480,000. Your effective hourly rate? $185.
+$480,000 divided by 2,600 hours of clinical work equals $185 per hour. For a surgeon who trained for over a decade. Who carries the liability of surgical outcomes. Who runs a practice collecting $2.4 million a year.
+And here's what happens when you know that number. Every financial decision starts to have a time cost. That $96,000 in debt service? That's 519 hours of your clinical time. More than ten weeks of work, just servicing debt.
+The gap between what you think you earn and what you actually keep is where wealth disappears. And that gap has consequences.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The $185/hr figure is the emotional centerpiece of the episode and creates immediate dissonance against surgeon-level collections, making it the strongest possible cover frame anchor.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$185/hr" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "What $2.4M in collections actually pays you" in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: precise, revelatory, grounded. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: Primary: "$185/hr" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), centered upper-center of safe zone. Secondary: "What $2.4M in collections actually pays you" in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text with 20px spacing. Brand mark: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>week-4-clip-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>$30 More Per Hour, $1M More Per Career</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>The number that matters more than collections</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>This clip demonstrates that structural improvements to overhead, entity design, and retirement contributions can move the effective hourly rate by $30/hour, compounding to over $1M across a decade. It bridges the diagnosis (Clip 1) to the prescription, showing that the gap is fixable without working more hours.</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+A $30 per hour difference doesn't sound like much. Over 2,600 clinical hours, it's $78,000 a year.
+Here's what moves the needle. Reduce overhead from 55% to 51% through disciplined cost management. Optimize your S-Corp salary and entity structure to bring the effective tax rate from 40% down to 37%. Add a cash balance plan that shelters an additional $63,000 in tax-deferred contributions.
+The effective hourly rate goes from $185 to $215. $78,000 a year in additional take-home. Over a ten-year career horizon, with modest investment returns, that's over a million dollars in additional wealth.
+From the same collections, the same clinical hours, the same practice. The only thing that changed is the structure.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The $30/hour to $1M framing makes the structural improvement tangible and scroll-stopping by compressing a small-sounding change into a career-scale outcome.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$30/hr = $1M+" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Same collections. Same hours. Different structure." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: authoritative, optimistic, precise. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: Primary: "$30/hr = $1M+" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), centered upper-center of safe zone. Secondary: "Same collections. Same hours. Different structure." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text with 20px spacing. Brand mark: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>week-4-clip-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Your Real Hourly Rate in 15 Minutes</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>The number that matters more than collections</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>This clip converts the episode's concept into a hands-on exercise. The five-step walkthrough gives the viewer a concrete action they can take in 15 minutes, making this the highest-utility clip in the set and a strong fit for the longer Instagram Reels format.</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Here's how to calculate your real hourly rate in 15 minutes. Five steps. One number that changes everything.
+Step one: Take your Q1 collections and annualize them. If Q1 was $600,000, your annualized estimate is $2.4 million.
+Step two: Subtract your overhead. If you don't know your exact percentage, use 55% as a starting estimate for an orthopedic practice.
+Step three: From the surgeon income that remains, subtract your effective tax rate. If you're not sure, use 40%.
+Step four: Subtract your annual retirement contributions and your annual debt service.
+Step five: Divide what's left by your annual clinical hours. Use 2,400 to 2,600 as a reasonable range for full-time practice.
+Write the number down. Then ask yourself: is this higher or lower than what I assumed? And which lever (entity structure, salary calibration, or overhead) is most likely dragging it down?
+You can't improve what you haven't measured. It takes fifteen minutes.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The "5 steps / 15 minutes" framing promises a quick, tangible outcome, which drives saves and shares on Reels where actionable content outperforms opinion content.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "5 Steps. 15 Minutes." in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Calculate the number that changes everything" in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: instructional, empowering, clear. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: Primary: "5 Steps. 15 Minutes." in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), centered upper-center of safe zone. Secondary: "Calculate the number that changes everything" in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text with 20px spacing. Brand mark: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>week-4-clip-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Same Collections. $80K Gap. Here's Why.</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>The number that matters more than collections</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>This clip attacks the most common misconception in surgeon compensation: that collections equals earnings. The two-surgeon comparison makes the structural gap concrete and challenges the viewer to question their own assumptions, functioning as a top-of-funnel hook for the full episode.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Two surgeons, both collecting $2.4 million a year. Same specialty, similar case volume. One takes home $480K. The other takes home $560K. Same collections, $80,000 difference in what they keep.
+How? The difference sits in everything that happens between the top line and the bottom line. Overhead structure, entity design, tax strategy, retirement plan contributions, debt load.
+Those are the variables that determine your real compensation. Collections doesn't touch any of them.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The side-by-side comparison of identical collections with an $80K gap creates immediate cognitive tension, the strongest scroll-stop pattern for YouTube Shorts where the first frame determines whether a viewer stays.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$80,000 Gap" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Two surgeons. Same collections. Different structure." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: confrontational, precise, eye-opening. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: Primary: "$80,000 Gap" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), centered upper-center of safe zone. Secondary: "Two surgeons. Same collections. Different structure." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text with 20px spacing. Brand mark: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>week-4-clip-4.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 5 (MARCH 23–29)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="3" t="n"/>
+      <c r="E13" s="3" t="n"/>
+      <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>The $172,000 Gap Hiding in Your Retirement Line</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Isolates the retirement contribution gap from the full episode into a standalone clip. The $172K gap and $2M compounding consequence are scroll-stopping numbers that make the cost of inaction viscerally concrete for surgeons who assume their 401(k) deferral is "enough."</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+A surgeon contributed $31,000 to retirement last year. The available capacity was $203,000. That $172,000 gap compounds every single year.
+Here's what the full picture looks like. The 401(k) deferral is one layer. But with a cash balance plan layered on top, the total available capacity can reach $203,000 or more per year.
+At a marginal rate of roughly 40%, that $172,000 in additional contributions would have reduced the current-year tax bill by approximately $69,000.
+And the money doesn't disappear. It compounds tax-deferred. Over 10 years, that single structural change produces nearly $2 million in additional retirement wealth.
+The retirement contribution line is the loudest finding on most surgeon returns. The gap is sitting right there, in plain view, every single year.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The $172K gap is the clip's core shock number and must dominate the frame to stop the scroll and make surgeons question whether their own retirement line looks the same.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$172,000 Gap" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Your retirement line is the loudest finding on the return." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: urgent, clarifying, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$172,000 Gap" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "Your retirement line is the loudest finding on the return." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>week-5-clip-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Your Tax Rate Is 4 Points Too High. That's $500K.</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Isolates the effective tax rate diagnostic from the full episode. The 4.3-point gap and $500K decade cost translate an abstract percentage into a dollar figure that makes surgeons want to check their own returns immediately.</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Your effective tax rate should be between 30% and 33% at $800K. If it's 36% or higher, your structure is leaking $35K a year.
+For a surgeon earning $820,000 with an effective rate of 36.3%, the total tax bill is $298,000. At 32%, it would be $262,400. That's a difference of $35,600. Not a deduction. Not a credit. Just the mathematical consequence of having a more efficiently structured financial picture.
+If that gap persists, and it will if nothing changes structurally, you're looking at $350,000 to $400,000 in excess taxes over a decade. Invested at a reasonable return, that compounds to something considerably north of half a million dollars.
+The effective tax rate is the vital sign of your return.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The 36% vs. 32% comparison is a simple, immediately graspable contrast that belongs front and center to provoke the question "what's my rate?"
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "36% vs. 32%" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "That 4-point gap is costing you $35K a year." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: precise, sobering, clinical. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "36% vs. 32%" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "That 4-point gap is costing you $35K a year." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>week-5-clip-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Four Findings. Four Fixes. $156K a Year. Zero Extra Cases.</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>The treatment plan summary is the episode's capstone moment, compressing all four diagnostic findings into a single actionable frame. This clip works as both a standalone takeaway and a curiosity driver back to the full episode for listeners who want the math behind each line item.</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Four findings on a tax return. Four structural fixes. Combined impact: $120,000 to $156,000 per year. No additional OR time.
+Effective tax rate too high? Structural review, target 31% to 33%. That's $25,000 to $40,000. QBI deduction at zero? S-Corp salary recalibration. That's $11,000 to $17,000. Retirement contributions at $31,000 versus $203,000 available? Add a cash balance plan. That's $69,000 in current-year tax reduction. State tax at $52,000? Entity restructuring and income sourcing. That's $15,000 to $30,000.
+None of these require you to earn more money. None require additional OR time. Every single one is a structural adjustment to how the money you already earn flows through your financial life.
+And the only input required was reading the return.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The $120K-$156K combined impact is the clip's payoff number and must anchor the frame, while "Zero Extra Cases" delivers the contrarian hook that differentiates this from typical "earn more" advice.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$120K to $156K" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Four structural fixes. No additional OR time." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: decisive, empowering, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$120K to $156K" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "Four structural fixes. No additional OR time." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>week-5-clip-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Your QBI Deduction Is Zero. That's a Torn ACL on Your Return.</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>The QBI deduction is one of the most misunderstood lines on a surgeon's S-Corp return. This clip isolates the salary calibration insight into a standalone moment that speaks directly to S-Corp owners, using the ACL metaphor to bridge surgical thinking with financial diagnostics.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+Your QBI deduction is zero. That's the financial equivalent of an ACL that should be intact but isn't. One number on your S-Corp setup could save you $17,000 a year.
+Under current law, S-Corp owners can deduct up to 20% of their qualified business income. For surgeons running their practice through an S-Corp, this deduction is potentially worth tens of thousands of dollars.
+So why was it zero? The answer lives in how the S-Corp salary was calibrated. The more income that flows through as salary, the less qualifies for QBI.
+A salary in the range of $350,000 to $400,000, still reasonable and well within IRS guidelines, would have generated a QBI deduction of approximately $30,000 to $45,000.
+At the marginal rate, that's $11,000 to $17,000 in annual tax savings. From a single calibration adjustment.
+If your QBI deduction is zero and you run an S-Corp, that's a finding. It deserves a follow-up conversation with your advisor.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The "QBI = $0" stat paired with the surgical metaphor creates immediate pattern recognition for surgeon viewers and signals that this clip speaks their language.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "QBI Deduction: $0" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "One number on your S-Corp could save you $17,000 a year." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: diagnostic, direct, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "QBI Deduction: $0" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "One number on your S-Corp could save you $17,000 a year." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>week-5-clip-4.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Three Decisions, One Date, Zero Strategy</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta — filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Isolates the cold open framing from the full episode to reveal that April 15 bundles three distinct financial decisions most surgeons handle on autopilot. The "three decisions" hook reframes a familiar deadline as a strategic moment, earning the click to the full episode.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+April 15 has three decisions hidden inside it. Most surgeons see only one.
+Most surgeons think April 15 is about one thing: taxes. File or extend. Pay what you owe. Move on.
+But April 15 is actually three separate financial decisions compressed into one day. You're deciding whether to file or extend your return. You're deciding whether to make a prior-year IRA contribution, which for many of you means the backdoor Roth question. And you're making your Q1 estimated tax payment for 2026, which is either calibrated to your actual income trajectory or it's a guess based on last year's numbers.
+Three decisions. One date. And the way most surgeons handle it is: they deal with the filing, let their CPA autopilot the estimated payment, and either fund the Roth because they always have or skip it because they forgot.
+That's not a strategy. That's inertia dressed up as a deadline.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The "3 decisions, 1 date" framing is the clip's core tension and must dominate the cover to stop the scroll and provoke curiosity about which decisions the viewer is missing.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "3 Decisions. 1 Date." in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "Most surgeons only see one of them." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: precise, authoritative, clarifying. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "3 Decisions. 1 Date." in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "Most surgeons only see one of them." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>week-6-clip-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>The Backdoor Roth Math Just Changed</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta — filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Extracts the OBBBA-driven Roth recalculation from Segment 2, turning the most reflexive April 15 action into a deliberate analysis. The "paying 40% to avoid 24%" framing is a scroll-stopping inversion that challenges a deeply held default among high earners.</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+You've been funding a backdoor Roth every year because someone told you to. OBBBA changed the math. Here's why.
+The backdoor Roth has been the default recommendation for high-income earners for years. Pay taxes now, let the money grow tax-free, withdraw it in retirement with no taxes owed.
+But OBBBA made the 37% top marginal rate permanent. Before that, there was an argument that rates might revert to 39.6% or higher, which made paying 37% now look like a bargain. That argument is substantially weaker today.
+If you're paying a combined rate of 40% or more going in, and your retirement rate drops to 22% to 24%, you paid 40% for the privilege of not paying 24% on the way out.
+Compare that to redirecting the same $7,500 into a cash balance plan increase. The full amount goes in pre-tax, saving you $3,150 in taxes immediately.
+April 15 should trigger a deliberate analysis, not a reflexive deposit.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The tax rate contrast (40% in vs. 24% out) is the clip's core provocation and must be the dominant visual to force the viewer to question a long-held assumption.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "40% In. 24% Out." in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "The backdoor Roth math just changed." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: provocative, analytical, clarifying. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "40% In. 24% Out." in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "The backdoor Roth math just changed." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>week-6-clip-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="120" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>The $100 Trade That Buys You Six Months</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta — filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Short-Form Clip (YouTube Shorts / Instagram Reels)</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Reframes the filing extension from procrastination to strategic advantage. The $100 forgone-interest calculation gives surgeons a concrete, low-stakes number that neutralizes the guilt of not filing by April 15, while opening a six-month planning window most never consider.</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>## Content
+### Caption Script
+The extension isn't procrastination. More than half of high-income taxpayers file extensions. Here's why it might be the smarter move.
+If you have K-1 income from partnerships, surgical centers, or real estate investments, those K-1s frequently arrive late. Filing before they're in means filing an incomplete return and then amending later. More work, more cost, more headache than extending in the first place.
+If your financial picture changed significantly last year (new practice, sold a piece of a surgery center, changed entity structures), an extension gives your CPA and your advisor time to model the return correctly rather than rushing under deadline pressure.
+And here's the one most surgeons don't consider: if you're evaluating major financial moves for this year (establishing a cash balance plan, recalibrating your S-Corp salary), the extension window gives you six months to make those decisions with better information.
+The cost of overpaying by $5,000 for six months? At the current fed funds rate, you're forgoing roughly $100 in interest. That's the price of getting your return right.
+I'll take that trade every time.
+### On-Screen Captions
+Captions required. Clean, readable style. No stylized or animated text.</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Cover Frame
+Image type: Short-form clip cover frame
+Rationale: The $100 figure is the clip's permission-granting data point and must anchor the cover to immediately reframe extensions as a smart trade rather than a failure.
+AI image prompt: Create a 1080x1920px vertical short-form clip cover frame. Background: solid Deep Muted Blue (#243A4B). Layout: text centered within center 4:5 safe zone (top and bottom 10% kept clear of critical content). Primary text: "$100 for 6 Months" in Playfair Display SemiBold, approximately 72pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper-center of the safe zone. Secondary text: "The extension isn't procrastination. It's a trade." in Inter Regular, approximately 36pt, Off-White (#F6F7F5), centered, below primary text with 20px spacing. A thin horizontal accent line (2px, Antique Gold #B08D57) spans 50% of the canvas width, centered, between text blocks. Bottom of safe zone: "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered. No cartoons, no clip art, no stock photography, no clickbait styling. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reassuring, strategic, confident. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$100 for 6 Months" in Playfair Display SemiBold, ~72pt, Antique Gold (#B08D57), upper-center of safe zone. "The extension isn't procrastination. It's a trade." in Inter Regular, ~36pt, Off-White (#F6F7F5), centered below primary text. "CAPABLE WEALTH" in Inter Medium, 20pt, Blue Slate (#5F7483), centered at bottom of safe zone.
+Platform and dimensions: YouTube Shorts / Instagram Reels, 1080x1920</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>week-6-clip-3.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2322,6 +2820,1228 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
+          <t>CMS Cut Your Reimbursement by 2.5%. Your Financial Advisor Probably Didn't Mention It.</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Reimbursement Shift and Practice Wealth</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Opens the week's LinkedIn sequence by reframing the CMS 2.5% efficiency adjustment as a financial planning event rather than a practice management issue. Drives curiosity and positions Capable Wealth as the advisor who connects practice economics to personal wealth.</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>CMS cut your reimbursement by 2.5%. Your practice manager told you. Your financial advisor probably didn't.
+That gap matters.
+The 2.5% efficiency adjustment on non-time-based orthopedic codes has been active since January 1. If you perform 400 procedures a year at an average reimbursement of $3,200, the math is simple: $80 less per procedure, $32,000 less per year.
+Your practice manager sees a billing issue. Your accountant will see it in your year-end numbers. But the question nobody seems to be asking is what $32,000 in reduced revenue means for your retirement contributions, your tax positioning, and the long-term trajectory of your personal wealth.
+A reimbursement cut is a financial planning event. Every dollar your practice earns just became more valuable, which means how those dollars flow from your entity to your personal balance sheet matters more than it did six months ago.
+If your S-Corp salary hasn't been recalibrated since revenues dropped, you may be compounding the loss. If your retirement plan contributions haven't been reexamined in light of reduced income, you could be leaving additional tax-deferred growth on the table.
+The surgeons who absorb this cut without feeling it are the ones whose financial structure was already built for efficiency. The ones who feel it most are the ones who were already running at the margin.
+Which side of that line are you on?</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The 2.5% number is the post's anchor data point and creates immediate recognition for any surgeon who has seen it in their Q1 statements. A bold stat card makes the number impossible to scroll past.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "2.5%" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper third of the canvas. Secondary text: "Your practice manager told you." in Inter Regular, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 32px below the primary text. Tertiary text: "Your financial advisor probably didn't." in Inter SemiBold, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 16px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: urgent, authoritative, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "2.5%" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), upper third center. "Your practice manager told you." in Inter Regular, ~22pt, Off-White (#F6F7F5), below primary. "Your financial advisor probably didn't." in Inter SemiBold, ~22pt, Off-White (#F6F7F5), below secondary.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>week-3-linkedin-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Adding 10 Procedures to Offset a $32K Loss Sounds Logical. Here's Why It Costs You More Than It Recovers.</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Reimbursement Shift and Practice Wealth</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Builds on Post 1 by challenging the instinctive "do more procedures" response to reimbursement cuts. Uses marginal cost math to show that volume increases are the most expensive way to recover lost revenue, and introduces structural optimization as the more efficient alternative.</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Adding 10 procedures to offset a $32K revenue loss sounds logical. Here's why it costs you more than it recovers.
+The CMS 2.5% efficiency adjustment reduced your average reimbursement by about $80 per procedure. At 400 procedures a year, that's $32,000 in lost revenue.
+The instinctive response: add 10 cases at $3,200 each to close the gap.
+But each additional procedure carries marginal costs that your existing caseload has already absorbed. OR time, anesthesia, supplies, implants, staff hours. At the margin, those costs consume roughly 60% of the revenue from each extra case.
+Here's how it actually plays out:
+→ 10 additional procedures: $32,000 gross revenue
+→ Marginal costs at 60%: $19,200
+→ Net recovery: $12,800
+→ Additional OR time: 30 to 40 hours
+You just spent a month's worth of extra surgical hours to recover 40 cents on every dollar you lost.
+Now compare that to structural optimization. A 2% reduction in practice overhead (on a $1.6M practice) saves $32,000 directly. No additional procedures. No additional OR time. No additional marginal costs. Dollar-for-dollar recovery.
+Working harder recovers 40 cents on the dollar. Reducing overhead by 2% recovers 100 cents.
+At surgeon-level income, your time is the most expensive input you have. Before adding cases to the schedule, it's worth asking: is there a way to recover this revenue without spending more of it?</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The 40-cents-on-the-dollar recovery figure is the post's most memorable data point. Isolating it as a stat card creates a scannable, shareable visual that captures the core argument without requiring the reader to process the full math.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "40¢" in Playfair Display SemiBold, approximately 108pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "recovered per dollar lost" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "when you add procedures to offset a cut" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: precise, authoritative, thought-provoking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "40¢" in Playfair Display SemiBold, ~108pt, Antique Gold (#B08D57), center. "recovered per dollar lost" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "when you add procedures to offset a cut" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below secondary.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>week-3-linkedin-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>OBBBA Tied Medicare Physician Payments to 75% of the MEI. Here's What That Number Means in Your Pocket.</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Reimbursement Shift and Practice Wealth</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Zooms out from the immediate 2.5% cut to the broader legislative context. The One Big Beautiful Bill Act (OBBBA) pegged Medicare physician payment updates to 75% of the Medicare Economic Index, creating a permanent structural gap between rising practice costs and reimbursement growth. This post frames the shift as long-term and structural, requiring a financial response beyond single-year adjustments.</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>OBBBA tied Medicare physician payments to 75% of the Medicare Economic Index in 2026. Here's what that number means in your pocket.
+The Medicare Economic Index tracks how much it actually costs to run a medical practice: staff wages, rent, malpractice, supplies, everything. When those costs go up 4%, the MEI reflects that increase.
+Before OBBBA, physician payment updates were set year by year through temporary legislative patches, usually at or near 0%. The new law replaced that system with an automatic annual update tied to 75% of the MEI.
+On the surface, that sounds like progress. And compared to a decade of flat or negative updates, it is.
+But 75% is a permanent structural gap. If your practice costs rise 4%, your Medicare reimbursement rises 3%. Every year, the difference compounds. Over five years, that gap between costs and reimbursement becomes meaningful. Over ten years, it reshapes practice economics.
+For a surgeon collecting $1.6M annually with 40% of revenue from Medicare, even a 1% annual gap means roughly $6,400 in lost ground per year. That's not dramatic in year one. By year five, the cumulative shortfall is over $30,000. By year ten, it's approaching $70,000.
+This is the important part: a structural shift requires a structural response. Adjusting your surgical schedule year by year won't close a gap that's built into the payment formula itself.
+What will close it: reducing overhead systematically, optimizing how your income flows from the practice to your personal wealth, and building a financial structure that doesn't depend on reimbursement growth to function.
+The payment formula changed. Has your financial plan?</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The 75% figure is the post's central data point and captures the structural gap in a single number. Presenting it as a bold stat card creates immediate visual impact and makes the legislative change feel concrete rather than abstract.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "75%" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "of cost increases covered" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "Medicare physician payment update, 2026 forward" in Inter Regular, approximately 15pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: clear, sobering, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "75%" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), center. "of cost increases covered" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "Medicare physician payment update, 2026 forward" in Inter Regular, ~15pt, Warm Gray (#9AA3A8), below secondary.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>week-3-linkedin-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Three Overhead Line Items Most Practices Never Benchmark</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Reimbursement Shift and Practice Wealth</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Extends the week's reimbursement theme into actionable territory. Posts 1 through 3 established why structural optimization matters more than volume increases. This post gives surgeons three specific overhead categories to examine, making the "2% overhead reduction" concept from the anchor blog concrete and immediately actionable.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Most orthopedic practices track revenue closely. Far fewer benchmark the three overhead categories that determine how much of that revenue the surgeon actually keeps.
+If a 2.5% reimbursement cut costs your practice $32,000 a year, and a 2% overhead reduction recovers the same $32,000 with zero additional procedures, the question becomes: where does that 2% come from?
+When you analyze orthopedic practice overhead, there are three line items that almost always have room:
+→ Supply and vendor contracts. When was the last time your practice benchmarked implant pricing, surgical supplies, and office materials against peer practices? Most practices haven't renegotiated in years. A 5% reduction in supply costs alone can recover $10,000 to $20,000 annually.
+→ Staffing ratios. And I want to be clear: this is not about cutting staff. Practices that have grown over time often carry staffing structures built for an earlier version of the practice. Aligning roles, scheduling workflows, and staffing ratios with current patient volume can reduce overhead 1% to 3% without reducing quality of care.
+→ Facility utilization. If you own your space or hold a long-term lease, unused operatory time, underutilized square footage, and energy costs add up quietly. For surgeon-owned buildings, a cost segregation study can also accelerate depreciation deductions on top of the overhead savings.
+None of these require adding a single case to your schedule. All three are within your control.
+The reimbursement environment is tightening. The practices that absorb it best are the ones that know exactly where their overhead sits relative to their peers.
+When was the last time your practice ran that comparison?</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: A clean card listing the three benchmark categories creates a scannable, saveable reference that surgeons can screenshot or forward to their practice manager. The list format matches the post's actionable, checklist-style tone.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: left-aligned text composition with generous margins (120px top and bottom, 100px left, 80px right). Header text: "3 line items to benchmark" in Playfair Display SemiBold, approximately 36pt, Off-White (#F6F7F5), left-aligned, positioned in the upper quarter of the canvas. A thin horizontal rule (1px, Antique Gold #B08D57) spans 50% of the canvas width, left-aligned with the header text, positioned 24px below the header. Three list items below the rule, each in Inter Medium, approximately 22pt, Off-White (#F6F7F5), left-aligned, with 36px vertical spacing between items. Item 1: "Supply &amp; vendor contracts". Item 2: "Staffing ratios". Item 3: "Facility utilization". A small square bullet (6px, Antique Gold #B08D57) precedes each item with 16px horizontal spacing. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: actionable, organized, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "3 line items to benchmark" in Playfair Display SemiBold, ~36pt, Off-White (#F6F7F5), upper quarter left. Three list items in Inter Medium, ~22pt, Off-White (#F6F7F5), with Antique Gold (#B08D57) bullet squares.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>week-3-linkedin-4.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Is Your Practice Structured to Build Wealth, or Just to Generate Revenue?</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Reimbursement Shift and Practice Wealth</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Closes the week's LinkedIn sequence with a reflective, strategic-level post that ties the reimbursement theme back to the broader Q2 arc. Connects Week 3's external pressure (reimbursement cuts) to Weeks 1 and 2's internal structural gaps (entity structure, S-Corp salary, retirement plans), reinforcing the cumulative argument that financial structure determines how much of what you earn you actually keep.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>There is a question worth asking every surgeon who owns a practice. It tends to land quietly, and then it stays with them.
+Is your practice structured to build wealth, or just to generate revenue?
+Because those are two very different things.
+A practice that generates revenue puts money through the door. A practice that builds wealth makes sure the surgeon keeps as much of it as possible, in the most tax-efficient way, through the most intentional structure.
+Over the past few weeks, we've looked at what happens when that structure has gaps. An S-Corp salary that hasn't been recalibrated in years can cost you $25,000 annually in misallocated self-employment tax. A missing cash balance plan leaves $45,000 to $80,000 per year in tax-deferred growth on the table. And now, a 2.5% reimbursement cut takes another $32,000 off the top.
+These are not separate problems. They compound. A surgeon earning $800,000 with all three gaps is losing over $100,000 a year to structural inefficiency. Over a decade, that's a seven-figure difference in personal wealth.
+And every one of those gaps is fixable. The S-Corp salary is adjustable. The cash balance plan can be established this year. The overhead can be benchmarked and reduced. The reimbursement cut, the one thing you can't control, becomes the smallest variable in the equation once the structure is right.
+You spent years building a practice that generates excellent revenue. The question worth sitting with is whether that practice is also structured to turn that revenue into lasting wealth.</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The central question of the post works as a bold typographic statement that prompts self-reflection. Presenting it as a clean quote-style card creates a thumb-stopping moment in the feed and invites engagement.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "Revenue is what you bill." in Playfair Display Regular, approximately 32pt, Off-White (#F6F7F5), centered horizontally, positioned above the vertical center of the canvas. Secondary text: "Wealth is what you keep." in Playfair Display SemiBold, approximately 38pt, Antique Gold (#B08D57), centered horizontally, positioned 28px below the primary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, positioned 48px below the secondary text. Tertiary text: "Are you structured for both?" in Inter Regular, approximately 18pt, Warm Gray (#9AA3A8), centered horizontally, positioned 24px below the rule. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: reflective, composed, forward-looking. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Revenue is what you bill." in Playfair Display Regular, ~32pt, Off-White (#F6F7F5), above center. "Wealth is what you keep." in Playfair Display SemiBold, ~38pt, Antique Gold (#B08D57), below primary. "Are you structured for both?" in Inter Regular, ~18pt, Warm Gray (#9AA3A8), below rule.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>week-3-linkedin-5.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 4 (MARCH 16–22)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="120" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Your Effective Hourly Rate Is the Number That Actually Matters</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>The Number That Matters More Than Collections</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Introduces the "surgeon effective hourly rate" concept as the true measure of financial health. Anchors the week's theme by contrasting collections (a practice metric) with effective hourly rate (a personal wealth metric), using real math to make the gap visceral.</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Your practice collected $2.4M last year. You kept $480K. Your effective hourly rate? $185.
+That number surprises most surgeons when they see it for the first time. And it should.
+Collections measure practice health. They tell you the business is generating revenue, the billing team is performing, and payers are reimbursing. Those are all good things to know.
+But collections don't tell you what you actually kept. And they definitely don't tell you what each hour of your time was worth after overhead, taxes, debt service, and retirement contributions came out.
+Here's the math on a $2.4M practice:
+→ 55% overhead: $1,320,000 gone before you see a dollar
+→ Federal and state taxes on the remainder
+→ Student loan payments, if applicable
+→ Retirement contributions (assuming you're maxing them)
+→ What's left: roughly $480,000
+Divide that by 2,600 clinical and administrative hours per year. You land at $185/hr.
+That's your effective hourly rate. The number that tells you what your time is actually producing for your family's wealth.
+Most surgeons have calculated their collections per case, their RVUs per quarter, their overhead percentage. Almost none have calculated this number. And yet this is the one that determines whether you're building wealth or just building a practice.
+If you've never run this calculation, this is the week to do it. The gap between what you collect and what you keep is where the real planning starts.</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The stark contrast between $2.4M collections and $185/hr effective rate creates immediate cognitive dissonance, which drives engagement. A clean stat card communicates the math at a glance and stops the scroll.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: vertically stacked text composition, centered horizontally with 80px side margins. Top section (upper 40%): "$2.4M collected" in Inter Regular, approximately 36pt, Warm Gray (#9AA3A8), centered, positioned at roughly 30% from top. A thin horizontal divider line (2px, Blue Slate #5F7483, 60% canvas width) separates the top and bottom sections, centered vertically. Bottom section (lower 40%): "$185/hr kept" in Playfair Display SemiBold, approximately 56pt, Antique Gold (#B08D57), centered, positioned at roughly 65% from top. Subtle thin-line downward arrow icon (Antique Gold #B08D57, 2px stroke) between the two text blocks, centered, approximately 40px tall. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: contemplative, precise, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "$2.4M collected" in Inter Regular, ~36pt, Warm Gray (#9AA3A8), upper center. "$185/hr kept" in Playfair Display SemiBold, ~56pt, Antique Gold (#B08D57), lower center.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>week-4-linkedin-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>As Q1 Wraps Up, Ask About Your Keep Rate Before Anything Else.</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>The Number That Matters More Than Collections</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Ties the effective hourly rate concept to the upcoming Q1 close, making the post timely and actionable. Introduces "keep rate" as a digestible metric surgeons can track quarterly. Positions revenue growth without structural improvement as a warning sign, not a celebration.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Q1 is wrapping up. When your revenue data lands, before you celebrate (or panic), ask this: did your keep rate go up or down?
+Keep rate is simple. It's the percentage of gross revenue that actually flows to your personal wealth after overhead, taxes, debt service, and savings. If your practice collected $600K in Q1 and you kept $120K, your keep rate is 20%.
+Here's why this matters more than the top-line number.
+This is a structural pattern that shows up frequently in surgeon-owned practices: a practice grows revenue by 8% year over year, the surgeon feels good about the trajectory, but overhead crept up by 10%. Taxes increased because the additional income pushed into a higher marginal bracket. And the retirement plan wasn't restructured to capture the growth.
+The result? Revenue went up. Keep rate went down. The practice got busier and more profitable on paper, and the surgeon's personal wealth-building actually slowed.
+Revenue growth without structural improvement means the practice generates more income for everyone except you. More for overhead. More for the IRS. More for lenders. The surgeon works harder, and the gap between collections and kept income widens.
+Your Q1 vital sign isn't revenue growth. It's keep rate direction.
+If revenue grew and keep rate grew with it, your structure is working. If revenue grew and keep rate stayed flat or declined, that's the signal to look under the hood before Q2 begins.
+One number. One question. That's your Q1 financial check-up when the numbers come in.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The question-driven format creates engagement by prompting self-reflection. A simple keep rate metric on the card gives surgeons a framework they can apply when their Q1 data comes in.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with 80px side margins. Upper third: "Q1 Keep Rate" in Inter Medium, approximately 28pt, Warm Gray (#9AA3A8), centered, positioned at roughly 28% from top. Center: a large upward or downward arrow icon composed of two versions side by side (one pointing up in Antique Gold #B08D57, one pointing down in Blue Slate #5F7483), each approximately 80px tall, separated by 40px, centered horizontally at 50% vertical. Lower third: "Which direction is yours?" in Playfair Display SemiBold, approximately 40pt, Off-White (#F6F7F5), centered, positioned at roughly 72% from top. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, direct, serious. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Q1 Keep Rate" in Inter Medium, ~28pt, Warm Gray (#9AA3A8), upper center. "Which direction is yours?" in Playfair Display SemiBold, ~40pt, Off-White (#F6F7F5), lower center.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>week-4-linkedin-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>The Five Components of Your Effective Hourly Rate</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>The Number That Matters More Than Collections</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Framework post that breaks the effective hourly rate into five actionable components. Gives surgeons a mental model for understanding which variables they can influence, shifting the conversation from "I need to earn more" to "I need to optimize what flows through." Supports the anchor blog's core math.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Your effective hourly rate has five components. You can influence four of them.
+Here's what sits between your gross collections and what each hour of your time actually produces:
+→ Gross Revenue: the total your practice collects. Largely driven by case volume, payer mix, and reimbursement rates. You have some control here, but the ceiling is set by how many hours you're willing to work.
+→ Overhead: the operating cost of the practice. Staffing, supplies, rent, insurance, billing. For most orthopedic practices, this runs between 50% and 60%. Even a 3-point reduction on $2.4M in collections frees up $72,000.
+→ Taxes: federal, state, self-employment, and payroll. This is where entity structure, S-Corp salary optimization, and deduction strategies make their biggest impact. The spread between a poorly structured and well-structured surgeon at the same income level can be $40,000 or more.
+→ Debt Service: student loans, practice acquisition debt, equipment financing. The interest rate, repayment timeline, and tax treatment of this debt all affect your hourly rate. Refinancing or restructuring can move the needle meaningfully.
+→ Retirement Savings: the money you're setting aside for future wealth. This is the one component where spending more actually improves your long-term hourly rate. Maximizing tax-deferred vehicles (401(k), cash balance plans) reduces your current tax burden and compounds over decades.
+The key insight: most surgeons try to improve their rate by increasing the first component. Working more hours, adding cases, negotiating higher rates. But the largest opportunity usually lives in components two through five, the structural side of the equation.</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: A clean numbered list on a card format makes the five components instantly scannable and shareable. The visual framework reinforces the teaching structure and gives surgeons a reference they'll return to.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: left-aligned text composition with 80px left margin and 80px right margin. Top section: "Your Effective Hourly Rate" in Playfair Display SemiBold, approximately 36pt, Off-White (#F6F7F5), left-aligned, positioned at roughly 15% from top. Below the title (starting at roughly 30% from top), five lines of text stacked vertically with 36px spacing between each line: "1. Gross Revenue" in Inter Medium, 24pt, Antique Gold (#B08D57). "2. Overhead" in Inter Medium, 24pt, Off-White (#F6F7F5). "3. Taxes" in Inter Medium, 24pt, Off-White (#F6F7F5). "4. Debt Service" in Inter Medium, 24pt, Off-White (#F6F7F5). "5. Retirement Savings" in Inter Medium, 24pt, Off-White (#F6F7F5). A thin vertical accent line (3px, Antique Gold #B08D57) runs along the left edge from the first item to the last item, positioned at 60px from the left edge. Bottom: "Which ones can you move?" in Inter Regular, 20pt, Warm Gray (#9AA3A8), left-aligned, positioned at roughly 85% from top. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: structured, educational, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Your Effective Hourly Rate" in Playfair Display SemiBold, ~36pt, Off-White (#F6F7F5), top left. Five numbered items in Inter Medium, ~24pt, stacked vertically. "Which ones can you move?" in Inter Regular, ~20pt, Warm Gray (#9AA3A8), bottom left.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>week-4-linkedin-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>From $185 to $215 Per Hour Without Adding a Single Case</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>The Number That Matters More Than Collections</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Connects the entire March content arc (entity structure, S-Corp salary, reimbursement response, effective hourly rate) into a single proof of concept. Shows that the $30/hr improvement ($78K/year) comes from structural changes discussed over the prior three weeks, reinforcing that structure, not effort, drives the gap.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>$185 per hour to $215 per hour. Same collections. Same hours. Same number of cases.
+The difference? $78,000 per year. And it comes entirely from structural improvements, not from working harder or seeing more patients.
+Over the past month, I've been walking through the specific changes that move this number. Here's how they add up for a surgeon collecting $2.4M annually:
+→ Entity structure optimization (proper S-Corp election, clean entity separation): reduces self-employment tax exposure and opens planning flexibility. Typical impact: $15,000 to $25,000.
+→ S-Corp salary calibration (setting reasonable compensation at the right level, not just the level your CPA defaulted to years ago): balances payroll tax savings against retirement contribution capacity and QBI deduction. Typical impact: $10,000 to $20,000.
+→ Proactive reimbursement response (restructuring overhead and revenue mix when payer rates shift): protects margins before they erode. Typical impact: $15,000 to $30,000 in preserved income.
+→ Retirement plan maximization (adding or optimizing a cash balance plan on top of a 401(k)): converts current taxable income into tax-deferred compounding. Typical impact: $20,000 to $40,000 in annual tax savings.
+None of these require you to operate on one more patient. None require a longer workday. They require a coordinated financial structure that's designed for surgeon-level income.
+The move from $185 to $215 per hour is a structural outcome. And it's available to most practice-owning orthopedic surgeons who haven't had this conversation yet.</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The before/after hourly rate comparison creates a clear visual payoff for the month's content arc. The $78K annual difference translates the per-hour improvement into a number that commands attention.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered composition with 80px side margins. Upper section (roughly 25% from top): "Same hours. Same cases." in Inter Regular, approximately 24pt, Warm Gray (#9AA3A8), centered. Center section: two large numbers side by side, separated by a rightward-pointing arrow. Left number: "$185/hr" in Playfair Display SemiBold, approximately 48pt, Blue Slate (#5F7483), positioned at roughly 40% from left, vertically centered. Right arrow: a simple rightward arrow (→) in Antique Gold (#B08D57), approximately 36pt, centered between the two numbers. Right number: "$215/hr" in Playfair Display SemiBold, approximately 48pt, Antique Gold (#B08D57), positioned at roughly 65% from left, vertically centered. Lower section (roughly 75% from top): "+$78,000/year" in Inter SemiBold, approximately 32pt, Off-White (#F6F7F5), centered. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: confident, precise, compelling. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Same hours. Same cases." in Inter Regular, ~24pt, Warm Gray (#9AA3A8), upper center. "$185/hr → $215/hr" in Playfair Display SemiBold, ~48pt, center. "+$78,000/year" in Inter SemiBold, ~32pt, Off-White (#F6F7F5), lower center.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>week-4-linkedin-4.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Week 4 (March 16–22)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Four Weeks, One Message: Structure Determines What You Keep</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>The Number That Matters More Than Collections</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>End-of-month synthesis post that wraps the entire March Q1 Financial Health Check arc into a single philosophical takeaway. Provides narrative closure across all four weeks while creating a soft, natural bridge toward a coordinated review before the April 15 tax deadline.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Four weeks. Four topics. One message.
+In the first week of March, we looked at entity structure: why the way your practice is organized determines your tax exposure, your liability protection, and your ability to build wealth through the business.
+In week two, we examined S-Corp salary calibration: the single number inside your entity that interacts with self-employment tax, retirement contributions, and the QBI deduction simultaneously.
+In week three, we addressed reimbursement cuts: how to respond structurally when payer rates decline, rather than simply absorbing the hit or working more hours to compensate.
+And this week, we put a number on all of it. Your effective hourly rate. The figure that tells you what each hour of your professional life actually produces for your family's wealth. For many surgeons, the structural improvements from weeks one through three move that rate from $185 to $215 per hour. That's $78,000 per year, with no additional cases and no longer days.
+The thread connecting all four weeks is simple: structure determines what you keep.
+You can't out-earn a broken structure. You can't out-save it either. At surgeon-level income, the difference between a well-designed financial structure and one that was never coordinated is six figures per year. Every year.
+April 15 is three weeks away. If you haven't looked at your entity, your salary, your retirement plan, and your effective hourly rate as a connected system, this is the window. A coordinated review before tax season closes can set the structure for the rest of the year.
+The work you put into your craft deserves a financial structure that matches.</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: A clean typographic card with the arc's core message serves as a capstone visual for the month. The philosophical framing elevates the post beyond tactical advice and gives it lasting shareability.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B) covering the full canvas. Layout: centered text composition with 100px side margins. Single block of text vertically centered on the canvas: "Structure determines what you keep." in Playfair Display SemiBold, approximately 44pt, Off-White (#F6F7F5), centered horizontally, line-broken naturally if needed for balance. A thin horizontal accent line (2px, Antique Gold #B08D57, approximately 120px wide) centered below the text with 24px spacing. Below the accent line: "Q1 Financial Health Check" in Inter Regular, approximately 18pt, Warm Gray (#9AA3A8), centered, with 16px spacing from the line. Small "CAPABLE WEALTH" wordmark in Inter Medium, approximately 12pt, Blue Slate (#5F7483), centered at the bottom of the canvas with 60px bottom margin. No photographs, no illustrations, no clip art, no stock imagery. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. Mood: reflective, authoritative, calm. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "Structure determines what you keep." in Playfair Display SemiBold, ~44pt, Off-White (#F6F7F5), centered. "Q1 Financial Health Check" in Inter Regular, ~18pt, Warm Gray (#9AA3A8), below accent line. "CAPABLE WEALTH" in Inter Medium, ~12pt, Blue Slate (#5F7483), bottom center.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>week-4-linkedin-5.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 5 (MARCH 23–29)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Your Tax Return Is a 30-Page Diagnostic Report. Nobody Read It for Strategy.</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Leads into April's "Post-Filing Insights" month by reframing the tax return from a compliance document into a strategic diagnostic. Compresses the anchor blog's four-marker framework into a single, actionable LinkedIn post that positions the return as the most underread financial document a surgeon owns.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a 30-page diagnostic report. Your CPA read it for compliance. Nobody read it for strategy.
+That is a problem worth fixing.
+Buried in those pages are four line items that tell you whether your financial structure is working or leaking. Your effective tax rate reveals whether you are actually paying what you think you are paying, or something significantly more. Your QBI deduction shows whether your S-Corp salary is calibrated correctly. Your retirement contributions tell you how much of your available tax-sheltered capacity you are using. And your state tax line tells you whether your entity geography is costing you money.
+For a surgeon earning $900,000, the spread between a well-structured return and a poorly structured one can exceed $120,000 in a single year. That is the difference between a return that was filed and a return that was read.
+Most CPAs are excellent at making sure you file correctly and on time. That is their job. But the question of whether your return reflects a financial structure that is actually optimized for your income, your practice, and your goals requires a different lens.
+Your return already has the answers. The question is whether anyone is asking the right questions of it.
+If you filed in the past two weeks, pull it back out. Look at those four lines. What do they tell you?</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The "30-page diagnostic report" framing is the post's central reframe. Presenting it as a bold typographic statement creates an immediate pattern interrupt for any surgeon scrolling past tax season content.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "30 Pages" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned in the upper third of the canvas. Secondary text: "Your CPA read it for compliance." in Inter Regular, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 32px below the primary text. Tertiary text: "Nobody read it for strategy." in Inter SemiBold, approximately 22pt, Off-White (#F6F7F5), centered horizontally, positioned 16px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 30% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: authoritative, provocative, clean. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "30 Pages" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), upper third center. "Your CPA read it for compliance." in Inter Regular, ~22pt, Off-White (#F6F7F5), below primary. "Nobody read it for strategy." in Inter SemiBold, ~22pt, Off-White (#F6F7F5), below secondary.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>week-5-linkedin-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>A Surgeon's Return Showed $31,000 in Retirement Contributions. The Available Capacity Was $203,000.</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Isolates the most visceral diagnostic marker from the anchor's four-line framework: the retirement contribution gap. Lets the numbers speak directly and positions the tax return as the document that exposes how much tax-sheltered capacity a surgeon is leaving unused every year.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>A surgeon's return showed $31,000 in retirement contributions. The available capacity was $203,000. That $172,000 gap compounds every single year.
+Here is what that gap looks like in practice.
+A 401(k) with catch-up contributions for a surgeon over 50 allows $32,500 annually. Add a profit-sharing layer through an S-Corp, and you reach roughly $70,000. Layer in a cash balance plan, and the total available capacity can push past $200,000 in a single year, all tax-deferred.
+Most surgeons at this income level are using the 401(k) only. Some are maxing the employee contribution. Very few are using the profit-sharing component at all. Almost none have a cash balance plan in place.
+The result shows up on one line of the return: retirement plan contributions. And when that line reads $31,000 instead of $203,000, you are looking at the single largest structural gap in most surgical practices.
+This is not about being irresponsible. The surgeon in this example was disciplined, productive, and well-compensated. But the plan structure underneath was never built for an income at this level. A 401(k) designed for a $150,000 earner does not do the same work for someone earning $900,000.
+The tax return is where this shows up most clearly. One line. One number. And a gap that, over a decade, costs more than most people's houses.
+What does your retirement contribution line say?</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Conceptual photograph (photorealistic, people)
+Rationale: The $172,000 retirement gap is fundamentally about a surgeon who doesn't realize the capacity available to them. A photorealistic image of a senior surgeon reviewing financial documents creates an immediate sense of "that could be me" and grounds the abstract gap in a concrete, relatable moment.
+AI image prompt: Create a 1080x1080px square photorealistic image. A male surgeon in his late 50s, wearing a tailored charcoal sport coat over a white open-collar dress shirt, seated at a clean modern walnut desk. He is reviewing a multi-page printed financial document, one hand resting on the pages, the other holding a pair of reading glasses. The setting is a private office with a large window behind and to the right, soft late-afternoon natural light illuminating the desk surface and the side of his face. Background softly out of focus: a few books on a minimal shelf, neutral gray wall. His expression is thoughtful and focused, slightly furrowed brow, as if discovering something unexpected in the numbers. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field, sharp focus on his hands and the document. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no handshakes, no stethoscope on money). Mood: sobering, precise, introspective. Photorealistic editorial photography style suitable for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>week-5-linkedin-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>The Extension Isn't Procrastination. It's a Strategy, If You Use It Right.</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Extends the anchor's "return as diagnostic" message to surgeons who haven't filed yet. Reframes the extension from a sign of disorganization into the most valuable planning window of the year, creating a bridge between the April 15 deadline and the October 15 opportunity.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>The extension isn't procrastination. It's a strategy, if you use it right.
+More than half of high-income taxpayers file extensions every year. There is a reason for that, and it has nothing to do with being behind.
+The six months between April 15 and October 15 represent the most valuable planning window on the tax calendar. During that period, you can finalize retirement plan contributions, restructure entity elections, establish or fund a cash balance plan, and make S-Corp salary adjustments that affect your current-year return.
+For a surgeon earning $1.2M, the planning decisions available during the extension period can shift the tax outcome by $40,000 to $80,000. That is not a rounding error. That is the difference between a return that was filed and a return that was optimized.
+The catch is that most people treat the extension as extra time to gather documents. They file the extension in April, put the return out of mind, and scramble again in September. The six-month window closes without a single strategic decision being made.
+Used correctly, the extension period is when you sit down with your return (or last year's return, if this year's is still being prepared), identify the four diagnostic markers, and build a plan to close any structural gaps before October.
+If you're planning to file an extension, or if you've already filed one, you are not behind. You are in the strongest planning position of the calendar. The question is whether you will use the time.
+What is one decision you could make before October 15 that would change next year's return?</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Simple infographic
+Rationale: The six-month planning window from April to October is a timeline-driven insight that benefits from a clean visual timeline rather than static text. A branded horizontal timeline shows the extension period as a deliberate strategic runway, making the abstract "six months" feel concrete and structured.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (100px all sides). A horizontal timeline runs across the center of the canvas from left to right. Left endpoint: a small filled circle (12px, Deep Muted Blue #243A4B) with the label "April 15" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), positioned above the circle. Right endpoint: a small filled circle (12px, Antique Gold #B08D57) with the label "October 15" in Inter SemiBold, 16pt, Antique Gold (#B08D57), positioned above the circle. The timeline bar connecting them: 3px, Blue Slate (#5F7483). Three evenly spaced milestone markers along the timeline (small open circles, 8px, Blue Slate #5F7483). Below each milestone, labels in Inter Regular, 13pt, Charcoal (#1E2428): "Fund cash balance plan", "Restructure entity elections", "Finalize retirement contributions". Headline above the timeline: "6 Months of Planning Capacity" in Playfair Display SemiBold, 28pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper third. Below the timeline, a supporting line: "The extension is a strategy, not a delay." in Inter Regular, 15pt, Blue Slate (#5F7483), centered, positioned 48px below the timeline. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows, no chart junk. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling. Mood: strategic, organized, empowering. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "6 Months of Planning Capacity" in Playfair Display SemiBold, ~28pt, Deep Muted Blue (#243A4B), upper third. Timeline labels and milestones in Inter, various sizes, Charcoal and Blue Slate.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>week-5-linkedin-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>There's a Deduction on Your Tax Return That's Either Worth $29,800 or $0. Which One Is Yours?</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Zooms into one specific diagnostic marker from the anchor's four-line framework: the QBI deduction. Expands on the anchor's finding that QBI presence or absence reveals whether S-Corp salary calibration is correct, giving surgeons a concrete line item to find on their own returns.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>There's a deduction on your tax return that's either worth $29,800 or $0. Which one is yours?
+The QBI deduction allows a 20% deduction on qualified business income. For a surgeon with $149,000 in S-Corp flow-through income, that translates to roughly $29,800 in deductions. At a 37% marginal rate, the tax savings approach $11,000 in a single year.
+But here's where it gets interesting. The QBI deduction is one of the most misunderstood lines on a surgeon's return because its presence or absence is almost entirely determined by how your S-Corp salary is set.
+Pay yourself too much in W-2 salary relative to the practice's net income, and the qualified business income shrinks or disappears entirely. The deduction drops to zero. Pay yourself a reasonable but carefully calibrated salary, and the QBI deduction appears, sometimes worth $25,000 to $35,000.
+The line between those two outcomes is not luck. It is structure. Specifically, it is the ratio between your W-2 salary and your total S-Corp distributions, and whether anyone has looked at that ratio since you set up the entity.
+Surgeons with nearly identical gross incomes can file returns with a $30,000 difference in QBI deductions. Same specialty, same region, same revenue range. The only variable is how the S-Corp salary has been calibrated.
+If your return shows a QBI deduction, check whether the amount reflects your full available capacity. If it shows zero, ask why. The answer usually points to a salary calibration conversation that should have happened a year ago.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Conceptual photograph (photorealistic, environment)
+Rationale: The QBI deduction is a hidden lever buried in the tax return. A photorealistic image of a calm, modern professional environment with a tax document visible on the surface creates a contemplative mood that pairs with the "look closer" message of the post without revealing the answer on the image itself.
+AI image prompt: Create a 1080x1080px square photorealistic image. A clean, modern executive desk surface shot from above at a slight angle. On the desk: a neatly printed multi-page tax return (1040 form partially visible), a fine-point pen resting on the pages, and a small potted succulent in the upper-left corner. The desk is walnut or dark wood grain. Soft natural light from a window on the right side casts gentle shadows across the surface. The background beyond the desk is softly out of focus: a neutral gray wall with a hint of a framed credential. No people visible, just the desk and documents suggesting someone has been studying the return. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field with sharp focus on the pen and the center of the document. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: precise, contemplative, quietly provocative. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>week-5-linkedin-4.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Week 5 (March 23–29)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Four Weeks of Structural Diagnosis. One Document That Confirms Everything.</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Your tax return is a diagnostic report</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Month-closing synthesis that bookends the transition from March's structural diagnosis arc to April's post-filing interpretation. Connects every prior week's insight (entity design, S-Corp salary, reimbursement pressure, effective hourly rate) to the tax return as the single validating document, reinforcing the cumulative argument built across the entire March content arc.</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Four weeks of structural diagnosis. One document that confirms everything.
+Over the past month, we've walked through the major structural levers in a surgical practice. Week by week, piece by piece.
+In Week 1, we looked at entity structure: whether your practice is organized as a sole proprietorship, an S-Corp, or something else entirely, and what that choice costs you in taxes every year. For surgeons earning above $500,000, the wrong entity election can mean $30,000 or more in unnecessary self-employment tax.
+In Week 2, we examined S-Corp salary calibration: the ratio between your W-2 and your distributions, and how that ratio determines whether you qualify for the QBI deduction, how much you pay in payroll taxes, and how much capacity you have for tax-deferred retirement contributions.
+In Week 3, the conversation shifted to external pressure. The CMS 2.5% efficiency adjustment reduced reimbursement for non-time-based orthopedic codes, making every dollar your practice earns more valuable and every structural inefficiency more costly.
+In Week 4, we reframed the entire picture through the effective hourly rate: the number that shows what you actually earn per hour of clinical work after taxes, overhead, and structural drag.
+Now here is the connection. Every one of those insights shows up on your tax return. Your entity election, your salary split, your retirement contributions, your effective rate. The return is the document that validates or contradicts everything.
+If the last four weeks prompted even one question about your financial structure, your tax return is where the answer lives.
+Have you looked at yours with fresh eyes?</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Data visualization
+Rationale: The post synthesizes four weeks of content into one closing argument. A convergence diagram showing four diagnostic threads flowing into a single document creates a visual summary that makes the cumulative narrative feel inevitable, rewarding readers who followed the arc while standing alone for new viewers.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "4 Weeks. 1 Document." in Playfair Display SemiBold, 28pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, four horizontal rounded-rectangle boxes (approximately 300px wide x 48px tall each) stacked vertically with 20px spacing, centered horizontally. Each box has a 2px border in Blue Slate (#5F7483) with Off-White fill. Labels inside each box in Inter Medium, 15pt, Deep Muted Blue (#243A4B), centered: Box 1: "Entity Structure", Box 2: "S-Corp Salary", Box 3: "Reimbursement Pressure", Box 4: "Effective Hourly Rate". From the right edge of each box, a thin connecting line (2px, Antique Gold #B08D57) curves downward and converges to a single point below all four boxes. At the convergence point, a larger rounded rectangle (320px wide x 56px tall) with a solid Deep Muted Blue (#243A4B) fill. Label inside: "Your Tax Return" in Inter SemiBold, 16pt, Off-White (#F6F7F5), centered. Below the bottom box, 24px of spacing, then: "Every answer is on one document." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: composed, authoritative, clarifying. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "4 Weeks. 1 Document." in Playfair Display SemiBold, ~28pt, Deep Muted Blue. Four labeled boxes and convergence to "Your Tax Return" box.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>week-5-linkedin-5.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 6 (MARCH 30 – APRIL 5)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>You've Been Funding a Backdoor Roth Every Year Because Someone Told You To. Here's Why the Math Might Have Changed.</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Opens the week's LinkedIn sequence by challenging the reflexive backdoor Roth habit. OBBBA made the 37% top rate permanent, which fundamentally changes the Roth calculus for high-income surgeons who expect lower rates in retirement. Distills the anchor blog's central argument into a provocative, shareable one-liner that positions Capable Wealth as the advisor who questions conventional wisdom with math.</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>You've been funding a backdoor Roth every year because someone told you to. Here's why the math might have changed.
+The backdoor Roth IRA became a reflex for high-income physicians sometime around 2015. Fund the non-deductible IRA, convert immediately, pay the tax, and enjoy tax-free growth forever. Simple, clean, and almost universally recommended.
+But the tax landscape shifted when OBBBA made the 37% top rate permanent. That changes the equation in a way most surgeons haven't reconsidered.
+Here's the core question: are you paying 37% on your Roth contribution today, and do you expect to withdraw at a rate lower than 37% in retirement?
+If the answer is yes to both, the backdoor Roth may be the most expensive way to save $7,500.
+Consider the math. A surgeon earning $1.2M contributes $7,500 to a backdoor Roth at a 37% federal rate (plus state taxes in most cases). That contribution costs roughly $2,775 in tax today, paid on dollars that could have been directed to a pre-tax vehicle like a cash balance plan, where the same $7,500 would generate an immediate deduction.
+The Roth makes sense when you expect your future tax rate to be the same or higher. For a 55-year-old surgeon planning to retire at 65 with a significantly lower income, that assumption deserves scrutiny.
+This is not an argument against Roth accounts. They have real value in the right circumstances. But "I've always done it" is a habit, not a strategy. And at surgeon-level income, a habit that costs an extra $2,775 per year in unnecessary tax is worth reexamining.
+Before April 15, it's worth asking: does the Roth still earn its place in your plan, or are you funding it out of momentum?</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Stat highlight card
+Rationale: The 37% rate is the post's anchor data point and creates immediate recognition for any surgeon who sees it on their pay stub. A bold stat card makes the tax rate impossible to scroll past and frames the Roth question as a math problem, not a default decision.
+AI image prompt: Create a 1080x1080px square social media graphic. Background: solid Deep Muted Blue (#243A4B). Layout: centered text composition with generous margins (minimum 120px all sides). Primary text: "37%" in Playfair Display SemiBold, approximately 96pt, Antique Gold (#B08D57), centered horizontally, positioned slightly above the vertical center of the canvas. Secondary text: "tax on every Roth dollar" in Inter Regular, approximately 20pt, Off-White (#F6F7F5), centered horizontally, positioned 20px below the primary text. Tertiary text: "Is that still the right move?" in Inter Regular, approximately 16pt, Warm Gray (#9AA3A8), centered horizontally, positioned 12px below the secondary text. A thin horizontal rule (1px, Warm Gray #9AA3A8) spans 25% of the canvas width, centered horizontally, positioned 48px below the tertiary text. Bottom-right corner: Capable Wealth logo mark in Off-White (#F6F7F5), 32px from edges, approximately 80px wide. No imagery, no illustrations, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8), 60/30/10 ratio. No cartoons, no clip art, no generic stock, no clickbait styling, no flashy or sensational elements, no busy compositions. Mood: precise, thought-provoking, authoritative. Professional financial advisory aesthetic for orthopedic surgeons ages 45-65.
+Text overlay: "37%" in Playfair Display SemiBold, ~96pt, Antique Gold (#B08D57), center. "tax on every Roth dollar" in Inter Regular, ~20pt, Off-White (#F6F7F5), below primary. "Is that still the right move?" in Inter Regular, ~16pt, Warm Gray (#9AA3A8), below secondary.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>week-6-linkedin-1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Estimated Taxes Aren't a Quarterly Bill. They're a Quarterly Strategy Session.</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Extends the April 15 theme from the Roth question to the broader estimated tax strategy. Reframes Q1 estimated tax payments from an obligation into an opportunity, introducing a "quarterly financial vital signs" framework that positions each payment as a recalibration point for withholding, income timing, and retirement contribution pacing.</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Estimated taxes aren't a quarterly bill. They're a quarterly strategy session.
+Most surgeons treat their Q1 estimated payment (due April 15) the same way they treated it last year: same amount, same calculation, same assumptions. Write the check, move on.
+But your income probably changed. Your practice revenue may have shifted with the CMS efficiency adjustment. Your retirement contributions may be pacing differently. And OBBBA changed the rate structure in ways that affect how much you should be setting aside.
+Every estimated tax payment is a chance to recalibrate three things at once.
+First, your withholding accuracy. If you're consistently getting large refunds, you're lending the government money interest-free. If you're consistently underpaying, you're setting yourself up for penalties. The target is 100% of last year's liability or 110% of adjusted gross income, whichever applies. At surgeon income levels, the difference between those two thresholds can be meaningful.
+Second, your retirement contribution pacing. Q1 is 25% of the year. Are your 401(k) contributions on pace to max out ($24,500, plus $8,000 catch-up if you're 50 or older)? Is your cash balance plan funded proportionally? Falling behind in Q1 means compressing contributions into later quarters, which can create cash flow pressure.
+Third, your income timing. If you control the timing of distributions from your practice entity, the Q1 payment is a natural checkpoint to evaluate whether your current distribution schedule still makes sense given year-to-date revenue.
+One payment. Three strategic decisions embedded inside it.
+Before you write the April 15 check this year, it's worth spending 30 minutes asking whether the number on that check still reflects your current reality.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Conceptual photograph (photorealistic, people)
+Rationale: The post reframes estimated tax payments as quarterly strategy sessions. A photorealistic image of a surgeon and financial advisor reviewing numbers together conveys the proactive, collaborative relationship the post advocates, moving the image from an abstract number to a tangible moment of financial intentionality.
+AI image prompt: Create a 1080x1080px square photorealistic image. Two professionals seated across from each other at a clean, modern conference table in a well-lit office. One is a male surgeon in his mid-50s wearing a navy blazer over an open-collar white shirt; the other is a female financial advisor in her 40s wearing a charcoal blazer. Between them on the table: a printed financial summary, a laptop angled toward the advisor, and two ceramic coffee cups. The advisor is pointing at a line on the printed document while the surgeon leans in slightly, expression engaged and focused. The setting is a modern office with floor-to-ceiling windows, natural afternoon light creating soft highlights. Background softly out of focus: a cityscape or green campus visible through the windows. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field, sharp focus on the two professionals and the document between them. No text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches (no posed handshakes, no pointing at charts on a whiteboard). Mood: strategic, composed, collaborative. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>week-6-linkedin-2.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>The April 15 Deadline Has Three Decisions Hidden Inside It. Most Surgeons See Only One.</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Unifying post that connects all three April 15 decisions into a single framework. Most surgeons see April 15 as a filing deadline. This post reveals that it is simultaneously the Q1 estimated payment deadline, the prior-year IRA contribution deadline, and the implicit start of the extension planning window. Positions Capable Wealth as the advisor who sees the full picture.</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 deadline has three decisions hidden inside it. Most surgeons see only one.
+Everyone knows April 15 is the tax filing deadline. But for a surgeon with a practice entity, retirement plans, and estimated tax obligations, that single date carries two additional decisions that are just as consequential.
+Here's what's actually on the table:
+Decision 1: File or extend. If your return is straightforward and your numbers are final, filing by April 15 makes sense. If your practice financials are still being reconciled, or if there are planning opportunities that need more time (cost segregation studies, entity restructuring, retirement plan amendments), an extension to October 15 buys you six months of runway. An extension is not a red flag. It is a planning tool.
+Decision 2: Make your Q1 estimated tax payment. This is due April 15 regardless of whether you file or extend. The amount you choose should reflect your 2026 income trajectory, not just last year's numbers. Underpaying triggers penalties. Overpaying ties up cash that could be working elsewhere.
+Decision 3: Make your prior-year IRA contribution. You have until April 15, 2026 to fund a 2025 IRA contribution (up to $7,000, or $8,000 if you were 50 or older in 2025). If you haven't contributed yet and you're planning a backdoor Roth conversion, this is your last window.
+Three decisions, one date, and they interact with each other. Your filing status affects your estimated tax calculation. Your IRA contribution affects your Roth conversion timing. Your extension decision affects how much planning flexibility you have for the rest of the year.
+Which of these three have you addressed?</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Simple infographic
+Rationale: The post reveals three decisions hidden inside a single deadline. A clean three-panel infographic makes the framework immediately scannable and creates a saveable reference visual that surgeons can revisit as April 15 approaches.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "April 15: Three Decisions, One Date" in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, three vertical panels arranged side by side with 24px spacing between them, each approximately 260px wide x 420px tall. Each panel has a 2px top border only (no sides or bottom). Panel 1 top border: Deep Muted Blue (#243A4B). Inside Panel 1: number "1" in Playfair Display SemiBold, 48pt, Deep Muted Blue (#243A4B), centered, at top. Below: "File or Extend" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Process decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Panel 2 top border: Antique Gold (#B08D57). Inside Panel 2: number "2" in Playfair Display SemiBold, 48pt, Antique Gold (#B08D57), centered, at top. Below: "Prior-Year IRA" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Strategy decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Panel 3 top border: Blue Slate (#5F7483). Inside Panel 3: number "3" in Playfair Display SemiBold, 48pt, Blue Slate (#5F7483), centered, at top. Below: "Q1 Estimated Tax" in Inter SemiBold, 16pt, Deep Muted Blue (#243A4B), centered. Below that: "Strategy decision" in Inter Regular, 13pt, Blue Slate (#5F7483), centered. Below all three panels, 32px spacing, then: "Which of these three have you addressed?" in Inter Regular, 15pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: clarifying, organized, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "April 15: Three Decisions, One Date" headline. Three numbered panels with decision labels and types.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>week-6-linkedin-3.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>$7,500 Into a Roth at 42% Tax, or $7,500 Into a Cash Balance Plan at 0% Tax. Same Money. Very Different Math.</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Zooms into the specific math comparison from the anchor blog, isolating the backdoor Roth vs. cash balance plan decision as a direct side-by-side. At surgeon income levels, the opportunity cost of a backdoor Roth contribution compared to redirecting those dollars to a cash balance plan is measurable and significant. This post makes the comparison visceral and concrete.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>$7,500 into a backdoor Roth at a 42% combined tax rate, or $7,500 into a cash balance plan at 0% tax. Same money. Very different math.
+Let's walk through what's actually happening with each dollar.
+The backdoor Roth: You contribute $7,500 of after-tax dollars to a non-deductible IRA and convert to Roth. Because the money was already taxed at your marginal rate (37% federal plus 5% state in most states with income tax), you paid roughly $3,150 in tax to get those dollars into the Roth. The upside: tax-free growth and tax-free withdrawals in retirement.
+The cash balance plan: You contribute $7,500 of pre-tax dollars to a defined benefit plan. That contribution generates an immediate deduction at your marginal rate, saving you the same $3,150 in tax this year. The money grows tax-deferred and is taxed at your retirement rate when you withdraw it.
+Here's where the math gets interesting.
+If you expect your retirement tax rate to be 24% (a reasonable estimate for a surgeon drawing $300,000 to $400,000 annually from retirement accounts), the cash balance plan lets you defer $3,150 in tax today and eventually pay roughly $1,800 on the same $7,500 at withdrawal. Net savings: $1,350 on a single year's contribution.
+Over 10 years of making this choice, the cumulative tax savings from redirecting to a cash balance plan instead of a Roth can exceed $13,000, before accounting for the additional compounding on those deferred tax dollars.
+And cash balance plans allow contributions far beyond $7,500. For surgeons over 50, annual contributions can range from $150,000 to $350,000 or more, depending on plan design.
+The Roth is a good tool. But at your income level, is it the best use of the next $7,500?</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Data visualization
+Rationale: The post's entire argument is a side-by-side math comparison. A branded bar chart showing the tax treatment of the same $7,500 in two vehicles makes the opportunity cost immediately visible and creates a visual that surgeons can share with colleagues to illustrate the point.
+AI image prompt: Create a 1080x1080px square infographic. Background: Off-White (#F6F7F5). Layout: centered composition with generous margins (80px all sides). Headline: "Same $7,500. Very Different Math." in Playfair Display SemiBold, 24pt, Deep Muted Blue (#243A4B), centered horizontally, positioned in the upper fifth. Below the headline, two vertical bar chart columns centered on the canvas with 80px horizontal spacing between them. Left bar: tall (approximately 340px height), filled with Blue Slate (#5F7483). Labeled above the bar: "42%" in Inter SemiBold, 28pt, Deep Muted Blue (#243A4B). Labeled below the bar in two lines: "Backdoor Roth" in Inter SemiBold, 15pt, Deep Muted Blue (#243A4B), then "Tax on contribution" in Inter Regular, 12pt, Blue Slate (#5F7483). Right bar: very short (approximately 20px height, representing near-zero), filled with Antique Gold (#B08D57). Labeled above the bar: "0%" in Inter SemiBold, 28pt, Antique Gold (#B08D57). Labeled below the bar in two lines: "Cash Balance Plan" in Inter SemiBold, 15pt, Deep Muted Blue (#243A4B), then "Immediate deduction" in Inter Regular, 12pt, Blue Slate (#5F7483). A thin Warm Gray (#9AA3A8) baseline (1px) connects the base of both bars. Below the chart, 40px spacing, then: "At surgeon income levels, the opportunity cost compounds." in Inter Regular, 14pt, Blue Slate (#5F7483), centered. Bottom-right: Capable Wealth logo mark in Charcoal (#1E2428), 24px from edges, approximately 60px wide. No photography, no 3D effects, no gradients, no drop shadows, no chart junk. Brand constraints: only Capable Wealth palette (#243A4B, #5F7483, #B08D57, #F6F7F5, #1E2428, #9AA3A8). No cartoons, no clip art. Mood: precise, comparative, authoritative. Professional financial infographic for orthopedic surgeons ages 45-65.
+Text overlay: "Same $7,500. Very Different Math." headline, "42%" and "0%" bar labels, vehicle names and descriptions below bars.
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>week-6-linkedin-4.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Week 6 (March 30 – April 5)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Every Quarter, Four Numbers Tell You Whether Your Financial Plan Is on Track. Most Surgeons Check Zero of Them.</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>The April 15 trifecta: filing, estimated taxes, and the Roth question</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>LinkedIn Post</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Closes the week's LinkedIn sequence by extending the estimated tax discussion into a broader quarterly discipline. Introduces a "quarterly vital signs" framework that gives surgeons four specific numbers to check each quarter, transforming a reactive tax compliance exercise into a proactive wealth-building habit. Positions Capable Wealth as the advisor who builds systems, not just solves problems.</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Every quarter, four numbers tell you whether your financial plan is on track. Most surgeons check zero of them.
+You check vital signs on every patient. You assess labs, imaging, and functional progress at regular intervals because waiting until something goes wrong is not a strategy. Your financial plan deserves the same discipline.
+Here are the four numbers worth reviewing every quarter:
+1. Year-to-date income vs. annual projection. Is your practice revenue tracking where you expected? If you're running 10% ahead, your tax obligations are higher than planned. If you're 10% behind (perhaps from the CMS efficiency adjustment), your retirement contributions and distributions may need adjusting.
+2. Retirement contribution pacing. At the end of Q1, you should be roughly 25% of the way to your annual maximum. For 2026, that means about $6,125 of your $24,500 401(k) limit (or $8,125 including catch-up contributions). If your cash balance plan calls for $200,000 this year, about $50,000 should be funded or committed.
+3. Estimated tax adequacy. Compare your Q1 payment to your projected annual liability. If your income is tracking higher than last year and your estimated payments haven't changed, you're building a shortfall that compounds each quarter. Better to catch it in April than discover it in January.
+4. Cash reserve level. How many months of personal and practice expenses can you cover without touching investments? The target for most surgeon households is three to six months of personal expenses and two to three months of practice overhead. If a large tax payment or equipment purchase just drew down your reserves, this is the quarter to rebuild.
+Four numbers. Fifteen minutes per quarter. The surgeons who check these consistently are the ones who never get surprised.
+Which of these four have you looked at this quarter?</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Primary Image
+Image type: Conceptual photograph (photorealistic, environment)
+Rationale: The post introduces a quarterly discipline framework using a clinical vital-signs analogy. A photorealistic image of a modern medical office environment evokes the clinical rigor the post advocates, connecting the surgeon's professional world to their financial discipline without being literal or heavy-handed.
+AI image prompt: Create a 1080x1080px square photorealistic image. A modern, well-lit medical office corridor viewed from a slight angle, early morning natural light filtering through large windows on the right side. The corridor is clean, minimal, and empty, with polished light-gray floors and white walls. A glass-walled conference room is partially visible on the left, with a clean table and two chairs inside, suggesting a structured meeting space. A single potted green plant sits at the far end of the corridor, providing a subtle touch of warmth. The overall feeling is one of order, discipline, and calm professionalism. Color grading: desaturated and cool-toned, shadows shifted toward Deep Muted Blue (#243A4B), midtones toward Blue Slate (#5F7483), highlights neutral Off-White (#F6F7F5). Shallow depth of field with the far end of the corridor softly out of focus. No people, no text overlays, no logos, no graphic elements. No cartoon, no illustration, no clip art, no generic stock cliches. Mood: organized, professional, forward-looking. Photorealistic editorial photography for a financial advisory brand serving orthopedic surgeons ages 45-65.
+Text overlay: None (photorealistic image, no text)
+Platform and dimensions: LinkedIn, 1080x1080</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>week-6-linkedin-5.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="85" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Strategic Context</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Visual Asset Brief</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Source File</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>WEEK 3 (MARCH 9–15)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="120" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Week 3 (March 9–15)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
           <t>Death by a Thousand Cuts</t>
         </is>
       </c>

</xml_diff>